<commit_message>
feat(ontology): V4.9 — vt_email→vt_id 흡수 + mentions 3종 통합 (노드 25→24, 엣지 61→57)
- vt_email 노드를 vt_id {platform:'email', id_val=소문자 주소}로 흡수
  - uses_email·eg_used_email 삭제 → uses_id·eg_used_id
  - 법적분류(통신자료)는 legal_category_by_platform, 표준테이블(TB_EML_ADDR_M)은 STANDARD_TABLE_MAP by_platform 으로 보존
- mentions_id·mentions_account·mentions_location → mentions (Message→DigitalID|BankAccount|Location)
  - mentions_account 추론 표시 제거 (confidence·extract_method)
- 적재기 rdb_to_graph: 이메일 → vt_id, uses_email → uses_id(platform=email)
- build_integrated_graph: 원본 EP 그래프의 vt_email/uses_email 을 V4.9 표기로 번역
- T2C 정적 스키마·방향표·ai_service 라벨 힌트 갱신 (t2c_v47 학습 프롬프트는 불변)
- 조회 호환: graph_service 방향표·UI 스타일은 이전 적재분 vt_email 조회용으로 유지
- handoff: 정의 스펙 재생성, README·설계이력·엑셀(카탈로그 57/24종, 변경이력 R25·R26), zip

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
+++ b/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="변경이력(V4.3→V4.9)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="엣지카탈로그(61종)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="노드카탈로그(25종)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="엣지카탈로그(57종)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="노드카탈로그(24종)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="노드 속성 사전" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="엣지 속성 사전" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="값 도메인 사전" sheetId="6" state="visible" r:id="rId6"/>
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="53" min="1" max="1"/>
@@ -2613,6 +2613,80 @@
       <c r="G53" s="53" t="inlineStr">
         <is>
           <t>전 그래프 적재 0건. filed_as 는 적재 299건이라 존치 쪽으로 통합</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="53" t="inlineStr">
+        <is>
+          <t>R25</t>
+        </is>
+      </c>
+      <c r="B54" s="53" t="inlineStr">
+        <is>
+          <t>V4.9</t>
+        </is>
+      </c>
+      <c r="C54" s="53" t="inlineStr">
+        <is>
+          <t>흡수</t>
+        </is>
+      </c>
+      <c r="D54" s="53" t="inlineStr">
+        <is>
+          <t>vt_email → vt_id</t>
+        </is>
+      </c>
+      <c r="E54" s="53" t="inlineStr">
+        <is>
+          <t>별도 노드 vt_email(email_addr) + uses_email·eg_used_email</t>
+        </is>
+      </c>
+      <c r="F54" s="53" t="inlineStr">
+        <is>
+          <t>vt_id {platform:'email', id_val=소문자 주소} + uses_id·eg_used_id (노드 25→24, 엣지 −2). 법적분류 통신자료·표준테이블 TB_EML_ADDR_M 은 platform 별 보존</t>
+        </is>
+      </c>
+      <c r="G54" s="53" t="inlineStr">
+        <is>
+          <t>계정과 이메일은 같은 "온라인 식별자" — 조회·연결 규칙이 같아 라벨 분리 이득 없음. 기존 적재 vt_email 5건·uses_email 5건은 재빌드/이관 대상</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="53" t="inlineStr">
+        <is>
+          <t>R26</t>
+        </is>
+      </c>
+      <c r="B55" s="53" t="inlineStr">
+        <is>
+          <t>V4.9</t>
+        </is>
+      </c>
+      <c r="C55" s="53" t="inlineStr">
+        <is>
+          <t>통합</t>
+        </is>
+      </c>
+      <c r="D55" s="53" t="inlineStr">
+        <is>
+          <t>mentions_id · mentions_account · mentions_location</t>
+        </is>
+      </c>
+      <c r="E55" s="53" t="inlineStr">
+        <is>
+          <t>메시지 기재 엣지 3종(mentions_account 는 추론 표시)</t>
+        </is>
+      </c>
+      <c r="F55" s="53" t="inlineStr">
+        <is>
+          <t>mentions 1종 (Message→DigitalID|BankAccount|Location, 도착 라벨로 구분, 엣지 −2). 추론 표시 제거 → confidence·extract_method</t>
+        </is>
+      </c>
+      <c r="G55" s="53" t="inlineStr">
+        <is>
+          <t>전 그래프 적재 0건. 명명 동결(학습데이터) 원칙의 예외 — T2C 다음 재학습 시 mentions 표기 반영</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="53" min="1" max="1"/>
@@ -3352,7 +3426,7 @@
       </c>
       <c r="B21" s="85" t="inlineStr">
         <is>
-          <t>uses_email</t>
+          <t>owns_wallet</t>
         </is>
       </c>
       <c r="C21" s="85" t="inlineStr">
@@ -3362,17 +3436,17 @@
       </c>
       <c r="D21" s="85" t="inlineStr">
         <is>
-          <t>vt_email</t>
+          <t>vt_crypto</t>
         </is>
       </c>
       <c r="E21" s="85" t="inlineStr">
         <is>
-          <t>valid_from, valid_to</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F21" s="86" t="inlineStr">
         <is>
-          <t>이메일 사용</t>
+          <t>가상자산 지갑 소유</t>
         </is>
       </c>
       <c r="G21" s="85" t="n"/>
@@ -3385,7 +3459,7 @@
       </c>
       <c r="B22" s="85" t="inlineStr">
         <is>
-          <t>owns_wallet</t>
+          <t>uses_device</t>
         </is>
       </c>
       <c r="C22" s="85" t="inlineStr">
@@ -3395,94 +3469,94 @@
       </c>
       <c r="D22" s="85" t="inlineStr">
         <is>
-          <t>vt_crypto</t>
+          <t>vt_dev</t>
         </is>
       </c>
       <c r="E22" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>valid_from, valid_to</t>
         </is>
       </c>
       <c r="F22" s="86" t="inlineStr">
         <is>
-          <t>가상자산 지갑 소유</t>
-        </is>
-      </c>
-      <c r="G22" s="85" t="n"/>
+          <t>기기 소유/사용</t>
+        </is>
+      </c>
+      <c r="G22" s="85" t="inlineStr">
+        <is>
+          <t>V4.9 owns_device 통합</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="54">
-      <c r="A23" s="84" t="inlineStr">
-        <is>
-          <t>D. Person→Digital</t>
+      <c r="A23" s="88" t="inlineStr">
+        <is>
+          <t>E. Object 관계</t>
         </is>
       </c>
       <c r="B23" s="85" t="inlineStr">
         <is>
-          <t>uses_device</t>
+          <t>registered_to</t>
         </is>
       </c>
       <c r="C23" s="85" t="inlineStr">
         <is>
+          <t>vt_telno|vt_id</t>
+        </is>
+      </c>
+      <c r="D23" s="85" t="inlineStr">
+        <is>
           <t>vt_psn</t>
         </is>
       </c>
-      <c r="D23" s="85" t="inlineStr">
-        <is>
-          <t>vt_dev</t>
-        </is>
-      </c>
       <c r="E23" s="85" t="inlineStr">
         <is>
-          <t>valid_from, valid_to</t>
+          <t>source_id, rec_created, valid_from, valid_to, duration_days</t>
         </is>
       </c>
       <c r="F23" s="86" t="inlineStr">
         <is>
-          <t>기기 소유/사용</t>
+          <t>전화/플랫폼 계정의 등록(실명확인) 명의자</t>
         </is>
       </c>
       <c r="G23" s="85" t="inlineStr">
         <is>
-          <t>V4.9 owns_device 통합</t>
+          <t>Object→Person 예외 허용 V4.4 유효구간 추가 (G5) [V4.8 domain+DigitalID]</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="54">
-      <c r="A24" s="88" t="inlineStr">
+      <c r="A24" s="84" t="inlineStr">
         <is>
           <t>E. Object 관계</t>
         </is>
       </c>
       <c r="B24" s="85" t="inlineStr">
         <is>
-          <t>registered_to</t>
+          <t>operates</t>
         </is>
       </c>
       <c r="C24" s="85" t="inlineStr">
         <is>
-          <t>vt_telno|vt_id</t>
+          <t>vt_psn/vt_org</t>
         </is>
       </c>
       <c r="D24" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_site/vt_id</t>
         </is>
       </c>
       <c r="E24" s="85" t="inlineStr">
         <is>
-          <t>source_id, rec_created, valid_from, valid_to, duration_days</t>
+          <t>valid_from, valid_to, role</t>
         </is>
       </c>
       <c r="F24" s="86" t="inlineStr">
         <is>
-          <t>전화/플랫폼 계정의 등록(실명확인) 명의자</t>
-        </is>
-      </c>
-      <c r="G24" s="85" t="inlineStr">
-        <is>
-          <t>Object→Person 예외 허용 V4.4 유효구간 추가 (G5) [V4.8 domain+DigitalID]</t>
-        </is>
-      </c>
+          <t>사이트·채널 운영자</t>
+        </is>
+      </c>
+      <c r="G24" s="85" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1" s="54">
       <c r="A25" s="84" t="inlineStr">
@@ -3492,27 +3566,27 @@
       </c>
       <c r="B25" s="85" t="inlineStr">
         <is>
-          <t>operates</t>
+          <t>hosts</t>
         </is>
       </c>
       <c r="C25" s="85" t="inlineStr">
         <is>
-          <t>vt_psn/vt_org</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="D25" s="85" t="inlineStr">
         <is>
-          <t>vt_site/vt_id</t>
+          <t>vt_site</t>
         </is>
       </c>
       <c r="E25" s="85" t="inlineStr">
         <is>
-          <t>valid_from, valid_to, role</t>
+          <t>port, detected_at</t>
         </is>
       </c>
       <c r="F25" s="86" t="inlineStr">
         <is>
-          <t>사이트·채널 운영자</t>
+          <t>서버 IP가 사이트 호스팅</t>
         </is>
       </c>
       <c r="G25" s="85" t="n"/>
@@ -3525,27 +3599,27 @@
       </c>
       <c r="B26" s="85" t="inlineStr">
         <is>
-          <t>hosts</t>
+          <t>belongs_to</t>
         </is>
       </c>
       <c r="C26" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D26" s="85" t="inlineStr">
         <is>
-          <t>vt_site</t>
+          <t>vt_org</t>
         </is>
       </c>
       <c r="E26" s="85" t="inlineStr">
         <is>
-          <t>port, detected_at</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F26" s="86" t="inlineStr">
         <is>
-          <t>서버 IP가 사이트 호스팅</t>
+          <t>계좌 소속 금융기관</t>
         </is>
       </c>
       <c r="G26" s="85" t="n"/>
@@ -3558,27 +3632,27 @@
       </c>
       <c r="B27" s="85" t="inlineStr">
         <is>
-          <t>belongs_to</t>
+          <t>resolves_to</t>
         </is>
       </c>
       <c r="C27" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_site</t>
         </is>
       </c>
       <c r="D27" s="85" t="inlineStr">
         <is>
-          <t>vt_org</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="E27" s="85" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="86" t="inlineStr">
-        <is>
-          <t>계좌 소속 금융기관</t>
+          <t>resolved_dt</t>
+        </is>
+      </c>
+      <c r="F27" s="85" t="inlineStr">
+        <is>
+          <t>DNS 해석 결과</t>
         </is>
       </c>
       <c r="G27" s="85" t="n"/>
@@ -3591,27 +3665,27 @@
       </c>
       <c r="B28" s="85" t="inlineStr">
         <is>
-          <t>resolves_to</t>
+          <t>contains_file</t>
         </is>
       </c>
       <c r="C28" s="85" t="inlineStr">
         <is>
-          <t>vt_site</t>
+          <t>vt_site/vt_msg/vt_id</t>
         </is>
       </c>
       <c r="D28" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_file</t>
         </is>
       </c>
       <c r="E28" s="85" t="inlineStr">
         <is>
-          <t>resolved_dt</t>
-        </is>
-      </c>
-      <c r="F28" s="85" t="inlineStr">
-        <is>
-          <t>DNS 해석 결과</t>
+          <t>file_role, detected_at</t>
+        </is>
+      </c>
+      <c r="F28" s="86" t="inlineStr">
+        <is>
+          <t>파일 내장·배포</t>
         </is>
       </c>
       <c r="G28" s="85" t="n"/>
@@ -3624,27 +3698,27 @@
       </c>
       <c r="B29" s="85" t="inlineStr">
         <is>
-          <t>contains_file</t>
+          <t>communicated_with</t>
         </is>
       </c>
       <c r="C29" s="85" t="inlineStr">
         <is>
-          <t>vt_site/vt_msg/vt_id</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="D29" s="85" t="inlineStr">
         <is>
-          <t>vt_file</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="E29" s="85" t="inlineStr">
         <is>
-          <t>file_role, detected_at</t>
-        </is>
-      </c>
-      <c r="F29" s="86" t="inlineStr">
-        <is>
-          <t>파일 내장·배포</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F29" s="85" t="inlineStr">
+        <is>
+          <t>IP 간 직접 통신</t>
         </is>
       </c>
       <c r="G29" s="85" t="n"/>
@@ -3657,32 +3731,32 @@
       </c>
       <c r="B30" s="85" t="inlineStr">
         <is>
-          <t>mentions_account</t>
+          <t>transferred_to</t>
         </is>
       </c>
       <c r="C30" s="85" t="inlineStr">
         <is>
-          <t>vt_msg</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D30" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_bacnt / vt_crypto</t>
         </is>
       </c>
       <c r="E30" s="85" t="inlineStr">
         <is>
-          <t>confidence(0.85), inference_basis_type, evidence_edge_ids, evidence_count</t>
+          <t>first_dlng_dt, last_dlng_dt, txn_count, total_amount, channel</t>
         </is>
       </c>
       <c r="F30" s="86" t="inlineStr">
         <is>
-          <t>메시지 내 계좌 언급(추론)</t>
+          <t>계좌(지갑) 간 이체 — 건별 거래를 (보낸 쪽, 받는 쪽) 쌍당 1엣지로 집계한 원천 사실</t>
         </is>
       </c>
       <c r="G30" s="85" t="inlineStr">
         <is>
-          <t>V4.4 근거 구조화 (G7)</t>
+          <t>V4.9 직접 엣지로 재정의(추론·직접생성 금지 해제) · 다단계 흐름은 경로 조회 · (쌍) 집계</t>
         </is>
       </c>
     </row>
@@ -3694,141 +3768,137 @@
       </c>
       <c r="B31" s="85" t="inlineStr">
         <is>
-          <t>communicated_with</t>
+          <t>linked_to</t>
         </is>
       </c>
       <c r="C31" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>(object)</t>
         </is>
       </c>
       <c r="D31" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>(object)</t>
         </is>
       </c>
       <c r="E31" s="85" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F31" s="85" t="inlineStr">
-        <is>
-          <t>IP 간 직접 통신</t>
-        </is>
-      </c>
-      <c r="G31" s="85" t="n"/>
+          <t>link_type, confidence</t>
+        </is>
+      </c>
+      <c r="F31" s="86" t="inlineStr">
+        <is>
+          <t>범용 연결(임시/추론)</t>
+        </is>
+      </c>
+      <c r="G31" s="86" t="inlineStr">
+        <is>
+          <t>V4.9 중복 행(Petition→Case, deprecated) 정리 — 진정서→사건은 filed_as</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1" s="54">
-      <c r="A32" s="88" t="inlineStr">
+      <c r="A32" s="84" t="inlineStr">
         <is>
           <t>E. Object 관계</t>
         </is>
       </c>
       <c r="B32" s="85" t="inlineStr">
         <is>
-          <t>transferred_to</t>
+          <t>belongs_to_campaign</t>
         </is>
       </c>
       <c r="C32" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_site</t>
         </is>
       </c>
       <c r="D32" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt / vt_crypto</t>
+          <t>site_cluster</t>
         </is>
       </c>
       <c r="E32" s="85" t="inlineStr">
         <is>
-          <t>first_dlng_dt, last_dlng_dt, txn_count, total_amount, channel</t>
+          <t>sim_score, detected_at</t>
         </is>
       </c>
       <c r="F32" s="86" t="inlineStr">
         <is>
-          <t>계좌(지갑) 간 이체 — 건별 거래를 (보낸 쪽, 받는 쪽) 쌍당 1엣지로 집계한 원천 사실</t>
+          <t>피싱 캠페인 소속</t>
         </is>
       </c>
       <c r="G32" s="85" t="inlineStr">
         <is>
-          <t>V4.9 직접 엣지로 재정의(추론·직접생성 금지 해제) · 다단계 흐름은 경로 조회 · (쌍) 집계</t>
+          <t>V4.9 파생 엣지(군집 결과, SiteClusterDetection 생성) — 원천 사실 아님</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" s="54">
       <c r="A33" s="84" t="inlineStr">
         <is>
-          <t>E. Object 관계</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B33" s="85" t="inlineStr">
         <is>
-          <t>linked_to</t>
+          <t>from_account</t>
         </is>
       </c>
       <c r="C33" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D33" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>vt_transfer</t>
         </is>
       </c>
       <c r="E33" s="85" t="inlineStr">
         <is>
-          <t>link_type, confidence</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F33" s="86" t="inlineStr">
         <is>
-          <t>범용 연결(임시/추론)</t>
-        </is>
-      </c>
-      <c r="G33" s="86" t="inlineStr">
-        <is>
-          <t>V4.9 중복 행(Petition→Case, deprecated) 정리 — 진정서→사건은 filed_as</t>
-        </is>
-      </c>
+          <t>이체 출금 계좌</t>
+        </is>
+      </c>
+      <c r="G33" s="85" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1" s="54">
       <c r="A34" s="84" t="inlineStr">
         <is>
-          <t>E. Object 관계</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B34" s="85" t="inlineStr">
         <is>
-          <t>belongs_to_campaign</t>
+          <t>to_account</t>
         </is>
       </c>
       <c r="C34" s="85" t="inlineStr">
         <is>
-          <t>vt_site</t>
+          <t>vt_transfer</t>
         </is>
       </c>
       <c r="D34" s="85" t="inlineStr">
         <is>
-          <t>site_cluster</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="E34" s="85" t="inlineStr">
         <is>
-          <t>sim_score, detected_at</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F34" s="86" t="inlineStr">
         <is>
-          <t>피싱 캠페인 소속</t>
-        </is>
-      </c>
-      <c r="G34" s="85" t="inlineStr">
-        <is>
-          <t>V4.9 파생 엣지(군집 결과, SiteClusterDetection 생성) — 원천 사실 아님</t>
-        </is>
-      </c>
+          <t>이체 입금 계좌</t>
+        </is>
+      </c>
+      <c r="G34" s="85" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1" s="54">
       <c r="A35" s="84" t="inlineStr">
@@ -3838,17 +3908,17 @@
       </c>
       <c r="B35" s="85" t="inlineStr">
         <is>
-          <t>from_account</t>
+          <t>caller</t>
         </is>
       </c>
       <c r="C35" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="D35" s="85" t="inlineStr">
         <is>
-          <t>vt_transfer</t>
+          <t>vt_call</t>
         </is>
       </c>
       <c r="E35" s="85" t="inlineStr">
@@ -3858,7 +3928,7 @@
       </c>
       <c r="F35" s="86" t="inlineStr">
         <is>
-          <t>이체 출금 계좌</t>
+          <t>발신 번호</t>
         </is>
       </c>
       <c r="G35" s="85" t="n"/>
@@ -3871,17 +3941,17 @@
       </c>
       <c r="B36" s="85" t="inlineStr">
         <is>
-          <t>to_account</t>
+          <t>callee</t>
         </is>
       </c>
       <c r="C36" s="85" t="inlineStr">
         <is>
-          <t>vt_transfer</t>
+          <t>vt_call</t>
         </is>
       </c>
       <c r="D36" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="E36" s="85" t="inlineStr">
@@ -3891,7 +3961,7 @@
       </c>
       <c r="F36" s="86" t="inlineStr">
         <is>
-          <t>이체 입금 계좌</t>
+          <t>수신 번호</t>
         </is>
       </c>
       <c r="G36" s="85" t="n"/>
@@ -3904,30 +3974,34 @@
       </c>
       <c r="B37" s="85" t="inlineStr">
         <is>
-          <t>caller</t>
+          <t>contacted</t>
         </is>
       </c>
       <c r="C37" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>vt_telno|vt_id</t>
         </is>
       </c>
       <c r="D37" s="85" t="inlineStr">
         <is>
-          <t>vt_call</t>
+          <t>vt_telno|vt_id</t>
         </is>
       </c>
       <c r="E37" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>channel, first_dt, last_dt, call_count, msg_count, total_dur_sec, source_id</t>
         </is>
       </c>
       <c r="F37" s="86" t="inlineStr">
         <is>
-          <t>발신 번호</t>
-        </is>
-      </c>
-      <c r="G37" s="85" t="n"/>
+          <t>전화/메신저 계정 간 통화·연락 관계 (요약 엣지)</t>
+        </is>
+      </c>
+      <c r="G37" s="85" t="inlineStr">
+        <is>
+          <t>[V4.8 domain/range+DigitalID, channel 속성] · V4.9 (쌍,channel) 집계 속성 명시</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1" s="54">
       <c r="A38" s="84" t="inlineStr">
@@ -3937,17 +4011,17 @@
       </c>
       <c r="B38" s="85" t="inlineStr">
         <is>
-          <t>callee</t>
+          <t>sent_msg</t>
         </is>
       </c>
       <c r="C38" s="85" t="inlineStr">
         <is>
-          <t>vt_call</t>
+          <t>vt_telno/vt_id</t>
         </is>
       </c>
       <c r="D38" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="E38" s="85" t="inlineStr">
@@ -3957,7 +4031,7 @@
       </c>
       <c r="F38" s="86" t="inlineStr">
         <is>
-          <t>수신 번호</t>
+          <t>메시지 발신</t>
         </is>
       </c>
       <c r="G38" s="85" t="n"/>
@@ -3970,34 +4044,30 @@
       </c>
       <c r="B39" s="85" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>received_msg</t>
         </is>
       </c>
       <c r="C39" s="85" t="inlineStr">
         <is>
-          <t>vt_telno|vt_id</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="D39" s="85" t="inlineStr">
         <is>
-          <t>vt_telno|vt_id</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="E39" s="85" t="inlineStr">
         <is>
-          <t>channel, first_dt, last_dt, call_count, msg_count, total_dur_sec, source_id</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F39" s="86" t="inlineStr">
         <is>
-          <t>전화/메신저 계정 간 통화·연락 관계 (요약 엣지)</t>
-        </is>
-      </c>
-      <c r="G39" s="85" t="inlineStr">
-        <is>
-          <t>[V4.8 domain/range+DigitalID, channel 속성] · V4.9 (쌍,channel) 집계 속성 명시</t>
-        </is>
-      </c>
+          <t>메시지 수신</t>
+        </is>
+      </c>
+      <c r="G39" s="85" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="54">
       <c r="A40" s="84" t="inlineStr">
@@ -4007,17 +4077,17 @@
       </c>
       <c r="B40" s="85" t="inlineStr">
         <is>
-          <t>sent_msg</t>
+          <t>accessed_from</t>
         </is>
       </c>
       <c r="C40" s="85" t="inlineStr">
         <is>
-          <t>vt_telno/vt_id</t>
+          <t>vt_access</t>
         </is>
       </c>
       <c r="D40" s="85" t="inlineStr">
         <is>
-          <t>vt_msg</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="E40" s="85" t="inlineStr">
@@ -4027,43 +4097,47 @@
       </c>
       <c r="F40" s="86" t="inlineStr">
         <is>
-          <t>메시지 발신</t>
+          <t>접속 출발 IP</t>
         </is>
       </c>
       <c r="G40" s="85" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1" s="54">
-      <c r="A41" s="84" t="inlineStr">
+      <c r="A41" s="90" t="inlineStr">
         <is>
           <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B41" s="85" t="inlineStr">
         <is>
-          <t>received_msg</t>
+          <t>accessed_to</t>
         </is>
       </c>
       <c r="C41" s="85" t="inlineStr">
         <is>
-          <t>vt_msg</t>
+          <t>vt_access</t>
         </is>
       </c>
       <c r="D41" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>vt_site / vt_bacnt / vt_id</t>
         </is>
       </c>
       <c r="E41" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>target_type, source_id</t>
         </is>
       </c>
       <c r="F41" s="86" t="inlineStr">
         <is>
-          <t>메시지 수신</t>
-        </is>
-      </c>
-      <c r="G41" s="85" t="n"/>
+          <t>접속 목적지 (웹사이트 · 인터넷뱅킹 대상 계좌 · 포털 계정)</t>
+        </is>
+      </c>
+      <c r="G41" s="85" t="inlineStr">
+        <is>
+          <t>V4.5 range 확장 (G8)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1" s="54">
       <c r="A42" s="84" t="inlineStr">
@@ -4073,17 +4147,17 @@
       </c>
       <c r="B42" s="85" t="inlineStr">
         <is>
-          <t>accessed_from</t>
+          <t>occurred_at</t>
         </is>
       </c>
       <c r="C42" s="85" t="inlineStr">
         <is>
-          <t>vt_access</t>
+          <t>(event)</t>
         </is>
       </c>
       <c r="D42" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_loc</t>
         </is>
       </c>
       <c r="E42" s="85" t="inlineStr">
@@ -4093,47 +4167,43 @@
       </c>
       <c r="F42" s="86" t="inlineStr">
         <is>
-          <t>접속 출발 IP</t>
+          <t>이벤트 발생 위치</t>
         </is>
       </c>
       <c r="G42" s="85" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="54">
-      <c r="A43" s="90" t="inlineStr">
+      <c r="A43" s="84" t="inlineStr">
         <is>
           <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B43" s="85" t="inlineStr">
         <is>
-          <t>accessed_to</t>
+          <t>recorded_in</t>
         </is>
       </c>
       <c r="C43" s="85" t="inlineStr">
         <is>
-          <t>vt_access</t>
+          <t>vt_vhcl/vt_telno</t>
         </is>
       </c>
       <c r="D43" s="85" t="inlineStr">
         <is>
-          <t>vt_site / vt_bacnt / vt_id</t>
+          <t>vt_movement</t>
         </is>
       </c>
       <c r="E43" s="85" t="inlineStr">
         <is>
-          <t>target_type, source_id</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F43" s="86" t="inlineStr">
         <is>
-          <t>접속 목적지 (웹사이트 · 인터넷뱅킹 대상 계좌 · 포털 계정)</t>
-        </is>
-      </c>
-      <c r="G43" s="85" t="inlineStr">
-        <is>
-          <t>V4.5 range 확장 (G8)</t>
-        </is>
-      </c>
+          <t>이동 기록의 주체</t>
+        </is>
+      </c>
+      <c r="G43" s="85" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1" s="54">
       <c r="A44" s="84" t="inlineStr">
@@ -4143,27 +4213,27 @@
       </c>
       <c r="B44" s="85" t="inlineStr">
         <is>
-          <t>occurred_at</t>
+          <t>used_in_device</t>
         </is>
       </c>
       <c r="C44" s="85" t="inlineStr">
         <is>
-          <t>(event)</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="D44" s="85" t="inlineStr">
         <is>
-          <t>vt_loc</t>
+          <t>vt_dev</t>
         </is>
       </c>
       <c r="E44" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>valid_from, valid_to, source_id</t>
         </is>
       </c>
       <c r="F44" s="86" t="inlineStr">
         <is>
-          <t>이벤트 발생 위치</t>
+          <t>전화-기기(IMEI) 사용</t>
         </is>
       </c>
       <c r="G44" s="85" t="n"/>
@@ -4171,22 +4241,22 @@
     <row r="45" ht="18" customHeight="1" s="54">
       <c r="A45" s="84" t="inlineStr">
         <is>
-          <t>F. Event 흐름</t>
+          <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B45" s="85" t="inlineStr">
         <is>
-          <t>recorded_in</t>
+          <t>used_for</t>
         </is>
       </c>
       <c r="C45" s="85" t="inlineStr">
         <is>
-          <t>vt_vhcl/vt_telno</t>
+          <t>(object)</t>
         </is>
       </c>
       <c r="D45" s="85" t="inlineStr">
         <is>
-          <t>vt_movement</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="E45" s="85" t="inlineStr">
@@ -4196,7 +4266,7 @@
       </c>
       <c r="F45" s="86" t="inlineStr">
         <is>
-          <t>이동 기록의 주체</t>
+          <t>사칭에 사용된 객체</t>
         </is>
       </c>
       <c r="G45" s="85" t="n"/>
@@ -4204,247 +4274,255 @@
     <row r="46" ht="18" customHeight="1" s="54">
       <c r="A46" s="84" t="inlineStr">
         <is>
-          <t>F. Event 흐름</t>
+          <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B46" s="85" t="inlineStr">
         <is>
-          <t>used_in_device</t>
+          <t>targets</t>
         </is>
       </c>
       <c r="C46" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="D46" s="85" t="inlineStr">
         <is>
-          <t>vt_dev</t>
+          <t>vt_org</t>
         </is>
       </c>
       <c r="E46" s="85" t="inlineStr">
         <is>
-          <t>valid_from, valid_to, source_id</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F46" s="86" t="inlineStr">
         <is>
-          <t>전화-기기(IMEI) 사용</t>
+          <t>사칭 대상 기관</t>
         </is>
       </c>
       <c r="G46" s="85" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="54">
-      <c r="A47" s="84" t="inlineStr">
+      <c r="A47" s="88" t="inlineStr">
         <is>
           <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B47" s="85" t="inlineStr">
         <is>
-          <t>used_for</t>
+          <t>performed_by</t>
         </is>
       </c>
       <c r="C47" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>vt_access/vt_movement</t>
         </is>
       </c>
       <c r="D47" s="85" t="inlineStr">
         <is>
-          <t>vt_impersonation</t>
+          <t>vt_psn / vt_telno / vt_id</t>
         </is>
       </c>
       <c r="E47" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>actor_type, resolved_to, resolved_at</t>
         </is>
       </c>
       <c r="F47" s="86" t="inlineStr">
         <is>
-          <t>사칭에 사용된 객체</t>
-        </is>
-      </c>
-      <c r="G47" s="85" t="n"/>
+          <t>접속·이동 수행 주체 (인물 미특정 단계에서는 번호·계정을 주체로 기록)</t>
+        </is>
+      </c>
+      <c r="G47" s="85" t="inlineStr">
+        <is>
+          <t>V4.4 range 확장 (G1)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1" s="54">
       <c r="A48" s="84" t="inlineStr">
         <is>
-          <t>G. 사칭/접속주체</t>
+          <t>H. Provenance</t>
         </is>
       </c>
       <c r="B48" s="85" t="inlineStr">
         <is>
-          <t>targets</t>
+          <t>sourced_from</t>
         </is>
       </c>
       <c r="C48" s="85" t="inlineStr">
         <is>
-          <t>vt_impersonation</t>
+          <t>(any)</t>
         </is>
       </c>
       <c r="D48" s="85" t="inlineStr">
         <is>
-          <t>vt_org</t>
+          <t>vt_src</t>
         </is>
       </c>
       <c r="E48" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>src_tier, rec_created</t>
         </is>
       </c>
       <c r="F48" s="86" t="inlineStr">
         <is>
-          <t>사칭 대상 기관</t>
-        </is>
-      </c>
-      <c r="G48" s="85" t="n"/>
+          <t>데이터 출처 참조</t>
+        </is>
+      </c>
+      <c r="G48" s="85" t="inlineStr">
+        <is>
+          <t>tier1~3만 엣지 생성</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1" s="54">
-      <c r="A49" s="88" t="inlineStr">
-        <is>
-          <t>G. 사칭/접속주체</t>
-        </is>
-      </c>
-      <c r="B49" s="85" t="inlineStr">
-        <is>
-          <t>performed_by</t>
-        </is>
-      </c>
-      <c r="C49" s="85" t="inlineStr">
-        <is>
-          <t>vt_access/vt_movement</t>
-        </is>
-      </c>
-      <c r="D49" s="85" t="inlineStr">
-        <is>
-          <t>vt_psn / vt_telno / vt_id</t>
-        </is>
-      </c>
-      <c r="E49" s="85" t="inlineStr">
-        <is>
-          <t>actor_type, resolved_to, resolved_at</t>
-        </is>
-      </c>
-      <c r="F49" s="86" t="inlineStr">
-        <is>
-          <t>접속·이동 수행 주체 (인물 미특정 단계에서는 번호·계정을 주체로 기록)</t>
-        </is>
-      </c>
-      <c r="G49" s="85" t="inlineStr">
-        <is>
-          <t>V4.4 range 확장 (G1)</t>
+      <c r="A49" s="91" t="inlineStr">
+        <is>
+          <t>C. Person 관계</t>
+        </is>
+      </c>
+      <c r="B49" s="53" t="inlineStr">
+        <is>
+          <t>controls</t>
+        </is>
+      </c>
+      <c r="C49" s="53" t="inlineStr">
+        <is>
+          <t>vt_psn</t>
+        </is>
+      </c>
+      <c r="D49" s="53" t="inlineStr">
+        <is>
+          <t>vt_bacnt</t>
+        </is>
+      </c>
+      <c r="E49" s="53" t="inlineStr">
+        <is>
+          <t>confidence, inference_basis_type, evidence_edge_ids, evidence_count, evidence_summary</t>
+        </is>
+      </c>
+      <c r="F49" s="92" t="inlineStr">
+        <is>
+          <t>실질 지배(명의≠실사용)</t>
+        </is>
+      </c>
+      <c r="G49" s="92" t="inlineStr">
+        <is>
+          <t>정합화 등재 V4.4 근거 구조화 (G7)</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="54">
-      <c r="A50" s="84" t="inlineStr">
-        <is>
-          <t>H. Provenance</t>
-        </is>
-      </c>
-      <c r="B50" s="85" t="inlineStr">
-        <is>
-          <t>sourced_from</t>
-        </is>
-      </c>
-      <c r="C50" s="85" t="inlineStr">
-        <is>
-          <t>(any)</t>
-        </is>
-      </c>
-      <c r="D50" s="85" t="inlineStr">
-        <is>
-          <t>vt_src</t>
-        </is>
-      </c>
-      <c r="E50" s="85" t="inlineStr">
-        <is>
-          <t>src_tier, rec_created</t>
-        </is>
-      </c>
-      <c r="F50" s="86" t="inlineStr">
-        <is>
-          <t>데이터 출처 참조</t>
-        </is>
-      </c>
-      <c r="G50" s="85" t="inlineStr">
-        <is>
-          <t>tier1~3만 엣지 생성</t>
+      <c r="A50" s="93" t="inlineStr">
+        <is>
+          <t>I. 위치</t>
+        </is>
+      </c>
+      <c r="B50" s="53" t="inlineStr">
+        <is>
+          <t>located_at</t>
+        </is>
+      </c>
+      <c r="C50" s="53" t="inlineStr">
+        <is>
+          <t>vt_atm/vt_org</t>
+        </is>
+      </c>
+      <c r="D50" s="53" t="inlineStr">
+        <is>
+          <t>vt_loc</t>
+        </is>
+      </c>
+      <c r="E50" s="53" t="inlineStr">
+        <is>
+          <t>first_dt, last_dt, evt_count, source_id</t>
+        </is>
+      </c>
+      <c r="F50" s="92" t="inlineStr">
+        <is>
+          <t>고정 객체의 정적 위치</t>
+        </is>
+      </c>
+      <c r="G50" s="92" t="inlineStr">
+        <is>
+          <t>정합화 등재 · V4.9 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1" s="54">
-      <c r="A51" s="91" t="inlineStr">
-        <is>
-          <t>C. Person 관계</t>
-        </is>
-      </c>
-      <c r="B51" s="53" t="inlineStr">
-        <is>
-          <t>controls</t>
-        </is>
-      </c>
-      <c r="C51" s="53" t="inlineStr">
+      <c r="A51" s="94" t="inlineStr">
+        <is>
+          <t>J. V4.3 시나리오</t>
+        </is>
+      </c>
+      <c r="B51" s="85" t="inlineStr">
+        <is>
+          <t>knows</t>
+        </is>
+      </c>
+      <c r="C51" s="85" t="inlineStr">
         <is>
           <t>vt_psn</t>
         </is>
       </c>
-      <c r="D51" s="53" t="inlineStr">
-        <is>
-          <t>vt_bacnt</t>
-        </is>
-      </c>
-      <c r="E51" s="53" t="inlineStr">
-        <is>
-          <t>confidence, inference_basis_type, evidence_edge_ids, evidence_count, evidence_summary</t>
-        </is>
-      </c>
-      <c r="F51" s="92" t="inlineStr">
-        <is>
-          <t>실질 지배(명의≠실사용)</t>
-        </is>
-      </c>
-      <c r="G51" s="92" t="inlineStr">
-        <is>
-          <t>정합화 등재 V4.4 근거 구조화 (G7)</t>
+      <c r="D51" s="85" t="inlineStr">
+        <is>
+          <t>vt_psn</t>
+        </is>
+      </c>
+      <c r="E51" s="85" t="inlineStr">
+        <is>
+          <t>relation_type, confidence, valid_from</t>
+        </is>
+      </c>
+      <c r="F51" s="86" t="inlineStr">
+        <is>
+          <t>두 인물의 사회적 지인 관계 (고향친구/동창 — 공범 여부는 그래프 엣지가 아니라 탐지 결과로 판단)</t>
+        </is>
+      </c>
+      <c r="G51" s="85" t="inlineStr">
+        <is>
+          <t>V4.3 신규</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="54">
-      <c r="A52" s="93" t="inlineStr">
-        <is>
-          <t>I. 위치</t>
-        </is>
-      </c>
-      <c r="B52" s="53" t="inlineStr">
-        <is>
-          <t>located_at</t>
-        </is>
-      </c>
-      <c r="C52" s="53" t="inlineStr">
-        <is>
-          <t>vt_atm/vt_org</t>
-        </is>
-      </c>
-      <c r="D52" s="53" t="inlineStr">
-        <is>
-          <t>vt_loc</t>
-        </is>
-      </c>
-      <c r="E52" s="53" t="inlineStr">
-        <is>
-          <t>first_dt, last_dt, evt_count, source_id</t>
-        </is>
-      </c>
-      <c r="F52" s="92" t="inlineStr">
-        <is>
-          <t>고정 객체의 정적 위치</t>
-        </is>
-      </c>
-      <c r="G52" s="92" t="inlineStr">
-        <is>
-          <t>정합화 등재 · V4.9 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count</t>
+      <c r="A52" s="95" t="inlineStr">
+        <is>
+          <t>J. V4.3 시나리오</t>
+        </is>
+      </c>
+      <c r="B52" s="85" t="inlineStr">
+        <is>
+          <t>linked_id</t>
+        </is>
+      </c>
+      <c r="C52" s="85" t="inlineStr">
+        <is>
+          <t>vt_bacnt / vt_telno / vt_ip</t>
+        </is>
+      </c>
+      <c r="D52" s="85" t="inlineStr">
+        <is>
+          <t>vt_id</t>
+        </is>
+      </c>
+      <c r="E52" s="85" t="inlineStr">
+        <is>
+          <t>link_basis, confidence, valid_from, valid_to, warrant_no</t>
+        </is>
+      </c>
+      <c r="F52" s="86" t="inlineStr">
+        <is>
+          <t>객체에 연결된 온라인 식별자 (공인인증서 발급 ID / 포털·통신사·금융 역조회 결과)</t>
+        </is>
+      </c>
+      <c r="G52" s="85" t="inlineStr">
+        <is>
+          <t>V4.3 신규 → V4.4 domain에 vt_ip 추가 (G4)</t>
         </is>
       </c>
     </row>
@@ -4456,180 +4534,180 @@
       </c>
       <c r="B53" s="85" t="inlineStr">
         <is>
-          <t>knows</t>
+          <t>mentions</t>
         </is>
       </c>
       <c r="C53" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="D53" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_id | vt_bacnt | vt_loc</t>
         </is>
       </c>
       <c r="E53" s="85" t="inlineStr">
         <is>
-          <t>relation_type, confidence, valid_from</t>
+          <t>confidence, extract_method, source_id, rec_created</t>
         </is>
       </c>
       <c r="F53" s="86" t="inlineStr">
         <is>
-          <t>두 인물의 사회적 지인 관계 (고향친구/동창 — 공범 여부는 그래프 엣지가 아니라 탐지 결과로 판단)</t>
+          <t>메시지·게시물 본문에 계정·계좌·장소가 기재됨 — 종류는 도착 라벨로 구분</t>
         </is>
       </c>
       <c r="G53" s="85" t="inlineStr">
         <is>
-          <t>V4.3 신규</t>
+          <t>V4.9 통합 (mentions_id·mentions_account·mentions_location)</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" s="54">
-      <c r="A54" s="95" t="inlineStr">
-        <is>
-          <t>J. V4.3 시나리오</t>
-        </is>
-      </c>
-      <c r="B54" s="85" t="inlineStr">
-        <is>
-          <t>linked_id</t>
-        </is>
-      </c>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>vt_bacnt / vt_telno / vt_ip</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
+      <c r="A54" s="98" t="inlineStr">
+        <is>
+          <t>B. Case→Object 증거</t>
+        </is>
+      </c>
+      <c r="B54" s="99" t="inlineStr">
+        <is>
+          <t>eg_used_id</t>
+        </is>
+      </c>
+      <c r="C54" s="99" t="inlineStr">
+        <is>
+          <t>vt_case</t>
+        </is>
+      </c>
+      <c r="D54" s="99" t="inlineStr">
         <is>
           <t>vt_id</t>
         </is>
       </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>link_basis, confidence, valid_from, valid_to, warrant_no</t>
-        </is>
-      </c>
-      <c r="F54" s="86" t="inlineStr">
-        <is>
-          <t>객체에 연결된 온라인 식별자 (공인인증서 발급 ID / 포털·통신사·금융 역조회 결과)</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>V4.3 신규 → V4.4 domain에 vt_ip 추가 (G4)</t>
+      <c r="E54" s="99" t="inlineStr">
+        <is>
+          <t>source_id, rec_created, valid_from, valid_to</t>
+        </is>
+      </c>
+      <c r="F54" s="100" t="inlineStr">
+        <is>
+          <t>사용 온라인 계정 증거 (네이버·카카오·구글 ID)</t>
+        </is>
+      </c>
+      <c r="G54" s="99" t="inlineStr">
+        <is>
+          <t>V4.4 신규 (R3)</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1" s="54">
-      <c r="A55" s="94" t="inlineStr">
-        <is>
-          <t>J. V4.3 시나리오</t>
-        </is>
-      </c>
-      <c r="B55" s="85" t="inlineStr">
-        <is>
-          <t>mentions_id</t>
-        </is>
-      </c>
-      <c r="C55" s="85" t="inlineStr">
+      <c r="A55" s="98" t="inlineStr">
+        <is>
+          <t>F. Event 흐름</t>
+        </is>
+      </c>
+      <c r="B55" s="99" t="inlineStr">
+        <is>
+          <t>sent_from_ip</t>
+        </is>
+      </c>
+      <c r="C55" s="99" t="inlineStr">
         <is>
           <t>vt_msg</t>
         </is>
       </c>
-      <c r="D55" s="85" t="inlineStr">
-        <is>
-          <t>vt_id</t>
-        </is>
-      </c>
-      <c r="E55" s="85" t="inlineStr">
-        <is>
-          <t>confidence, source_id</t>
-        </is>
-      </c>
-      <c r="F55" s="86" t="inlineStr">
-        <is>
-          <t>게시물/메시지에 기재된 온라인 계정 (광고글의 텔레그램 ID Zion7950)</t>
-        </is>
-      </c>
-      <c r="G55" s="85" t="inlineStr">
-        <is>
-          <t>V4.3 신규</t>
+      <c r="D55" s="99" t="inlineStr">
+        <is>
+          <t>vt_ip</t>
+        </is>
+      </c>
+      <c r="E55" s="99" t="inlineStr">
+        <is>
+          <t>detected_at, source_id</t>
+        </is>
+      </c>
+      <c r="F55" s="100" t="inlineStr">
+        <is>
+          <t>메시지 발신 시점의 접속 IP (착발신내역이 메시지+접속을 한 레코드로 제공하는 경우)</t>
+        </is>
+      </c>
+      <c r="G55" s="99" t="inlineStr">
+        <is>
+          <t>V4.4 신규 (G2)</t>
         </is>
       </c>
     </row>
     <row r="56" ht="36" customHeight="1" s="54">
       <c r="A56" s="98" t="inlineStr">
         <is>
-          <t>B. Case→Object 증거</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B56" s="99" t="inlineStr">
         <is>
-          <t>eg_used_id</t>
+          <t>exchanged_to</t>
         </is>
       </c>
       <c r="C56" s="99" t="inlineStr">
         <is>
-          <t>vt_case</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D56" s="99" t="inlineStr">
         <is>
-          <t>vt_id</t>
+          <t>vt_crypto</t>
         </is>
       </c>
       <c r="E56" s="99" t="inlineStr">
         <is>
-          <t>source_id, rec_created, valid_from, valid_to</t>
+          <t>exchange_nm, dlng_dt, fiat_amt, asset_amt, confidence, inference</t>
         </is>
       </c>
       <c r="F56" s="100" t="inlineStr">
         <is>
-          <t>사용 온라인 계정 증거 (네이버·카카오·구글 ID)</t>
+          <t>원화 계좌 → 가상자산 전환 (자금추적 종단 브리지)</t>
         </is>
       </c>
       <c r="G56" s="99" t="inlineStr">
         <is>
-          <t>V4.4 신규 (R3)</t>
+          <t>V4.4 신규 (G6)</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1" s="54">
       <c r="A57" s="98" t="inlineStr">
         <is>
-          <t>B. Case→Object 증거</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B57" s="99" t="inlineStr">
         <is>
-          <t>eg_used_email</t>
+          <t>access_via</t>
         </is>
       </c>
       <c r="C57" s="99" t="inlineStr">
         <is>
-          <t>vt_case</t>
+          <t>vt_access</t>
         </is>
       </c>
       <c r="D57" s="99" t="inlineStr">
         <is>
-          <t>vt_email</t>
+          <t>vt_telno / vt_id / vt_bacnt</t>
         </is>
       </c>
       <c r="E57" s="99" t="inlineStr">
         <is>
-          <t>source_id, rec_created, valid_from, valid_to</t>
+          <t>valid_from, confidence, verified</t>
         </is>
       </c>
       <c r="F57" s="100" t="inlineStr">
         <is>
-          <t>사용 이메일 증거</t>
+          <t>접속 이벤트가 경유·사용한 수단(전화/디지털ID/계좌) 연결</t>
         </is>
       </c>
       <c r="G57" s="99" t="inlineStr">
         <is>
-          <t>V4.4 신규 (R3)</t>
+          <t>V4.5 (access 다형화)</t>
         </is>
       </c>
     </row>
@@ -4641,12 +4719,12 @@
       </c>
       <c r="B58" s="99" t="inlineStr">
         <is>
-          <t>sent_from_ip</t>
+          <t>via_ip</t>
         </is>
       </c>
       <c r="C58" s="99" t="inlineStr">
         <is>
-          <t>vt_msg</t>
+          <t>vt_transfer</t>
         </is>
       </c>
       <c r="D58" s="99" t="inlineStr">
@@ -4656,168 +4734,24 @@
       </c>
       <c r="E58" s="99" t="inlineStr">
         <is>
-          <t>detected_at, source_id</t>
+          <t>source_id, rec_created</t>
         </is>
       </c>
       <c r="F58" s="100" t="inlineStr">
         <is>
-          <t>메시지 발신 시점의 접속 IP (착발신내역이 메시지+접속을 한 레코드로 제공하는 경우)</t>
+          <t>이체 이벤트에 사용된 접속 IP 연결</t>
         </is>
       </c>
       <c r="G58" s="99" t="inlineStr">
         <is>
-          <t>V4.4 신규 (G2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="36" customHeight="1" s="54">
-      <c r="A59" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B59" s="99" t="inlineStr">
-        <is>
-          <t>exchanged_to</t>
-        </is>
-      </c>
-      <c r="C59" s="99" t="inlineStr">
-        <is>
-          <t>vt_bacnt</t>
-        </is>
-      </c>
-      <c r="D59" s="99" t="inlineStr">
-        <is>
-          <t>vt_crypto</t>
-        </is>
-      </c>
-      <c r="E59" s="99" t="inlineStr">
-        <is>
-          <t>exchange_nm, dlng_dt, fiat_amt, asset_amt, confidence, inference</t>
-        </is>
-      </c>
-      <c r="F59" s="100" t="inlineStr">
-        <is>
-          <t>원화 계좌 → 가상자산 전환 (자금추적 종단 브리지)</t>
-        </is>
-      </c>
-      <c r="G59" s="99" t="inlineStr">
-        <is>
-          <t>V4.4 신규 (G6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="16.5" customHeight="1" s="54">
-      <c r="A60" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B60" s="99" t="inlineStr">
-        <is>
-          <t>access_via</t>
-        </is>
-      </c>
-      <c r="C60" s="99" t="inlineStr">
-        <is>
-          <t>vt_access</t>
-        </is>
-      </c>
-      <c r="D60" s="99" t="inlineStr">
-        <is>
-          <t>vt_telno / vt_id / vt_bacnt</t>
-        </is>
-      </c>
-      <c r="E60" s="99" t="inlineStr">
-        <is>
-          <t>valid_from, confidence, verified</t>
-        </is>
-      </c>
-      <c r="F60" s="100" t="inlineStr">
-        <is>
-          <t>접속 이벤트가 경유·사용한 수단(전화/디지털ID/계좌) 연결</t>
-        </is>
-      </c>
-      <c r="G60" s="99" t="inlineStr">
-        <is>
-          <t>V4.5 (access 다형화)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="16.5" customHeight="1" s="54">
-      <c r="A61" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B61" s="99" t="inlineStr">
-        <is>
-          <t>via_ip</t>
-        </is>
-      </c>
-      <c r="C61" s="99" t="inlineStr">
-        <is>
-          <t>vt_transfer</t>
-        </is>
-      </c>
-      <c r="D61" s="99" t="inlineStr">
-        <is>
-          <t>vt_ip</t>
-        </is>
-      </c>
-      <c r="E61" s="99" t="inlineStr">
-        <is>
-          <t>source_id, rec_created</t>
-        </is>
-      </c>
-      <c r="F61" s="100" t="inlineStr">
-        <is>
-          <t>이체 이벤트에 사용된 접속 IP 연결</t>
-        </is>
-      </c>
-      <c r="G61" s="99" t="inlineStr">
-        <is>
           <t>V4.5</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="16.5" customHeight="1" s="54">
-      <c r="A62" s="98" t="inlineStr">
-        <is>
-          <t>I. 위치</t>
-        </is>
-      </c>
-      <c r="B62" s="99" t="inlineStr">
-        <is>
-          <t>mentions_location</t>
-        </is>
-      </c>
-      <c r="C62" s="99" t="inlineStr">
-        <is>
-          <t>vt_msg</t>
-        </is>
-      </c>
-      <c r="D62" s="99" t="inlineStr">
-        <is>
-          <t>vt_loc</t>
-        </is>
-      </c>
-      <c r="E62" s="99" t="inlineStr">
-        <is>
-          <t>confidence, verified</t>
-        </is>
-      </c>
-      <c r="F62" s="100" t="inlineStr">
-        <is>
-          <t>메시지가 언급한 위치 연결</t>
-        </is>
-      </c>
-      <c r="G62" s="99" t="inlineStr">
-        <is>
-          <t>V4.5</t>
-        </is>
-      </c>
-    </row>
+    <row r="59" ht="36" customHeight="1" s="54"/>
+    <row r="60" ht="16.5" customHeight="1" s="54"/>
+    <row r="61" ht="16.5" customHeight="1" s="54"/>
+    <row r="62" ht="16.5" customHeight="1" s="54"/>
     <row r="63" ht="54" customHeight="1" s="54"/>
     <row r="64" ht="54" customHeight="1" s="54"/>
     <row r="65" ht="54" customHeight="1" s="54"/>
@@ -4839,7 +4773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="53" min="1" max="1"/>
@@ -5258,7 +5192,7 @@
       </c>
       <c r="D14" s="85" t="inlineStr">
         <is>
-          <t>id_val (+platform)</t>
+          <t>(platform, id_val) — 이메일은 platform=email, id_val=소문자 주소</t>
         </is>
       </c>
       <c r="E14" s="85" t="inlineStr">
@@ -5268,7 +5202,7 @@
       </c>
       <c r="F14" s="85" t="inlineStr">
         <is>
-          <t>platform, is_anonymous</t>
+          <t>platform, is_anonymous · 이메일(platform=email): domain, provider, is_disposable</t>
         </is>
       </c>
     </row>
@@ -5281,14 +5215,14 @@
           <t>Object</t>
         </is>
       </c>
-      <c r="C15" s="85" t="inlineStr">
-        <is>
-          <t>vt_email</t>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>vt_crypto</t>
         </is>
       </c>
       <c r="D15" s="85" t="inlineStr">
         <is>
-          <t>email_addr</t>
+          <t>wallet_addr</t>
         </is>
       </c>
       <c r="E15" s="85" t="inlineStr">
@@ -5298,7 +5232,7 @@
       </c>
       <c r="F15" s="85" t="inlineStr">
         <is>
-          <t>domain, is_disposable</t>
+          <t>blockchain, risk_score · vt_bacnt→exchanged_to 로 진입</t>
         </is>
       </c>
     </row>
@@ -5311,14 +5245,14 @@
           <t>Object</t>
         </is>
       </c>
-      <c r="C16" s="95" t="inlineStr">
-        <is>
-          <t>vt_crypto</t>
+      <c r="C16" s="85" t="inlineStr">
+        <is>
+          <t>vt_vhcl</t>
         </is>
       </c>
       <c r="D16" s="85" t="inlineStr">
         <is>
-          <t>wallet_addr</t>
+          <t>vhclno</t>
         </is>
       </c>
       <c r="E16" s="85" t="inlineStr">
@@ -5328,7 +5262,7 @@
       </c>
       <c r="F16" s="85" t="inlineStr">
         <is>
-          <t>blockchain, risk_score · vt_bacnt→exchanged_to 로 진입</t>
+          <t>carmdl_nm, stolen_yn</t>
         </is>
       </c>
     </row>
@@ -5341,14 +5275,14 @@
           <t>Object</t>
         </is>
       </c>
-      <c r="C17" s="85" t="inlineStr">
-        <is>
-          <t>vt_vhcl</t>
+      <c r="C17" s="102" t="inlineStr">
+        <is>
+          <t>vt_dev</t>
         </is>
       </c>
       <c r="D17" s="85" t="inlineStr">
         <is>
-          <t>vhclno</t>
+          <t>device_id</t>
         </is>
       </c>
       <c r="E17" s="85" t="inlineStr">
@@ -5358,7 +5292,7 @@
       </c>
       <c r="F17" s="85" t="inlineStr">
         <is>
-          <t>carmdl_nm, stolen_yn</t>
+          <t>dev_type, imei, mac_addr · used_ip 로 IP 연결 가능</t>
         </is>
       </c>
     </row>
@@ -5371,14 +5305,14 @@
           <t>Object</t>
         </is>
       </c>
-      <c r="C18" s="102" t="inlineStr">
-        <is>
-          <t>vt_dev</t>
+      <c r="C18" s="85" t="inlineStr">
+        <is>
+          <t>vt_atm</t>
         </is>
       </c>
       <c r="D18" s="85" t="inlineStr">
         <is>
-          <t>device_id</t>
+          <t>atm_id</t>
         </is>
       </c>
       <c r="E18" s="85" t="inlineStr">
@@ -5388,7 +5322,7 @@
       </c>
       <c r="F18" s="85" t="inlineStr">
         <is>
-          <t>dev_type, imei, mac_addr · used_ip 로 IP 연결 가능</t>
+          <t>bank_nm, address</t>
         </is>
       </c>
     </row>
@@ -5398,27 +5332,27 @@
       </c>
       <c r="B19" s="85" t="inlineStr">
         <is>
-          <t>Object</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="C19" s="85" t="inlineStr">
         <is>
-          <t>vt_atm</t>
+          <t>vt_transfer</t>
         </is>
       </c>
       <c r="D19" s="85" t="inlineStr">
         <is>
-          <t>atm_id</t>
+          <t>transfer_id</t>
         </is>
       </c>
       <c r="E19" s="85" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="F19" s="85" t="inlineStr">
         <is>
-          <t>bank_nm, address</t>
+          <t>dlng_amt, dlng_dt</t>
         </is>
       </c>
     </row>
@@ -5433,12 +5367,12 @@
       </c>
       <c r="C20" s="85" t="inlineStr">
         <is>
-          <t>vt_transfer</t>
+          <t>vt_call</t>
         </is>
       </c>
       <c r="D20" s="85" t="inlineStr">
         <is>
-          <t>transfer_id</t>
+          <t>call_id</t>
         </is>
       </c>
       <c r="E20" s="85" t="inlineStr">
@@ -5448,7 +5382,7 @@
       </c>
       <c r="F20" s="85" t="inlineStr">
         <is>
-          <t>dlng_amt, dlng_dt</t>
+          <t>call_strt_dt, call_dur_sec</t>
         </is>
       </c>
     </row>
@@ -5461,14 +5395,14 @@
           <t>Event</t>
         </is>
       </c>
-      <c r="C21" s="85" t="inlineStr">
-        <is>
-          <t>vt_call</t>
+      <c r="C21" s="102" t="inlineStr">
+        <is>
+          <t>vt_access</t>
         </is>
       </c>
       <c r="D21" s="85" t="inlineStr">
         <is>
-          <t>call_id</t>
+          <t>access_id</t>
         </is>
       </c>
       <c r="E21" s="85" t="inlineStr">
@@ -5478,7 +5412,7 @@
       </c>
       <c r="F21" s="85" t="inlineStr">
         <is>
-          <t>call_strt_dt, call_dur_sec</t>
+          <t>access_dt, actor_type, aggregation_level · 웹로그 5속성 optional</t>
         </is>
       </c>
     </row>
@@ -5493,12 +5427,12 @@
       </c>
       <c r="C22" s="102" t="inlineStr">
         <is>
-          <t>vt_access</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="D22" s="85" t="inlineStr">
         <is>
-          <t>access_id</t>
+          <t>msg_id</t>
         </is>
       </c>
       <c r="E22" s="85" t="inlineStr">
@@ -5508,7 +5442,7 @@
       </c>
       <c r="F22" s="85" t="inlineStr">
         <is>
-          <t>access_dt, actor_type, aggregation_level · 웹로그 5속성 optional</t>
+          <t>msg_type, content_hash, peer_count, aggregation_level</t>
         </is>
       </c>
     </row>
@@ -5521,14 +5455,14 @@
           <t>Event</t>
         </is>
       </c>
-      <c r="C23" s="102" t="inlineStr">
-        <is>
-          <t>vt_msg</t>
+      <c r="C23" s="85" t="inlineStr">
+        <is>
+          <t>vt_movement</t>
         </is>
       </c>
       <c r="D23" s="85" t="inlineStr">
         <is>
-          <t>msg_id</t>
+          <t>mov_id</t>
         </is>
       </c>
       <c r="E23" s="85" t="inlineStr">
@@ -5538,7 +5472,7 @@
       </c>
       <c r="F23" s="85" t="inlineStr">
         <is>
-          <t>msg_type, content_hash, peer_count, aggregation_level</t>
+          <t>mov_type, timestamp</t>
         </is>
       </c>
     </row>
@@ -5553,12 +5487,12 @@
       </c>
       <c r="C24" s="85" t="inlineStr">
         <is>
-          <t>vt_movement</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="D24" s="85" t="inlineStr">
         <is>
-          <t>mov_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E24" s="85" t="inlineStr">
@@ -5568,7 +5502,7 @@
       </c>
       <c r="F24" s="85" t="inlineStr">
         <is>
-          <t>mov_type, timestamp</t>
+          <t>method, fake_name</t>
         </is>
       </c>
     </row>
@@ -5578,60 +5512,31 @@
       </c>
       <c r="B25" s="85" t="inlineStr">
         <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="C25" s="85" t="inlineStr">
-        <is>
-          <t>vt_impersonation</t>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C25" s="95" t="inlineStr">
+        <is>
+          <t>vt_loc</t>
         </is>
       </c>
       <c r="D25" s="85" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>loc_id</t>
         </is>
       </c>
       <c r="E25" s="85" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>plain</t>
         </is>
       </c>
       <c r="F25" s="85" t="inlineStr">
         <is>
-          <t>method, fake_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1" s="54">
-      <c r="A26" s="85" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="85" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="C26" s="95" t="inlineStr">
-        <is>
-          <t>vt_loc</t>
-        </is>
-      </c>
-      <c r="D26" s="85" t="inlineStr">
-        <is>
-          <t>loc_id</t>
-        </is>
-      </c>
-      <c r="E26" s="85" t="inlineStr">
-        <is>
-          <t>plain</t>
-        </is>
-      </c>
-      <c r="F26" s="85" t="inlineStr">
-        <is>
           <t>loc_type(값도메인), address, lat, lng</t>
         </is>
       </c>
     </row>
+    <row r="26" ht="18" customHeight="1" s="54"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9626,12 +9531,12 @@
     <row r="148" ht="18" customHeight="1" s="54">
       <c r="A148" s="104" t="inlineStr">
         <is>
-          <t>vt_email</t>
+          <t>vt_id</t>
         </is>
       </c>
       <c r="B148" s="85" t="inlineStr">
         <is>
-          <t>email_addr</t>
+          <t>platform=email</t>
         </is>
       </c>
       <c r="C148" s="85" t="inlineStr">
@@ -9641,19 +9546,19 @@
       </c>
       <c r="D148" s="86" t="inlineStr">
         <is>
-          <t>이메일 주소(필수 식별자)</t>
+          <t>이메일 주소는 platform='email' 인 vt_id, id_val=소문자 정규화 주소 (V4.9 vt_email 흡수, 구 email_addr)</t>
         </is>
       </c>
       <c r="E148" s="92" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="149" ht="18" customHeight="1" s="54">
       <c r="A149" s="85" t="inlineStr">
         <is>
-          <t>vt_email</t>
+          <t>vt_id</t>
         </is>
       </c>
       <c r="B149" s="85" t="inlineStr">
@@ -9668,7 +9573,7 @@
       </c>
       <c r="D149" s="86" t="inlineStr">
         <is>
-          <t>도메인 부분(추출)</t>
+          <t>도메인 부분(추출) (platform=email)</t>
         </is>
       </c>
       <c r="E149" s="92" t="inlineStr">
@@ -9680,7 +9585,7 @@
     <row r="150" ht="18" customHeight="1" s="54">
       <c r="A150" s="85" t="inlineStr">
         <is>
-          <t>vt_email</t>
+          <t>vt_id</t>
         </is>
       </c>
       <c r="B150" s="85" t="inlineStr">
@@ -9695,7 +9600,7 @@
       </c>
       <c r="D150" s="85" t="inlineStr">
         <is>
-          <t>Gmail|Naver|Daum|Unknown</t>
+          <t>Gmail|Naver|Daum|Unknown (platform=email)</t>
         </is>
       </c>
       <c r="E150" s="92" t="inlineStr">
@@ -9707,7 +9612,7 @@
     <row r="151" ht="18" customHeight="1" s="54">
       <c r="A151" s="85" t="inlineStr">
         <is>
-          <t>vt_email</t>
+          <t>vt_id</t>
         </is>
       </c>
       <c r="B151" s="85" t="inlineStr">
@@ -9722,7 +9627,7 @@
       </c>
       <c r="D151" s="86" t="inlineStr">
         <is>
-          <t>일회용 이메일 여부</t>
+          <t>일회용 이메일 여부 (platform=email)</t>
         </is>
       </c>
       <c r="E151" s="92" t="inlineStr">
@@ -16622,7 +16527,7 @@
       </c>
       <c r="B20" s="110" t="inlineStr">
         <is>
-          <t>61종 (deprecated 0) — V4.9: 추론 결과 엣지 4종 + 중복·폐기 엣지 7종(owns_device·impersonates·involves·owns·verified_by·linked_petition·works_at) 삭제. 검증자는 엣지 메타 verified_by 속성.</t>
+          <t>57종 (deprecated 0) — V4.9: vt_email→vt_id 흡수(uses_email·eg_used_email 삭제) + mentions_* 3종→mentions 통합 + 추론 결과 엣지 4종 + 중복·폐기 엣지 7종(owns_device·impersonates·involves·owns·verified_by·linked_petition·works_at) 삭제. 검증자는 엣지 메타 verified_by 속성.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ontology): V4.9 3단계 — 같은 의미 엣지 4종 통합 (엣지 57→53)
- via_ip(이체→IP)·sent_from_ip(메시지→IP) → accessed_from (Access|Transfer|Message→IP)
  - T2C 학습 프롬프트에 있는 accessed_from 쪽으로 모아 재학습 불요
- occurred_at → located_at (객체 고정 위치 + 이벤트 발생 위치, 출발 라벨로 구분)
  - rdb 적재기가 ATM 고정 위치를 occurred_at 으로 쓰던 것도 located_at 으로 정정
- linked_id → linked_to (link_basis·confidence). valid_from 은 두지 않아 시간 연속성 N형 유지
- parse_kakao_logs: sent_from_ip → accessed_from
- T2C 정적 스키마·방향표 갱신 (t2c_v47 학습 프롬프트 불변), graph_service 는 이전 적재분 조회 호환 유지
- handoff: 정의 스펙 재생성, README·설계이력·엑셀(엣지카탈로그 53종, 변경이력 R27), zip

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
+++ b/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="변경이력(V4.3→V4.9)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="엣지카탈로그(57종)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="엣지카탈로그(53종)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="노드카탈로그(24종)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="노드 속성 사전" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="엣지 속성 사전" sheetId="5" state="visible" r:id="rId5"/>
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="53" min="1" max="1"/>
@@ -2687,6 +2687,43 @@
       <c r="G55" s="53" t="inlineStr">
         <is>
           <t>전 그래프 적재 0건. 명명 동결(학습데이터) 원칙의 예외 — T2C 다음 재학습 시 mentions 표기 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="53" t="inlineStr">
+        <is>
+          <t>R27</t>
+        </is>
+      </c>
+      <c r="B56" s="53" t="inlineStr">
+        <is>
+          <t>V4.9</t>
+        </is>
+      </c>
+      <c r="C56" s="53" t="inlineStr">
+        <is>
+          <t>통합</t>
+        </is>
+      </c>
+      <c r="D56" s="53" t="inlineStr">
+        <is>
+          <t>via_ip · sent_from_ip · occurred_at · linked_id</t>
+        </is>
+      </c>
+      <c r="E56" s="53" t="inlineStr">
+        <is>
+          <t>같은 의미 엣지 4종 (이벤트→IP 3종 · 위치 2종 · 계정 연결 2종)</t>
+        </is>
+      </c>
+      <c r="F56" s="53" t="inlineStr">
+        <is>
+          <t>accessed_from(Access|Transfer|Message→IP) · located_at(객체·이벤트→위치) · linked_to(link_basis) 로 통합 (엣지 57→53)</t>
+        </is>
+      </c>
+      <c r="G56" s="53" t="inlineStr">
+        <is>
+          <t>전 그래프 적재 occurred_at 2건(ku 테스트) 외 0건. T2C 학습 표기(accessed_from)를 남기는 쪽으로 통합해 재학습 불요. ATM 고정 위치를 occurred_at 으로 쓰던 적재기도 located_at 으로 정정</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="53" min="1" max="1"/>
@@ -3773,27 +3810,27 @@
       </c>
       <c r="C31" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>(object) — vt_bacnt/vt_telno/vt_ip 포함</t>
         </is>
       </c>
       <c r="D31" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>(object) — vt_id 포함</t>
         </is>
       </c>
       <c r="E31" s="85" t="inlineStr">
         <is>
-          <t>link_type, confidence</t>
+          <t>link_basis, confidence, source_id, rec_created</t>
         </is>
       </c>
       <c r="F31" s="86" t="inlineStr">
         <is>
-          <t>범용 연결(임시/추론)</t>
+          <t>두 증거의 연결 — 계좌·전화·IP → 계정 역조회 포함 (근거 link_basis)</t>
         </is>
       </c>
       <c r="G31" s="86" t="inlineStr">
         <is>
-          <t>V4.9 중복 행(Petition→Case, deprecated) 정리 — 진정서→사건은 filed_as</t>
+          <t>V4.9 중복 행(Petition→Case, deprecated) 정리 — 진정서→사건은 filed_as · V4.9 linked_id 통합</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4119,7 @@
       </c>
       <c r="C40" s="85" t="inlineStr">
         <is>
-          <t>vt_access</t>
+          <t>vt_access | vt_transfer | vt_msg</t>
         </is>
       </c>
       <c r="D40" s="85" t="inlineStr">
@@ -4092,15 +4129,19 @@
       </c>
       <c r="E40" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>source_id, rec_created</t>
         </is>
       </c>
       <c r="F40" s="86" t="inlineStr">
         <is>
-          <t>접속 출발 IP</t>
-        </is>
-      </c>
-      <c r="G40" s="85" t="n"/>
+          <t>이벤트(접속·이체·메시지 발신)의 출발 IP — 이벤트 종류는 출발 라벨로 구분</t>
+        </is>
+      </c>
+      <c r="G40" s="85" t="inlineStr">
+        <is>
+          <t>V4.9 통합 (via_ip·sent_from_ip) — T2C 학습 표기 유지</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="54">
       <c r="A41" s="90" t="inlineStr">
@@ -4147,17 +4188,17 @@
       </c>
       <c r="B42" s="85" t="inlineStr">
         <is>
-          <t>occurred_at</t>
+          <t>recorded_in</t>
         </is>
       </c>
       <c r="C42" s="85" t="inlineStr">
         <is>
-          <t>(event)</t>
+          <t>vt_vhcl/vt_telno</t>
         </is>
       </c>
       <c r="D42" s="85" t="inlineStr">
         <is>
-          <t>vt_loc</t>
+          <t>vt_movement</t>
         </is>
       </c>
       <c r="E42" s="85" t="inlineStr">
@@ -4167,7 +4208,7 @@
       </c>
       <c r="F42" s="86" t="inlineStr">
         <is>
-          <t>이벤트 발생 위치</t>
+          <t>이동 기록의 주체</t>
         </is>
       </c>
       <c r="G42" s="85" t="n"/>
@@ -4180,27 +4221,27 @@
       </c>
       <c r="B43" s="85" t="inlineStr">
         <is>
-          <t>recorded_in</t>
+          <t>used_in_device</t>
         </is>
       </c>
       <c r="C43" s="85" t="inlineStr">
         <is>
-          <t>vt_vhcl/vt_telno</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="D43" s="85" t="inlineStr">
         <is>
-          <t>vt_movement</t>
+          <t>vt_dev</t>
         </is>
       </c>
       <c r="E43" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>valid_from, valid_to, source_id</t>
         </is>
       </c>
       <c r="F43" s="86" t="inlineStr">
         <is>
-          <t>이동 기록의 주체</t>
+          <t>전화-기기(IMEI) 사용</t>
         </is>
       </c>
       <c r="G43" s="85" t="n"/>
@@ -4208,32 +4249,32 @@
     <row r="44" ht="18" customHeight="1" s="54">
       <c r="A44" s="84" t="inlineStr">
         <is>
-          <t>F. Event 흐름</t>
+          <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B44" s="85" t="inlineStr">
         <is>
-          <t>used_in_device</t>
+          <t>used_for</t>
         </is>
       </c>
       <c r="C44" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>(object)</t>
         </is>
       </c>
       <c r="D44" s="85" t="inlineStr">
         <is>
-          <t>vt_dev</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="E44" s="85" t="inlineStr">
         <is>
-          <t>valid_from, valid_to, source_id</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F44" s="86" t="inlineStr">
         <is>
-          <t>전화-기기(IMEI) 사용</t>
+          <t>사칭에 사용된 객체</t>
         </is>
       </c>
       <c r="G44" s="85" t="n"/>
@@ -4246,17 +4287,17 @@
       </c>
       <c r="B45" s="85" t="inlineStr">
         <is>
-          <t>used_for</t>
+          <t>targets</t>
         </is>
       </c>
       <c r="C45" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="D45" s="85" t="inlineStr">
         <is>
-          <t>vt_impersonation</t>
+          <t>vt_org</t>
         </is>
       </c>
       <c r="E45" s="85" t="inlineStr">
@@ -4266,189 +4307,193 @@
       </c>
       <c r="F45" s="86" t="inlineStr">
         <is>
-          <t>사칭에 사용된 객체</t>
+          <t>사칭 대상 기관</t>
         </is>
       </c>
       <c r="G45" s="85" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1" s="54">
-      <c r="A46" s="84" t="inlineStr">
+      <c r="A46" s="88" t="inlineStr">
         <is>
           <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B46" s="85" t="inlineStr">
         <is>
-          <t>targets</t>
+          <t>performed_by</t>
         </is>
       </c>
       <c r="C46" s="85" t="inlineStr">
         <is>
-          <t>vt_impersonation</t>
+          <t>vt_access/vt_movement</t>
         </is>
       </c>
       <c r="D46" s="85" t="inlineStr">
         <is>
-          <t>vt_org</t>
+          <t>vt_psn / vt_telno / vt_id</t>
         </is>
       </c>
       <c r="E46" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>actor_type, resolved_to, resolved_at</t>
         </is>
       </c>
       <c r="F46" s="86" t="inlineStr">
         <is>
-          <t>사칭 대상 기관</t>
-        </is>
-      </c>
-      <c r="G46" s="85" t="n"/>
+          <t>접속·이동 수행 주체 (인물 미특정 단계에서는 번호·계정을 주체로 기록)</t>
+        </is>
+      </c>
+      <c r="G46" s="85" t="inlineStr">
+        <is>
+          <t>V4.4 range 확장 (G1)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1" s="54">
-      <c r="A47" s="88" t="inlineStr">
-        <is>
-          <t>G. 사칭/접속주체</t>
+      <c r="A47" s="84" t="inlineStr">
+        <is>
+          <t>H. Provenance</t>
         </is>
       </c>
       <c r="B47" s="85" t="inlineStr">
         <is>
-          <t>performed_by</t>
+          <t>sourced_from</t>
         </is>
       </c>
       <c r="C47" s="85" t="inlineStr">
         <is>
-          <t>vt_access/vt_movement</t>
+          <t>(any)</t>
         </is>
       </c>
       <c r="D47" s="85" t="inlineStr">
         <is>
-          <t>vt_psn / vt_telno / vt_id</t>
+          <t>vt_src</t>
         </is>
       </c>
       <c r="E47" s="85" t="inlineStr">
         <is>
-          <t>actor_type, resolved_to, resolved_at</t>
+          <t>src_tier, rec_created</t>
         </is>
       </c>
       <c r="F47" s="86" t="inlineStr">
         <is>
-          <t>접속·이동 수행 주체 (인물 미특정 단계에서는 번호·계정을 주체로 기록)</t>
+          <t>데이터 출처 참조</t>
         </is>
       </c>
       <c r="G47" s="85" t="inlineStr">
         <is>
-          <t>V4.4 range 확장 (G1)</t>
+          <t>tier1~3만 엣지 생성</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1" s="54">
-      <c r="A48" s="84" t="inlineStr">
-        <is>
-          <t>H. Provenance</t>
-        </is>
-      </c>
-      <c r="B48" s="85" t="inlineStr">
-        <is>
-          <t>sourced_from</t>
-        </is>
-      </c>
-      <c r="C48" s="85" t="inlineStr">
-        <is>
-          <t>(any)</t>
-        </is>
-      </c>
-      <c r="D48" s="85" t="inlineStr">
-        <is>
-          <t>vt_src</t>
-        </is>
-      </c>
-      <c r="E48" s="85" t="inlineStr">
-        <is>
-          <t>src_tier, rec_created</t>
-        </is>
-      </c>
-      <c r="F48" s="86" t="inlineStr">
-        <is>
-          <t>데이터 출처 참조</t>
-        </is>
-      </c>
-      <c r="G48" s="85" t="inlineStr">
-        <is>
-          <t>tier1~3만 엣지 생성</t>
+      <c r="A48" s="91" t="inlineStr">
+        <is>
+          <t>C. Person 관계</t>
+        </is>
+      </c>
+      <c r="B48" s="53" t="inlineStr">
+        <is>
+          <t>controls</t>
+        </is>
+      </c>
+      <c r="C48" s="53" t="inlineStr">
+        <is>
+          <t>vt_psn</t>
+        </is>
+      </c>
+      <c r="D48" s="53" t="inlineStr">
+        <is>
+          <t>vt_bacnt</t>
+        </is>
+      </c>
+      <c r="E48" s="53" t="inlineStr">
+        <is>
+          <t>confidence, inference_basis_type, evidence_edge_ids, evidence_count, evidence_summary</t>
+        </is>
+      </c>
+      <c r="F48" s="92" t="inlineStr">
+        <is>
+          <t>실질 지배(명의≠실사용)</t>
+        </is>
+      </c>
+      <c r="G48" s="92" t="inlineStr">
+        <is>
+          <t>정합화 등재 V4.4 근거 구조화 (G7)</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1" s="54">
-      <c r="A49" s="91" t="inlineStr">
-        <is>
-          <t>C. Person 관계</t>
+      <c r="A49" s="93" t="inlineStr">
+        <is>
+          <t>I. 위치</t>
         </is>
       </c>
       <c r="B49" s="53" t="inlineStr">
         <is>
-          <t>controls</t>
+          <t>located_at</t>
         </is>
       </c>
       <c r="C49" s="53" t="inlineStr">
         <is>
+          <t>vt_atm/vt_org · (event)</t>
+        </is>
+      </c>
+      <c r="D49" s="53" t="inlineStr">
+        <is>
+          <t>vt_loc</t>
+        </is>
+      </c>
+      <c r="E49" s="53" t="inlineStr">
+        <is>
+          <t>first_dt, last_dt, evt_count, source_id</t>
+        </is>
+      </c>
+      <c r="F49" s="92" t="inlineStr">
+        <is>
+          <t>객체의 위치 또는 이벤트의 발생 위치 — 출발 라벨로 구분</t>
+        </is>
+      </c>
+      <c r="G49" s="92" t="inlineStr">
+        <is>
+          <t>정합화 등재 · V4.9 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count · V4.9 occurred_at 통합</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="54">
+      <c r="A50" s="94" t="inlineStr">
+        <is>
+          <t>J. V4.3 시나리오</t>
+        </is>
+      </c>
+      <c r="B50" s="85" t="inlineStr">
+        <is>
+          <t>knows</t>
+        </is>
+      </c>
+      <c r="C50" s="85" t="inlineStr">
+        <is>
           <t>vt_psn</t>
         </is>
       </c>
-      <c r="D49" s="53" t="inlineStr">
-        <is>
-          <t>vt_bacnt</t>
-        </is>
-      </c>
-      <c r="E49" s="53" t="inlineStr">
-        <is>
-          <t>confidence, inference_basis_type, evidence_edge_ids, evidence_count, evidence_summary</t>
-        </is>
-      </c>
-      <c r="F49" s="92" t="inlineStr">
-        <is>
-          <t>실질 지배(명의≠실사용)</t>
-        </is>
-      </c>
-      <c r="G49" s="92" t="inlineStr">
-        <is>
-          <t>정합화 등재 V4.4 근거 구조화 (G7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1" s="54">
-      <c r="A50" s="93" t="inlineStr">
-        <is>
-          <t>I. 위치</t>
-        </is>
-      </c>
-      <c r="B50" s="53" t="inlineStr">
-        <is>
-          <t>located_at</t>
-        </is>
-      </c>
-      <c r="C50" s="53" t="inlineStr">
-        <is>
-          <t>vt_atm/vt_org</t>
-        </is>
-      </c>
-      <c r="D50" s="53" t="inlineStr">
-        <is>
-          <t>vt_loc</t>
-        </is>
-      </c>
-      <c r="E50" s="53" t="inlineStr">
-        <is>
-          <t>first_dt, last_dt, evt_count, source_id</t>
-        </is>
-      </c>
-      <c r="F50" s="92" t="inlineStr">
-        <is>
-          <t>고정 객체의 정적 위치</t>
-        </is>
-      </c>
-      <c r="G50" s="92" t="inlineStr">
-        <is>
-          <t>정합화 등재 · V4.9 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count</t>
+      <c r="D50" s="85" t="inlineStr">
+        <is>
+          <t>vt_psn</t>
+        </is>
+      </c>
+      <c r="E50" s="85" t="inlineStr">
+        <is>
+          <t>relation_type, confidence, valid_from</t>
+        </is>
+      </c>
+      <c r="F50" s="86" t="inlineStr">
+        <is>
+          <t>두 인물의 사회적 지인 관계 (고향친구/동창 — 공범 여부는 그래프 엣지가 아니라 탐지 결과로 판단)</t>
+        </is>
+      </c>
+      <c r="G50" s="85" t="inlineStr">
+        <is>
+          <t>V4.3 신규</t>
         </is>
       </c>
     </row>
@@ -4460,294 +4505,150 @@
       </c>
       <c r="B51" s="85" t="inlineStr">
         <is>
-          <t>knows</t>
+          <t>mentions</t>
         </is>
       </c>
       <c r="C51" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="D51" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_id | vt_bacnt | vt_loc</t>
         </is>
       </c>
       <c r="E51" s="85" t="inlineStr">
         <is>
-          <t>relation_type, confidence, valid_from</t>
+          <t>confidence, extract_method, source_id, rec_created</t>
         </is>
       </c>
       <c r="F51" s="86" t="inlineStr">
         <is>
-          <t>두 인물의 사회적 지인 관계 (고향친구/동창 — 공범 여부는 그래프 엣지가 아니라 탐지 결과로 판단)</t>
+          <t>메시지·게시물 본문에 계정·계좌·장소가 기재됨 — 종류는 도착 라벨로 구분</t>
         </is>
       </c>
       <c r="G51" s="85" t="inlineStr">
         <is>
-          <t>V4.3 신규</t>
+          <t>V4.9 통합 (mentions_id·mentions_account·mentions_location)</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="54">
-      <c r="A52" s="95" t="inlineStr">
-        <is>
-          <t>J. V4.3 시나리오</t>
-        </is>
-      </c>
-      <c r="B52" s="85" t="inlineStr">
-        <is>
-          <t>linked_id</t>
-        </is>
-      </c>
-      <c r="C52" s="85" t="inlineStr">
-        <is>
-          <t>vt_bacnt / vt_telno / vt_ip</t>
-        </is>
-      </c>
-      <c r="D52" s="85" t="inlineStr">
+      <c r="A52" s="98" t="inlineStr">
+        <is>
+          <t>B. Case→Object 증거</t>
+        </is>
+      </c>
+      <c r="B52" s="99" t="inlineStr">
+        <is>
+          <t>eg_used_id</t>
+        </is>
+      </c>
+      <c r="C52" s="99" t="inlineStr">
+        <is>
+          <t>vt_case</t>
+        </is>
+      </c>
+      <c r="D52" s="99" t="inlineStr">
         <is>
           <t>vt_id</t>
         </is>
       </c>
-      <c r="E52" s="85" t="inlineStr">
-        <is>
-          <t>link_basis, confidence, valid_from, valid_to, warrant_no</t>
-        </is>
-      </c>
-      <c r="F52" s="86" t="inlineStr">
-        <is>
-          <t>객체에 연결된 온라인 식별자 (공인인증서 발급 ID / 포털·통신사·금융 역조회 결과)</t>
-        </is>
-      </c>
-      <c r="G52" s="85" t="inlineStr">
-        <is>
-          <t>V4.3 신규 → V4.4 domain에 vt_ip 추가 (G4)</t>
+      <c r="E52" s="99" t="inlineStr">
+        <is>
+          <t>source_id, rec_created, valid_from, valid_to</t>
+        </is>
+      </c>
+      <c r="F52" s="100" t="inlineStr">
+        <is>
+          <t>사용 온라인 계정 증거 (네이버·카카오·구글 ID)</t>
+        </is>
+      </c>
+      <c r="G52" s="99" t="inlineStr">
+        <is>
+          <t>V4.4 신규 (R3)</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" s="54">
-      <c r="A53" s="94" t="inlineStr">
-        <is>
-          <t>J. V4.3 시나리오</t>
-        </is>
-      </c>
-      <c r="B53" s="85" t="inlineStr">
-        <is>
-          <t>mentions</t>
-        </is>
-      </c>
-      <c r="C53" s="85" t="inlineStr">
-        <is>
-          <t>vt_msg</t>
-        </is>
-      </c>
-      <c r="D53" s="85" t="inlineStr">
-        <is>
-          <t>vt_id | vt_bacnt | vt_loc</t>
-        </is>
-      </c>
-      <c r="E53" s="85" t="inlineStr">
-        <is>
-          <t>confidence, extract_method, source_id, rec_created</t>
-        </is>
-      </c>
-      <c r="F53" s="86" t="inlineStr">
-        <is>
-          <t>메시지·게시물 본문에 계정·계좌·장소가 기재됨 — 종류는 도착 라벨로 구분</t>
-        </is>
-      </c>
-      <c r="G53" s="85" t="inlineStr">
-        <is>
-          <t>V4.9 통합 (mentions_id·mentions_account·mentions_location)</t>
+      <c r="A53" s="98" t="inlineStr">
+        <is>
+          <t>F. Event 흐름</t>
+        </is>
+      </c>
+      <c r="B53" s="99" t="inlineStr">
+        <is>
+          <t>exchanged_to</t>
+        </is>
+      </c>
+      <c r="C53" s="99" t="inlineStr">
+        <is>
+          <t>vt_bacnt</t>
+        </is>
+      </c>
+      <c r="D53" s="99" t="inlineStr">
+        <is>
+          <t>vt_crypto</t>
+        </is>
+      </c>
+      <c r="E53" s="99" t="inlineStr">
+        <is>
+          <t>exchange_nm, dlng_dt, fiat_amt, asset_amt, confidence, inference</t>
+        </is>
+      </c>
+      <c r="F53" s="100" t="inlineStr">
+        <is>
+          <t>원화 계좌 → 가상자산 전환 (자금추적 종단 브리지)</t>
+        </is>
+      </c>
+      <c r="G53" s="99" t="inlineStr">
+        <is>
+          <t>V4.4 신규 (G6)</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" s="54">
       <c r="A54" s="98" t="inlineStr">
         <is>
-          <t>B. Case→Object 증거</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B54" s="99" t="inlineStr">
         <is>
-          <t>eg_used_id</t>
+          <t>access_via</t>
         </is>
       </c>
       <c r="C54" s="99" t="inlineStr">
         <is>
-          <t>vt_case</t>
+          <t>vt_access</t>
         </is>
       </c>
       <c r="D54" s="99" t="inlineStr">
         <is>
-          <t>vt_id</t>
+          <t>vt_telno / vt_id / vt_bacnt</t>
         </is>
       </c>
       <c r="E54" s="99" t="inlineStr">
         <is>
-          <t>source_id, rec_created, valid_from, valid_to</t>
+          <t>valid_from, confidence, verified</t>
         </is>
       </c>
       <c r="F54" s="100" t="inlineStr">
         <is>
-          <t>사용 온라인 계정 증거 (네이버·카카오·구글 ID)</t>
+          <t>접속 이벤트가 경유·사용한 수단(전화/디지털ID/계좌) 연결</t>
         </is>
       </c>
       <c r="G54" s="99" t="inlineStr">
         <is>
-          <t>V4.4 신규 (R3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1" s="54">
-      <c r="A55" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B55" s="99" t="inlineStr">
-        <is>
-          <t>sent_from_ip</t>
-        </is>
-      </c>
-      <c r="C55" s="99" t="inlineStr">
-        <is>
-          <t>vt_msg</t>
-        </is>
-      </c>
-      <c r="D55" s="99" t="inlineStr">
-        <is>
-          <t>vt_ip</t>
-        </is>
-      </c>
-      <c r="E55" s="99" t="inlineStr">
-        <is>
-          <t>detected_at, source_id</t>
-        </is>
-      </c>
-      <c r="F55" s="100" t="inlineStr">
-        <is>
-          <t>메시지 발신 시점의 접속 IP (착발신내역이 메시지+접속을 한 레코드로 제공하는 경우)</t>
-        </is>
-      </c>
-      <c r="G55" s="99" t="inlineStr">
-        <is>
-          <t>V4.4 신규 (G2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="36" customHeight="1" s="54">
-      <c r="A56" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B56" s="99" t="inlineStr">
-        <is>
-          <t>exchanged_to</t>
-        </is>
-      </c>
-      <c r="C56" s="99" t="inlineStr">
-        <is>
-          <t>vt_bacnt</t>
-        </is>
-      </c>
-      <c r="D56" s="99" t="inlineStr">
-        <is>
-          <t>vt_crypto</t>
-        </is>
-      </c>
-      <c r="E56" s="99" t="inlineStr">
-        <is>
-          <t>exchange_nm, dlng_dt, fiat_amt, asset_amt, confidence, inference</t>
-        </is>
-      </c>
-      <c r="F56" s="100" t="inlineStr">
-        <is>
-          <t>원화 계좌 → 가상자산 전환 (자금추적 종단 브리지)</t>
-        </is>
-      </c>
-      <c r="G56" s="99" t="inlineStr">
-        <is>
-          <t>V4.4 신규 (G6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1" s="54">
-      <c r="A57" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B57" s="99" t="inlineStr">
-        <is>
-          <t>access_via</t>
-        </is>
-      </c>
-      <c r="C57" s="99" t="inlineStr">
-        <is>
-          <t>vt_access</t>
-        </is>
-      </c>
-      <c r="D57" s="99" t="inlineStr">
-        <is>
-          <t>vt_telno / vt_id / vt_bacnt</t>
-        </is>
-      </c>
-      <c r="E57" s="99" t="inlineStr">
-        <is>
-          <t>valid_from, confidence, verified</t>
-        </is>
-      </c>
-      <c r="F57" s="100" t="inlineStr">
-        <is>
-          <t>접속 이벤트가 경유·사용한 수단(전화/디지털ID/계좌) 연결</t>
-        </is>
-      </c>
-      <c r="G57" s="99" t="inlineStr">
-        <is>
           <t>V4.5 (access 다형화)</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="18" customHeight="1" s="54">
-      <c r="A58" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B58" s="99" t="inlineStr">
-        <is>
-          <t>via_ip</t>
-        </is>
-      </c>
-      <c r="C58" s="99" t="inlineStr">
-        <is>
-          <t>vt_transfer</t>
-        </is>
-      </c>
-      <c r="D58" s="99" t="inlineStr">
-        <is>
-          <t>vt_ip</t>
-        </is>
-      </c>
-      <c r="E58" s="99" t="inlineStr">
-        <is>
-          <t>source_id, rec_created</t>
-        </is>
-      </c>
-      <c r="F58" s="100" t="inlineStr">
-        <is>
-          <t>이체 이벤트에 사용된 접속 IP 연결</t>
-        </is>
-      </c>
-      <c r="G58" s="99" t="inlineStr">
-        <is>
-          <t>V4.5</t>
-        </is>
-      </c>
-    </row>
+    <row r="55" ht="18" customHeight="1" s="54"/>
+    <row r="56" ht="36" customHeight="1" s="54"/>
+    <row r="57" ht="18" customHeight="1" s="54"/>
+    <row r="58" ht="18" customHeight="1" s="54"/>
     <row r="59" ht="36" customHeight="1" s="54"/>
     <row r="60" ht="16.5" customHeight="1" s="54"/>
     <row r="61" ht="16.5" customHeight="1" s="54"/>
@@ -13536,7 +13437,7 @@
       </c>
       <c r="D28" s="85" t="inlineStr">
         <is>
-          <t>linked_id</t>
+          <t>linked_to(구 linked_id)</t>
         </is>
       </c>
       <c r="E28" s="86" t="inlineStr">
@@ -13833,7 +13734,7 @@
       </c>
       <c r="D39" s="99" t="inlineStr">
         <is>
-          <t>linked_id, eg_used_* 4종</t>
+          <t>linked_to(구 linked_id), eg_used_* 4종</t>
         </is>
       </c>
       <c r="E39" s="100" t="inlineStr">
@@ -14461,7 +14362,7 @@
       </c>
       <c r="B2" s="99" t="inlineStr">
         <is>
-          <t>linked_id</t>
+          <t>linked_to(구 linked_id)</t>
         </is>
       </c>
       <c r="C2" s="105" t="inlineStr">
@@ -14479,7 +14380,7 @@
       <c r="A3" s="105" t="n"/>
       <c r="B3" s="99" t="inlineStr">
         <is>
-          <t>linked_id</t>
+          <t>linked_to(구 linked_id)</t>
         </is>
       </c>
       <c r="C3" s="105" t="inlineStr">
@@ -14497,7 +14398,7 @@
       <c r="A4" s="105" t="n"/>
       <c r="B4" s="99" t="inlineStr">
         <is>
-          <t>linked_id</t>
+          <t>linked_to(구 linked_id)</t>
         </is>
       </c>
       <c r="C4" s="105" t="inlineStr">
@@ -14515,7 +14416,7 @@
       <c r="A5" s="105" t="n"/>
       <c r="B5" s="99" t="inlineStr">
         <is>
-          <t>linked_id</t>
+          <t>linked_to(구 linked_id)</t>
         </is>
       </c>
       <c r="C5" s="105" t="inlineStr">
@@ -16527,7 +16428,7 @@
       </c>
       <c r="B20" s="110" t="inlineStr">
         <is>
-          <t>57종 (deprecated 0) — V4.9: vt_email→vt_id 흡수(uses_email·eg_used_email 삭제) + mentions_* 3종→mentions 통합 + 추론 결과 엣지 4종 + 중복·폐기 엣지 7종(owns_device·impersonates·involves·owns·verified_by·linked_petition·works_at) 삭제. 검증자는 엣지 메타 verified_by 속성.</t>
+          <t>53종 (deprecated 0) — V4.9: via_ip·sent_from_ip→accessed_from·occurred_at→located_at·linked_id→linked_to 통합 + vt_email→vt_id 흡수(uses_email·eg_used_email 삭제) + mentions_* 3종→mentions 통합 + 추론 결과 엣지 4종 + 중복·폐기 엣지 7종(owns_device·impersonates·involves·owns·verified_by·linked_petition·works_at) 삭제. 검증자는 엣지 메타 verified_by 속성.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ontology): V4.9 — hosts→resolves_to(basis) 통합 (엣지 53→52)
- hosts(IP→사이트) 삭제, resolves_to(사이트→IP)에 basis 속성 추가
  - 'dns' = DNS 조회 관측(기본), 'origin' = 원본 서버 확인(호스팅사 회신·압수)
  - resolves_to 의 inference 표시 제거 (DNS 결과는 관측 사실) → SoT 추론 표시 엣지 0종
  - 근거: osint_ontology 13,769건이 모두 DNS 결과의 역방향 복사본(짝 없는 hosts 0건, 속성 없음)
- OSINT 제출 검증기·적재기: 이전 표기 변환(normalize_edge)
  - hosts → resolves_to(방향 반전, basis=origin), mentions_account → mentions, sameAs → same_as
  - 경고 후 변환 적재, resolves_to basis 기본값 dns
- OSINT 빌더 2종의 hosts 라벨 선언 제거, UI 엣지 선택지·예시 질의 resolves_to 로
- graph_service 방향표는 이전 적재분 조회 호환 유지
- handoff: 정의 스펙 재생성, README·설계이력·엑셀(엣지카탈로그 52종, basis 속성, 변경이력 R28), zip

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
+++ b/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="변경이력(V4.3→V4.9)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="엣지카탈로그(53종)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="엣지카탈로그(52종)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="노드카탈로그(24종)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="노드 속성 사전" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="엣지 속성 사전" sheetId="5" state="visible" r:id="rId5"/>
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="53" min="1" max="1"/>
@@ -2724,6 +2724,43 @@
       <c r="G56" s="53" t="inlineStr">
         <is>
           <t>전 그래프 적재 occurred_at 2건(ku 테스트) 외 0건. T2C 학습 표기(accessed_from)를 남기는 쪽으로 통합해 재학습 불요. ATM 고정 위치를 occurred_at 으로 쓰던 적재기도 located_at 으로 정정</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="53" t="inlineStr">
+        <is>
+          <t>R28</t>
+        </is>
+      </c>
+      <c r="B57" s="53" t="inlineStr">
+        <is>
+          <t>V4.9</t>
+        </is>
+      </c>
+      <c r="C57" s="53" t="inlineStr">
+        <is>
+          <t>통합</t>
+        </is>
+      </c>
+      <c r="D57" s="53" t="inlineStr">
+        <is>
+          <t>hosts → resolves_to</t>
+        </is>
+      </c>
+      <c r="E57" s="53" t="inlineStr">
+        <is>
+          <t>hosts(IP→사이트)·resolves_to(사이트→IP) 별도 엣지, resolves_to 는 추론 표시</t>
+        </is>
+      </c>
+      <c r="F57" s="53" t="inlineStr">
+        <is>
+          <t>resolves_to 1종 + basis('dns' DNS 관측 · 'origin' 원본 서버 확인), 추론 표시 제거 (엣지 53→52)</t>
+        </is>
+      </c>
+      <c r="G57" s="53" t="inlineStr">
+        <is>
+          <t>OSINT 13,769건이 모두 DNS 결과의 역방향 복사본(짝 없는 hosts 0건, 속성 없음). 호스팅·DNS 구분은 CDN·가상호스팅 수사에 필요해 속성으로 보존. OSINT 제출 hosts 는 경고 후 변환</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="53" min="1" max="1"/>
@@ -3603,27 +3640,27 @@
       </c>
       <c r="B25" s="85" t="inlineStr">
         <is>
-          <t>hosts</t>
+          <t>belongs_to</t>
         </is>
       </c>
       <c r="C25" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D25" s="85" t="inlineStr">
         <is>
-          <t>vt_site</t>
+          <t>vt_org</t>
         </is>
       </c>
       <c r="E25" s="85" t="inlineStr">
         <is>
-          <t>port, detected_at</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F25" s="86" t="inlineStr">
         <is>
-          <t>서버 IP가 사이트 호스팅</t>
+          <t>계좌 소속 금융기관</t>
         </is>
       </c>
       <c r="G25" s="85" t="n"/>
@@ -3636,30 +3673,34 @@
       </c>
       <c r="B26" s="85" t="inlineStr">
         <is>
-          <t>belongs_to</t>
+          <t>resolves_to</t>
         </is>
       </c>
       <c r="C26" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_site</t>
         </is>
       </c>
       <c r="D26" s="85" t="inlineStr">
         <is>
-          <t>vt_org</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="E26" s="85" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="86" t="inlineStr">
-        <is>
-          <t>계좌 소속 금융기관</t>
-        </is>
-      </c>
-      <c r="G26" s="85" t="n"/>
+          <t>basis, resolved_dt, port</t>
+        </is>
+      </c>
+      <c r="F26" s="85" t="inlineStr">
+        <is>
+          <t>사이트→IP 연결 — basis 'dns'(DNS 조회 관측) · 'origin'(원본 서버 확인)</t>
+        </is>
+      </c>
+      <c r="G26" s="85" t="inlineStr">
+        <is>
+          <t>V4.9 hosts 통합 (OSINT 13,769건은 DNS 결과 역방향 복사본)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="54">
       <c r="A27" s="84" t="inlineStr">
@@ -3669,27 +3710,27 @@
       </c>
       <c r="B27" s="85" t="inlineStr">
         <is>
-          <t>resolves_to</t>
+          <t>contains_file</t>
         </is>
       </c>
       <c r="C27" s="85" t="inlineStr">
         <is>
-          <t>vt_site</t>
+          <t>vt_site/vt_msg/vt_id</t>
         </is>
       </c>
       <c r="D27" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_file</t>
         </is>
       </c>
       <c r="E27" s="85" t="inlineStr">
         <is>
-          <t>resolved_dt</t>
-        </is>
-      </c>
-      <c r="F27" s="85" t="inlineStr">
-        <is>
-          <t>DNS 해석 결과</t>
+          <t>file_role, detected_at</t>
+        </is>
+      </c>
+      <c r="F27" s="86" t="inlineStr">
+        <is>
+          <t>파일 내장·배포</t>
         </is>
       </c>
       <c r="G27" s="85" t="n"/>
@@ -3702,98 +3743,102 @@
       </c>
       <c r="B28" s="85" t="inlineStr">
         <is>
-          <t>contains_file</t>
+          <t>communicated_with</t>
         </is>
       </c>
       <c r="C28" s="85" t="inlineStr">
         <is>
-          <t>vt_site/vt_msg/vt_id</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="D28" s="85" t="inlineStr">
         <is>
-          <t>vt_file</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="E28" s="85" t="inlineStr">
         <is>
-          <t>file_role, detected_at</t>
-        </is>
-      </c>
-      <c r="F28" s="86" t="inlineStr">
-        <is>
-          <t>파일 내장·배포</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="85" t="inlineStr">
+        <is>
+          <t>IP 간 직접 통신</t>
         </is>
       </c>
       <c r="G28" s="85" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1" s="54">
-      <c r="A29" s="84" t="inlineStr">
+      <c r="A29" s="88" t="inlineStr">
         <is>
           <t>E. Object 관계</t>
         </is>
       </c>
       <c r="B29" s="85" t="inlineStr">
         <is>
-          <t>communicated_with</t>
+          <t>transferred_to</t>
         </is>
       </c>
       <c r="C29" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D29" s="85" t="inlineStr">
         <is>
-          <t>vt_ip</t>
+          <t>vt_bacnt / vt_crypto</t>
         </is>
       </c>
       <c r="E29" s="85" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="85" t="inlineStr">
-        <is>
-          <t>IP 간 직접 통신</t>
-        </is>
-      </c>
-      <c r="G29" s="85" t="n"/>
+          <t>first_dlng_dt, last_dlng_dt, txn_count, total_amount, channel</t>
+        </is>
+      </c>
+      <c r="F29" s="86" t="inlineStr">
+        <is>
+          <t>계좌(지갑) 간 이체 — 건별 거래를 (보낸 쪽, 받는 쪽) 쌍당 1엣지로 집계한 원천 사실</t>
+        </is>
+      </c>
+      <c r="G29" s="85" t="inlineStr">
+        <is>
+          <t>V4.9 직접 엣지로 재정의(추론·직접생성 금지 해제) · 다단계 흐름은 경로 조회 · (쌍) 집계</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="54">
-      <c r="A30" s="88" t="inlineStr">
+      <c r="A30" s="84" t="inlineStr">
         <is>
           <t>E. Object 관계</t>
         </is>
       </c>
       <c r="B30" s="85" t="inlineStr">
         <is>
-          <t>transferred_to</t>
+          <t>linked_to</t>
         </is>
       </c>
       <c r="C30" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>(object) — vt_bacnt/vt_telno/vt_ip 포함</t>
         </is>
       </c>
       <c r="D30" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt / vt_crypto</t>
+          <t>(object) — vt_id 포함</t>
         </is>
       </c>
       <c r="E30" s="85" t="inlineStr">
         <is>
-          <t>first_dlng_dt, last_dlng_dt, txn_count, total_amount, channel</t>
+          <t>link_basis, confidence, source_id, rec_created</t>
         </is>
       </c>
       <c r="F30" s="86" t="inlineStr">
         <is>
-          <t>계좌(지갑) 간 이체 — 건별 거래를 (보낸 쪽, 받는 쪽) 쌍당 1엣지로 집계한 원천 사실</t>
-        </is>
-      </c>
-      <c r="G30" s="85" t="inlineStr">
-        <is>
-          <t>V4.9 직접 엣지로 재정의(추론·직접생성 금지 해제) · 다단계 흐름은 경로 조회 · (쌍) 집계</t>
+          <t>두 증거의 연결 — 계좌·전화·IP → 계정 역조회 포함 (근거 link_basis)</t>
+        </is>
+      </c>
+      <c r="G30" s="86" t="inlineStr">
+        <is>
+          <t>V4.9 중복 행(Petition→Case, deprecated) 정리 — 진정서→사건은 filed_as · V4.9 linked_id 통합</t>
         </is>
       </c>
     </row>
@@ -3805,71 +3850,67 @@
       </c>
       <c r="B31" s="85" t="inlineStr">
         <is>
-          <t>linked_to</t>
+          <t>belongs_to_campaign</t>
         </is>
       </c>
       <c r="C31" s="85" t="inlineStr">
         <is>
-          <t>(object) — vt_bacnt/vt_telno/vt_ip 포함</t>
+          <t>vt_site</t>
         </is>
       </c>
       <c r="D31" s="85" t="inlineStr">
         <is>
-          <t>(object) — vt_id 포함</t>
+          <t>site_cluster</t>
         </is>
       </c>
       <c r="E31" s="85" t="inlineStr">
         <is>
-          <t>link_basis, confidence, source_id, rec_created</t>
+          <t>sim_score, detected_at</t>
         </is>
       </c>
       <c r="F31" s="86" t="inlineStr">
         <is>
-          <t>두 증거의 연결 — 계좌·전화·IP → 계정 역조회 포함 (근거 link_basis)</t>
-        </is>
-      </c>
-      <c r="G31" s="86" t="inlineStr">
-        <is>
-          <t>V4.9 중복 행(Petition→Case, deprecated) 정리 — 진정서→사건은 filed_as · V4.9 linked_id 통합</t>
+          <t>피싱 캠페인 소속</t>
+        </is>
+      </c>
+      <c r="G31" s="85" t="inlineStr">
+        <is>
+          <t>V4.9 파생 엣지(군집 결과, SiteClusterDetection 생성) — 원천 사실 아님</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1" s="54">
       <c r="A32" s="84" t="inlineStr">
         <is>
-          <t>E. Object 관계</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B32" s="85" t="inlineStr">
         <is>
-          <t>belongs_to_campaign</t>
+          <t>from_account</t>
         </is>
       </c>
       <c r="C32" s="85" t="inlineStr">
         <is>
-          <t>vt_site</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D32" s="85" t="inlineStr">
         <is>
-          <t>site_cluster</t>
+          <t>vt_transfer</t>
         </is>
       </c>
       <c r="E32" s="85" t="inlineStr">
         <is>
-          <t>sim_score, detected_at</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F32" s="86" t="inlineStr">
         <is>
-          <t>피싱 캠페인 소속</t>
-        </is>
-      </c>
-      <c r="G32" s="85" t="inlineStr">
-        <is>
-          <t>V4.9 파생 엣지(군집 결과, SiteClusterDetection 생성) — 원천 사실 아님</t>
-        </is>
-      </c>
+          <t>이체 출금 계좌</t>
+        </is>
+      </c>
+      <c r="G32" s="85" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1" s="54">
       <c r="A33" s="84" t="inlineStr">
@@ -3879,19 +3920,19 @@
       </c>
       <c r="B33" s="85" t="inlineStr">
         <is>
-          <t>from_account</t>
+          <t>to_account</t>
         </is>
       </c>
       <c r="C33" s="85" t="inlineStr">
         <is>
+          <t>vt_transfer</t>
+        </is>
+      </c>
+      <c r="D33" s="85" t="inlineStr">
+        <is>
           <t>vt_bacnt</t>
         </is>
       </c>
-      <c r="D33" s="85" t="inlineStr">
-        <is>
-          <t>vt_transfer</t>
-        </is>
-      </c>
       <c r="E33" s="85" t="inlineStr">
         <is>
           <t>-</t>
@@ -3899,7 +3940,7 @@
       </c>
       <c r="F33" s="86" t="inlineStr">
         <is>
-          <t>이체 출금 계좌</t>
+          <t>이체 입금 계좌</t>
         </is>
       </c>
       <c r="G33" s="85" t="n"/>
@@ -3912,17 +3953,17 @@
       </c>
       <c r="B34" s="85" t="inlineStr">
         <is>
-          <t>to_account</t>
+          <t>caller</t>
         </is>
       </c>
       <c r="C34" s="85" t="inlineStr">
         <is>
-          <t>vt_transfer</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="D34" s="85" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_call</t>
         </is>
       </c>
       <c r="E34" s="85" t="inlineStr">
@@ -3932,7 +3973,7 @@
       </c>
       <c r="F34" s="86" t="inlineStr">
         <is>
-          <t>이체 입금 계좌</t>
+          <t>발신 번호</t>
         </is>
       </c>
       <c r="G34" s="85" t="n"/>
@@ -3945,19 +3986,19 @@
       </c>
       <c r="B35" s="85" t="inlineStr">
         <is>
-          <t>caller</t>
+          <t>callee</t>
         </is>
       </c>
       <c r="C35" s="85" t="inlineStr">
         <is>
+          <t>vt_call</t>
+        </is>
+      </c>
+      <c r="D35" s="85" t="inlineStr">
+        <is>
           <t>vt_telno</t>
         </is>
       </c>
-      <c r="D35" s="85" t="inlineStr">
-        <is>
-          <t>vt_call</t>
-        </is>
-      </c>
       <c r="E35" s="85" t="inlineStr">
         <is>
           <t>-</t>
@@ -3965,7 +4006,7 @@
       </c>
       <c r="F35" s="86" t="inlineStr">
         <is>
-          <t>발신 번호</t>
+          <t>수신 번호</t>
         </is>
       </c>
       <c r="G35" s="85" t="n"/>
@@ -3978,30 +4019,34 @@
       </c>
       <c r="B36" s="85" t="inlineStr">
         <is>
-          <t>callee</t>
+          <t>contacted</t>
         </is>
       </c>
       <c r="C36" s="85" t="inlineStr">
         <is>
-          <t>vt_call</t>
+          <t>vt_telno|vt_id</t>
         </is>
       </c>
       <c r="D36" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>vt_telno|vt_id</t>
         </is>
       </c>
       <c r="E36" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>channel, first_dt, last_dt, call_count, msg_count, total_dur_sec, source_id</t>
         </is>
       </c>
       <c r="F36" s="86" t="inlineStr">
         <is>
-          <t>수신 번호</t>
-        </is>
-      </c>
-      <c r="G36" s="85" t="n"/>
+          <t>전화/메신저 계정 간 통화·연락 관계 (요약 엣지)</t>
+        </is>
+      </c>
+      <c r="G36" s="85" t="inlineStr">
+        <is>
+          <t>[V4.8 domain/range+DigitalID, channel 속성] · V4.9 (쌍,channel) 집계 속성 명시</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="54">
       <c r="A37" s="84" t="inlineStr">
@@ -4011,34 +4056,30 @@
       </c>
       <c r="B37" s="85" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>sent_msg</t>
         </is>
       </c>
       <c r="C37" s="85" t="inlineStr">
         <is>
-          <t>vt_telno|vt_id</t>
+          <t>vt_telno/vt_id</t>
         </is>
       </c>
       <c r="D37" s="85" t="inlineStr">
         <is>
-          <t>vt_telno|vt_id</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="E37" s="85" t="inlineStr">
         <is>
-          <t>channel, first_dt, last_dt, call_count, msg_count, total_dur_sec, source_id</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F37" s="86" t="inlineStr">
         <is>
-          <t>전화/메신저 계정 간 통화·연락 관계 (요약 엣지)</t>
-        </is>
-      </c>
-      <c r="G37" s="85" t="inlineStr">
-        <is>
-          <t>[V4.8 domain/range+DigitalID, channel 속성] · V4.9 (쌍,channel) 집계 속성 명시</t>
-        </is>
-      </c>
+          <t>메시지 발신</t>
+        </is>
+      </c>
+      <c r="G37" s="85" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1" s="54">
       <c r="A38" s="84" t="inlineStr">
@@ -4048,17 +4089,17 @@
       </c>
       <c r="B38" s="85" t="inlineStr">
         <is>
-          <t>sent_msg</t>
+          <t>received_msg</t>
         </is>
       </c>
       <c r="C38" s="85" t="inlineStr">
         <is>
-          <t>vt_telno/vt_id</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="D38" s="85" t="inlineStr">
         <is>
-          <t>vt_msg</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="E38" s="85" t="inlineStr">
@@ -4068,7 +4109,7 @@
       </c>
       <c r="F38" s="86" t="inlineStr">
         <is>
-          <t>메시지 발신</t>
+          <t>메시지 수신</t>
         </is>
       </c>
       <c r="G38" s="85" t="n"/>
@@ -4081,104 +4122,104 @@
       </c>
       <c r="B39" s="85" t="inlineStr">
         <is>
-          <t>received_msg</t>
+          <t>accessed_from</t>
         </is>
       </c>
       <c r="C39" s="85" t="inlineStr">
         <is>
-          <t>vt_msg</t>
+          <t>vt_access | vt_transfer | vt_msg</t>
         </is>
       </c>
       <c r="D39" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>vt_ip</t>
         </is>
       </c>
       <c r="E39" s="85" t="inlineStr">
         <is>
+          <t>source_id, rec_created</t>
+        </is>
+      </c>
+      <c r="F39" s="86" t="inlineStr">
+        <is>
+          <t>이벤트(접속·이체·메시지 발신)의 출발 IP — 이벤트 종류는 출발 라벨로 구분</t>
+        </is>
+      </c>
+      <c r="G39" s="85" t="inlineStr">
+        <is>
+          <t>V4.9 통합 (via_ip·sent_from_ip) — T2C 학습 표기 유지</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="54">
+      <c r="A40" s="90" t="inlineStr">
+        <is>
+          <t>F. Event 흐름</t>
+        </is>
+      </c>
+      <c r="B40" s="85" t="inlineStr">
+        <is>
+          <t>accessed_to</t>
+        </is>
+      </c>
+      <c r="C40" s="85" t="inlineStr">
+        <is>
+          <t>vt_access</t>
+        </is>
+      </c>
+      <c r="D40" s="85" t="inlineStr">
+        <is>
+          <t>vt_site / vt_bacnt / vt_id</t>
+        </is>
+      </c>
+      <c r="E40" s="85" t="inlineStr">
+        <is>
+          <t>target_type, source_id</t>
+        </is>
+      </c>
+      <c r="F40" s="86" t="inlineStr">
+        <is>
+          <t>접속 목적지 (웹사이트 · 인터넷뱅킹 대상 계좌 · 포털 계정)</t>
+        </is>
+      </c>
+      <c r="G40" s="85" t="inlineStr">
+        <is>
+          <t>V4.5 range 확장 (G8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="54">
+      <c r="A41" s="84" t="inlineStr">
+        <is>
+          <t>F. Event 흐름</t>
+        </is>
+      </c>
+      <c r="B41" s="85" t="inlineStr">
+        <is>
+          <t>recorded_in</t>
+        </is>
+      </c>
+      <c r="C41" s="85" t="inlineStr">
+        <is>
+          <t>vt_vhcl/vt_telno</t>
+        </is>
+      </c>
+      <c r="D41" s="85" t="inlineStr">
+        <is>
+          <t>vt_movement</t>
+        </is>
+      </c>
+      <c r="E41" s="85" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F39" s="86" t="inlineStr">
-        <is>
-          <t>메시지 수신</t>
-        </is>
-      </c>
-      <c r="G39" s="85" t="n"/>
-    </row>
-    <row r="40" ht="18" customHeight="1" s="54">
-      <c r="A40" s="84" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B40" s="85" t="inlineStr">
-        <is>
-          <t>accessed_from</t>
-        </is>
-      </c>
-      <c r="C40" s="85" t="inlineStr">
-        <is>
-          <t>vt_access | vt_transfer | vt_msg</t>
-        </is>
-      </c>
-      <c r="D40" s="85" t="inlineStr">
-        <is>
-          <t>vt_ip</t>
-        </is>
-      </c>
-      <c r="E40" s="85" t="inlineStr">
-        <is>
-          <t>source_id, rec_created</t>
-        </is>
-      </c>
-      <c r="F40" s="86" t="inlineStr">
-        <is>
-          <t>이벤트(접속·이체·메시지 발신)의 출발 IP — 이벤트 종류는 출발 라벨로 구분</t>
-        </is>
-      </c>
-      <c r="G40" s="85" t="inlineStr">
-        <is>
-          <t>V4.9 통합 (via_ip·sent_from_ip) — T2C 학습 표기 유지</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1" s="54">
-      <c r="A41" s="90" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B41" s="85" t="inlineStr">
-        <is>
-          <t>accessed_to</t>
-        </is>
-      </c>
-      <c r="C41" s="85" t="inlineStr">
-        <is>
-          <t>vt_access</t>
-        </is>
-      </c>
-      <c r="D41" s="85" t="inlineStr">
-        <is>
-          <t>vt_site / vt_bacnt / vt_id</t>
-        </is>
-      </c>
-      <c r="E41" s="85" t="inlineStr">
-        <is>
-          <t>target_type, source_id</t>
-        </is>
-      </c>
       <c r="F41" s="86" t="inlineStr">
         <is>
-          <t>접속 목적지 (웹사이트 · 인터넷뱅킹 대상 계좌 · 포털 계정)</t>
-        </is>
-      </c>
-      <c r="G41" s="85" t="inlineStr">
-        <is>
-          <t>V4.5 range 확장 (G8)</t>
-        </is>
-      </c>
+          <t>이동 기록의 주체</t>
+        </is>
+      </c>
+      <c r="G41" s="85" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1" s="54">
       <c r="A42" s="84" t="inlineStr">
@@ -4188,27 +4229,27 @@
       </c>
       <c r="B42" s="85" t="inlineStr">
         <is>
-          <t>recorded_in</t>
+          <t>used_in_device</t>
         </is>
       </c>
       <c r="C42" s="85" t="inlineStr">
         <is>
-          <t>vt_vhcl/vt_telno</t>
+          <t>vt_telno</t>
         </is>
       </c>
       <c r="D42" s="85" t="inlineStr">
         <is>
-          <t>vt_movement</t>
+          <t>vt_dev</t>
         </is>
       </c>
       <c r="E42" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>valid_from, valid_to, source_id</t>
         </is>
       </c>
       <c r="F42" s="86" t="inlineStr">
         <is>
-          <t>이동 기록의 주체</t>
+          <t>전화-기기(IMEI) 사용</t>
         </is>
       </c>
       <c r="G42" s="85" t="n"/>
@@ -4216,32 +4257,32 @@
     <row r="43" ht="18" customHeight="1" s="54">
       <c r="A43" s="84" t="inlineStr">
         <is>
-          <t>F. Event 흐름</t>
+          <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B43" s="85" t="inlineStr">
         <is>
-          <t>used_in_device</t>
+          <t>used_for</t>
         </is>
       </c>
       <c r="C43" s="85" t="inlineStr">
         <is>
-          <t>vt_telno</t>
+          <t>(object)</t>
         </is>
       </c>
       <c r="D43" s="85" t="inlineStr">
         <is>
-          <t>vt_dev</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="E43" s="85" t="inlineStr">
         <is>
-          <t>valid_from, valid_to, source_id</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F43" s="86" t="inlineStr">
         <is>
-          <t>전화-기기(IMEI) 사용</t>
+          <t>사칭에 사용된 객체</t>
         </is>
       </c>
       <c r="G43" s="85" t="n"/>
@@ -4254,17 +4295,17 @@
       </c>
       <c r="B44" s="85" t="inlineStr">
         <is>
-          <t>used_for</t>
+          <t>targets</t>
         </is>
       </c>
       <c r="C44" s="85" t="inlineStr">
         <is>
-          <t>(object)</t>
+          <t>vt_impersonation</t>
         </is>
       </c>
       <c r="D44" s="85" t="inlineStr">
         <is>
-          <t>vt_impersonation</t>
+          <t>vt_org</t>
         </is>
       </c>
       <c r="E44" s="85" t="inlineStr">
@@ -4274,189 +4315,193 @@
       </c>
       <c r="F44" s="86" t="inlineStr">
         <is>
-          <t>사칭에 사용된 객체</t>
+          <t>사칭 대상 기관</t>
         </is>
       </c>
       <c r="G44" s="85" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1" s="54">
-      <c r="A45" s="84" t="inlineStr">
+      <c r="A45" s="88" t="inlineStr">
         <is>
           <t>G. 사칭/접속주체</t>
         </is>
       </c>
       <c r="B45" s="85" t="inlineStr">
         <is>
-          <t>targets</t>
+          <t>performed_by</t>
         </is>
       </c>
       <c r="C45" s="85" t="inlineStr">
         <is>
-          <t>vt_impersonation</t>
+          <t>vt_access/vt_movement</t>
         </is>
       </c>
       <c r="D45" s="85" t="inlineStr">
         <is>
-          <t>vt_org</t>
+          <t>vt_psn / vt_telno / vt_id</t>
         </is>
       </c>
       <c r="E45" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>actor_type, resolved_to, resolved_at</t>
         </is>
       </c>
       <c r="F45" s="86" t="inlineStr">
         <is>
-          <t>사칭 대상 기관</t>
-        </is>
-      </c>
-      <c r="G45" s="85" t="n"/>
+          <t>접속·이동 수행 주체 (인물 미특정 단계에서는 번호·계정을 주체로 기록)</t>
+        </is>
+      </c>
+      <c r="G45" s="85" t="inlineStr">
+        <is>
+          <t>V4.4 range 확장 (G1)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1" s="54">
-      <c r="A46" s="88" t="inlineStr">
-        <is>
-          <t>G. 사칭/접속주체</t>
+      <c r="A46" s="84" t="inlineStr">
+        <is>
+          <t>H. Provenance</t>
         </is>
       </c>
       <c r="B46" s="85" t="inlineStr">
         <is>
-          <t>performed_by</t>
+          <t>sourced_from</t>
         </is>
       </c>
       <c r="C46" s="85" t="inlineStr">
         <is>
-          <t>vt_access/vt_movement</t>
+          <t>(any)</t>
         </is>
       </c>
       <c r="D46" s="85" t="inlineStr">
         <is>
-          <t>vt_psn / vt_telno / vt_id</t>
+          <t>vt_src</t>
         </is>
       </c>
       <c r="E46" s="85" t="inlineStr">
         <is>
-          <t>actor_type, resolved_to, resolved_at</t>
+          <t>src_tier, rec_created</t>
         </is>
       </c>
       <c r="F46" s="86" t="inlineStr">
         <is>
-          <t>접속·이동 수행 주체 (인물 미특정 단계에서는 번호·계정을 주체로 기록)</t>
+          <t>데이터 출처 참조</t>
         </is>
       </c>
       <c r="G46" s="85" t="inlineStr">
         <is>
-          <t>V4.4 range 확장 (G1)</t>
+          <t>tier1~3만 엣지 생성</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1" s="54">
-      <c r="A47" s="84" t="inlineStr">
-        <is>
-          <t>H. Provenance</t>
-        </is>
-      </c>
-      <c r="B47" s="85" t="inlineStr">
-        <is>
-          <t>sourced_from</t>
-        </is>
-      </c>
-      <c r="C47" s="85" t="inlineStr">
-        <is>
-          <t>(any)</t>
-        </is>
-      </c>
-      <c r="D47" s="85" t="inlineStr">
-        <is>
-          <t>vt_src</t>
-        </is>
-      </c>
-      <c r="E47" s="85" t="inlineStr">
-        <is>
-          <t>src_tier, rec_created</t>
-        </is>
-      </c>
-      <c r="F47" s="86" t="inlineStr">
-        <is>
-          <t>데이터 출처 참조</t>
-        </is>
-      </c>
-      <c r="G47" s="85" t="inlineStr">
-        <is>
-          <t>tier1~3만 엣지 생성</t>
+      <c r="A47" s="91" t="inlineStr">
+        <is>
+          <t>C. Person 관계</t>
+        </is>
+      </c>
+      <c r="B47" s="53" t="inlineStr">
+        <is>
+          <t>controls</t>
+        </is>
+      </c>
+      <c r="C47" s="53" t="inlineStr">
+        <is>
+          <t>vt_psn</t>
+        </is>
+      </c>
+      <c r="D47" s="53" t="inlineStr">
+        <is>
+          <t>vt_bacnt</t>
+        </is>
+      </c>
+      <c r="E47" s="53" t="inlineStr">
+        <is>
+          <t>confidence, inference_basis_type, evidence_edge_ids, evidence_count, evidence_summary</t>
+        </is>
+      </c>
+      <c r="F47" s="92" t="inlineStr">
+        <is>
+          <t>실질 지배(명의≠실사용)</t>
+        </is>
+      </c>
+      <c r="G47" s="92" t="inlineStr">
+        <is>
+          <t>정합화 등재 V4.4 근거 구조화 (G7)</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1" s="54">
-      <c r="A48" s="91" t="inlineStr">
-        <is>
-          <t>C. Person 관계</t>
+      <c r="A48" s="93" t="inlineStr">
+        <is>
+          <t>I. 위치</t>
         </is>
       </c>
       <c r="B48" s="53" t="inlineStr">
         <is>
-          <t>controls</t>
+          <t>located_at</t>
         </is>
       </c>
       <c r="C48" s="53" t="inlineStr">
         <is>
+          <t>vt_atm/vt_org · (event)</t>
+        </is>
+      </c>
+      <c r="D48" s="53" t="inlineStr">
+        <is>
+          <t>vt_loc</t>
+        </is>
+      </c>
+      <c r="E48" s="53" t="inlineStr">
+        <is>
+          <t>first_dt, last_dt, evt_count, source_id</t>
+        </is>
+      </c>
+      <c r="F48" s="92" t="inlineStr">
+        <is>
+          <t>객체의 위치 또는 이벤트의 발생 위치 — 출발 라벨로 구분</t>
+        </is>
+      </c>
+      <c r="G48" s="92" t="inlineStr">
+        <is>
+          <t>정합화 등재 · V4.9 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count · V4.9 occurred_at 통합</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="54">
+      <c r="A49" s="94" t="inlineStr">
+        <is>
+          <t>J. V4.3 시나리오</t>
+        </is>
+      </c>
+      <c r="B49" s="85" t="inlineStr">
+        <is>
+          <t>knows</t>
+        </is>
+      </c>
+      <c r="C49" s="85" t="inlineStr">
+        <is>
           <t>vt_psn</t>
         </is>
       </c>
-      <c r="D48" s="53" t="inlineStr">
-        <is>
-          <t>vt_bacnt</t>
-        </is>
-      </c>
-      <c r="E48" s="53" t="inlineStr">
-        <is>
-          <t>confidence, inference_basis_type, evidence_edge_ids, evidence_count, evidence_summary</t>
-        </is>
-      </c>
-      <c r="F48" s="92" t="inlineStr">
-        <is>
-          <t>실질 지배(명의≠실사용)</t>
-        </is>
-      </c>
-      <c r="G48" s="92" t="inlineStr">
-        <is>
-          <t>정합화 등재 V4.4 근거 구조화 (G7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1" s="54">
-      <c r="A49" s="93" t="inlineStr">
-        <is>
-          <t>I. 위치</t>
-        </is>
-      </c>
-      <c r="B49" s="53" t="inlineStr">
-        <is>
-          <t>located_at</t>
-        </is>
-      </c>
-      <c r="C49" s="53" t="inlineStr">
-        <is>
-          <t>vt_atm/vt_org · (event)</t>
-        </is>
-      </c>
-      <c r="D49" s="53" t="inlineStr">
-        <is>
-          <t>vt_loc</t>
-        </is>
-      </c>
-      <c r="E49" s="53" t="inlineStr">
-        <is>
-          <t>first_dt, last_dt, evt_count, source_id</t>
-        </is>
-      </c>
-      <c r="F49" s="92" t="inlineStr">
-        <is>
-          <t>객체의 위치 또는 이벤트의 발생 위치 — 출발 라벨로 구분</t>
-        </is>
-      </c>
-      <c r="G49" s="92" t="inlineStr">
-        <is>
-          <t>정합화 등재 · V4.9 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count · V4.9 occurred_at 통합</t>
+      <c r="D49" s="85" t="inlineStr">
+        <is>
+          <t>vt_psn</t>
+        </is>
+      </c>
+      <c r="E49" s="85" t="inlineStr">
+        <is>
+          <t>relation_type, confidence, valid_from</t>
+        </is>
+      </c>
+      <c r="F49" s="86" t="inlineStr">
+        <is>
+          <t>두 인물의 사회적 지인 관계 (고향친구/동창 — 공범 여부는 그래프 엣지가 아니라 탐지 결과로 판단)</t>
+        </is>
+      </c>
+      <c r="G49" s="85" t="inlineStr">
+        <is>
+          <t>V4.3 신규</t>
         </is>
       </c>
     </row>
@@ -4468,106 +4513,106 @@
       </c>
       <c r="B50" s="85" t="inlineStr">
         <is>
-          <t>knows</t>
+          <t>mentions</t>
         </is>
       </c>
       <c r="C50" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_msg</t>
         </is>
       </c>
       <c r="D50" s="85" t="inlineStr">
         <is>
-          <t>vt_psn</t>
+          <t>vt_id | vt_bacnt | vt_loc</t>
         </is>
       </c>
       <c r="E50" s="85" t="inlineStr">
         <is>
-          <t>relation_type, confidence, valid_from</t>
+          <t>confidence, extract_method, source_id, rec_created</t>
         </is>
       </c>
       <c r="F50" s="86" t="inlineStr">
         <is>
-          <t>두 인물의 사회적 지인 관계 (고향친구/동창 — 공범 여부는 그래프 엣지가 아니라 탐지 결과로 판단)</t>
+          <t>메시지·게시물 본문에 계정·계좌·장소가 기재됨 — 종류는 도착 라벨로 구분</t>
         </is>
       </c>
       <c r="G50" s="85" t="inlineStr">
         <is>
-          <t>V4.3 신규</t>
+          <t>V4.9 통합 (mentions_id·mentions_account·mentions_location)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1" s="54">
-      <c r="A51" s="94" t="inlineStr">
-        <is>
-          <t>J. V4.3 시나리오</t>
-        </is>
-      </c>
-      <c r="B51" s="85" t="inlineStr">
-        <is>
-          <t>mentions</t>
-        </is>
-      </c>
-      <c r="C51" s="85" t="inlineStr">
-        <is>
-          <t>vt_msg</t>
-        </is>
-      </c>
-      <c r="D51" s="85" t="inlineStr">
-        <is>
-          <t>vt_id | vt_bacnt | vt_loc</t>
-        </is>
-      </c>
-      <c r="E51" s="85" t="inlineStr">
-        <is>
-          <t>confidence, extract_method, source_id, rec_created</t>
-        </is>
-      </c>
-      <c r="F51" s="86" t="inlineStr">
-        <is>
-          <t>메시지·게시물 본문에 계정·계좌·장소가 기재됨 — 종류는 도착 라벨로 구분</t>
-        </is>
-      </c>
-      <c r="G51" s="85" t="inlineStr">
-        <is>
-          <t>V4.9 통합 (mentions_id·mentions_account·mentions_location)</t>
+      <c r="A51" s="98" t="inlineStr">
+        <is>
+          <t>B. Case→Object 증거</t>
+        </is>
+      </c>
+      <c r="B51" s="99" t="inlineStr">
+        <is>
+          <t>eg_used_id</t>
+        </is>
+      </c>
+      <c r="C51" s="99" t="inlineStr">
+        <is>
+          <t>vt_case</t>
+        </is>
+      </c>
+      <c r="D51" s="99" t="inlineStr">
+        <is>
+          <t>vt_id</t>
+        </is>
+      </c>
+      <c r="E51" s="99" t="inlineStr">
+        <is>
+          <t>source_id, rec_created, valid_from, valid_to</t>
+        </is>
+      </c>
+      <c r="F51" s="100" t="inlineStr">
+        <is>
+          <t>사용 온라인 계정 증거 (네이버·카카오·구글 ID)</t>
+        </is>
+      </c>
+      <c r="G51" s="99" t="inlineStr">
+        <is>
+          <t>V4.4 신규 (R3)</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="54">
       <c r="A52" s="98" t="inlineStr">
         <is>
-          <t>B. Case→Object 증거</t>
+          <t>F. Event 흐름</t>
         </is>
       </c>
       <c r="B52" s="99" t="inlineStr">
         <is>
-          <t>eg_used_id</t>
+          <t>exchanged_to</t>
         </is>
       </c>
       <c r="C52" s="99" t="inlineStr">
         <is>
-          <t>vt_case</t>
+          <t>vt_bacnt</t>
         </is>
       </c>
       <c r="D52" s="99" t="inlineStr">
         <is>
-          <t>vt_id</t>
+          <t>vt_crypto</t>
         </is>
       </c>
       <c r="E52" s="99" t="inlineStr">
         <is>
-          <t>source_id, rec_created, valid_from, valid_to</t>
+          <t>exchange_nm, dlng_dt, fiat_amt, asset_amt, confidence, inference</t>
         </is>
       </c>
       <c r="F52" s="100" t="inlineStr">
         <is>
-          <t>사용 온라인 계정 증거 (네이버·카카오·구글 ID)</t>
+          <t>원화 계좌 → 가상자산 전환 (자금추적 종단 브리지)</t>
         </is>
       </c>
       <c r="G52" s="99" t="inlineStr">
         <is>
-          <t>V4.4 신규 (R3)</t>
+          <t>V4.4 신규 (G6)</t>
         </is>
       </c>
     </row>
@@ -4579,72 +4624,36 @@
       </c>
       <c r="B53" s="99" t="inlineStr">
         <is>
-          <t>exchanged_to</t>
+          <t>access_via</t>
         </is>
       </c>
       <c r="C53" s="99" t="inlineStr">
         <is>
-          <t>vt_bacnt</t>
+          <t>vt_access</t>
         </is>
       </c>
       <c r="D53" s="99" t="inlineStr">
         <is>
-          <t>vt_crypto</t>
+          <t>vt_telno / vt_id / vt_bacnt</t>
         </is>
       </c>
       <c r="E53" s="99" t="inlineStr">
         <is>
-          <t>exchange_nm, dlng_dt, fiat_amt, asset_amt, confidence, inference</t>
+          <t>valid_from, confidence, verified</t>
         </is>
       </c>
       <c r="F53" s="100" t="inlineStr">
         <is>
-          <t>원화 계좌 → 가상자산 전환 (자금추적 종단 브리지)</t>
+          <t>접속 이벤트가 경유·사용한 수단(전화/디지털ID/계좌) 연결</t>
         </is>
       </c>
       <c r="G53" s="99" t="inlineStr">
         <is>
-          <t>V4.4 신규 (G6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1" s="54">
-      <c r="A54" s="98" t="inlineStr">
-        <is>
-          <t>F. Event 흐름</t>
-        </is>
-      </c>
-      <c r="B54" s="99" t="inlineStr">
-        <is>
-          <t>access_via</t>
-        </is>
-      </c>
-      <c r="C54" s="99" t="inlineStr">
-        <is>
-          <t>vt_access</t>
-        </is>
-      </c>
-      <c r="D54" s="99" t="inlineStr">
-        <is>
-          <t>vt_telno / vt_id / vt_bacnt</t>
-        </is>
-      </c>
-      <c r="E54" s="99" t="inlineStr">
-        <is>
-          <t>valid_from, confidence, verified</t>
-        </is>
-      </c>
-      <c r="F54" s="100" t="inlineStr">
-        <is>
-          <t>접속 이벤트가 경유·사용한 수단(전화/디지털ID/계좌) 연결</t>
-        </is>
-      </c>
-      <c r="G54" s="99" t="inlineStr">
-        <is>
           <t>V4.5 (access 다형화)</t>
         </is>
       </c>
     </row>
+    <row r="54" ht="18" customHeight="1" s="54"/>
     <row r="55" ht="18" customHeight="1" s="54"/>
     <row r="56" ht="36" customHeight="1" s="54"/>
     <row r="57" ht="18" customHeight="1" s="54"/>
@@ -12682,7 +12691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="53" min="1" max="1"/>
@@ -13059,7 +13068,7 @@
       </c>
       <c r="D14" s="85" t="inlineStr">
         <is>
-          <t>hosts, contains_file</t>
+          <t>contains_file, resolves_to(구 hosts)</t>
         </is>
       </c>
       <c r="E14" s="92" t="inlineStr">
@@ -13098,22 +13107,22 @@
     <row r="16" ht="18" customHeight="1" s="54">
       <c r="A16" s="85" t="inlineStr">
         <is>
-          <t>src_tier</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="B16" s="85" t="inlineStr">
         <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C16" s="86" t="inlineStr">
-        <is>
-          <t>출처 신뢰등급(1~5)</t>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C16" s="85" t="inlineStr">
+        <is>
+          <t>연결 근거 — 'dns'(DNS 조회 관측, 미기재 시 기본) · 'origin'(원본 서버 확인: 호스팅사 회신·압수)</t>
         </is>
       </c>
       <c r="D16" s="85" t="inlineStr">
         <is>
-          <t>sourced_from</t>
+          <t>resolves_to</t>
         </is>
       </c>
       <c r="E16" s="92" t="inlineStr">
@@ -13125,22 +13134,22 @@
     <row r="17" ht="18" customHeight="1" s="54">
       <c r="A17" s="85" t="inlineStr">
         <is>
-          <t>link_type / link_reason</t>
+          <t>src_tier</t>
         </is>
       </c>
       <c r="B17" s="85" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C17" s="86" t="inlineStr">
         <is>
-          <t>연결 유형 / 사유</t>
+          <t>출처 신뢰등급(1~5)</t>
         </is>
       </c>
       <c r="D17" s="85" t="inlineStr">
         <is>
-          <t>linked_to</t>
+          <t>sourced_from</t>
         </is>
       </c>
       <c r="E17" s="92" t="inlineStr">
@@ -13152,7 +13161,7 @@
     <row r="18" ht="18" customHeight="1" s="54">
       <c r="A18" s="85" t="inlineStr">
         <is>
-          <t>first_seen / last_seen</t>
+          <t>link_type / link_reason</t>
         </is>
       </c>
       <c r="B18" s="85" t="inlineStr">
@@ -13162,24 +13171,24 @@
       </c>
       <c r="C18" s="86" t="inlineStr">
         <is>
-          <t>최초/최종 관측 시각</t>
+          <t>연결 유형 / 사유</t>
         </is>
       </c>
       <c r="D18" s="85" t="inlineStr">
         <is>
-          <t>used_in_device</t>
+          <t>linked_to</t>
         </is>
       </c>
       <c r="E18" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="54">
       <c r="A19" s="85" t="inlineStr">
         <is>
-          <t>converted_dt / converted_by</t>
+          <t>first_seen / last_seen</t>
         </is>
       </c>
       <c r="B19" s="85" t="inlineStr">
@@ -13189,12 +13198,12 @@
       </c>
       <c r="C19" s="86" t="inlineStr">
         <is>
-          <t>사건 전환 시각 / 주체</t>
+          <t>최초/최종 관측 시각</t>
         </is>
       </c>
       <c r="D19" s="85" t="inlineStr">
         <is>
-          <t>filed_as</t>
+          <t>used_in_device</t>
         </is>
       </c>
       <c r="E19" s="92" t="inlineStr">
@@ -13206,61 +13215,61 @@
     <row r="20" ht="18" customHeight="1" s="54">
       <c r="A20" s="85" t="inlineStr">
         <is>
-          <t>damage_amount</t>
+          <t>converted_dt / converted_by</t>
         </is>
       </c>
       <c r="B20" s="85" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C20" s="86" t="inlineStr">
         <is>
-          <t>피해금액(원)</t>
+          <t>사건 전환 시각 / 주체</t>
         </is>
       </c>
       <c r="D20" s="85" t="inlineStr">
         <is>
-          <t>victim_in</t>
+          <t>filed_as</t>
         </is>
       </c>
       <c r="E20" s="92" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="54">
       <c r="A21" s="85" t="inlineStr">
         <is>
-          <t>statement_date</t>
+          <t>damage_amount</t>
         </is>
       </c>
       <c r="B21" s="85" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C21" s="86" t="inlineStr">
         <is>
-          <t>참고인 진술일</t>
+          <t>피해금액(원)</t>
         </is>
       </c>
       <c r="D21" s="85" t="inlineStr">
         <is>
-          <t>witness_in</t>
+          <t>victim_in</t>
         </is>
       </c>
       <c r="E21" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="54">
       <c r="A22" s="85" t="inlineStr">
         <is>
-          <t>recruit_type / payment</t>
+          <t>statement_date</t>
         </is>
       </c>
       <c r="B22" s="85" t="inlineStr">
@@ -13270,24 +13279,24 @@
       </c>
       <c r="C22" s="86" t="inlineStr">
         <is>
-          <t>모집 유형 / 대가</t>
+          <t>참고인 진술일</t>
         </is>
       </c>
       <c r="D22" s="85" t="inlineStr">
         <is>
-          <t>recruits</t>
+          <t>witness_in</t>
         </is>
       </c>
       <c r="E22" s="92" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="54">
       <c r="A23" s="85" t="inlineStr">
         <is>
-          <t>method / date</t>
+          <t>recruit_type / payment</t>
         </is>
       </c>
       <c r="B23" s="85" t="inlineStr">
@@ -13297,24 +13306,24 @@
       </c>
       <c r="C23" s="86" t="inlineStr">
         <is>
-          <t>협박 방법 / 일자</t>
+          <t>모집 유형 / 대가</t>
         </is>
       </c>
       <c r="D23" s="85" t="inlineStr">
         <is>
-          <t>blackmails</t>
+          <t>recruits</t>
         </is>
       </c>
       <c r="E23" s="92" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="54">
       <c r="A24" s="85" t="inlineStr">
         <is>
-          <t>file_role</t>
+          <t>method / date</t>
         </is>
       </c>
       <c r="B24" s="85" t="inlineStr">
@@ -13324,12 +13333,12 @@
       </c>
       <c r="C24" s="86" t="inlineStr">
         <is>
-          <t>파일의 역할(첨부/배포/증거)</t>
+          <t>협박 방법 / 일자</t>
         </is>
       </c>
       <c r="D24" s="85" t="inlineStr">
         <is>
-          <t>contains_file</t>
+          <t>blackmails</t>
         </is>
       </c>
       <c r="E24" s="92" t="inlineStr">
@@ -13341,61 +13350,61 @@
     <row r="25" ht="18" customHeight="1" s="54">
       <c r="A25" s="85" t="inlineStr">
         <is>
-          <t>usage_count</t>
+          <t>file_role</t>
         </is>
       </c>
       <c r="B25" s="85" t="inlineStr">
         <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C25" s="85" t="inlineStr">
-        <is>
-          <t>IP 사용(접속) 행 수 — (주체,IP)쌍 집계 시 합계 (V4.9)</t>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C25" s="86" t="inlineStr">
+        <is>
+          <t>파일의 역할(첨부/배포/증거)</t>
         </is>
       </c>
       <c r="D25" s="85" t="inlineStr">
         <is>
-          <t>used_ip</t>
+          <t>contains_file</t>
         </is>
       </c>
       <c r="E25" s="92" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="54">
       <c r="A26" s="85" t="inlineStr">
         <is>
-          <t>verified_dt</t>
+          <t>usage_count</t>
         </is>
       </c>
       <c r="B26" s="85" t="inlineStr">
         <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C26" s="86" t="inlineStr">
-        <is>
-          <t>검증 시각</t>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C26" s="85" t="inlineStr">
+        <is>
+          <t>IP 사용(접속) 행 수 — (주체,IP)쌍 집계 시 합계 (V4.9)</t>
         </is>
       </c>
       <c r="D26" s="85" t="inlineStr">
         <is>
-          <t>verified_by</t>
+          <t>used_ip</t>
         </is>
       </c>
       <c r="E26" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="54">
       <c r="A27" s="85" t="inlineStr">
         <is>
-          <t>relation_type</t>
+          <t>verified_dt</t>
         </is>
       </c>
       <c r="B27" s="85" t="inlineStr">
@@ -13405,69 +13414,69 @@
       </c>
       <c r="C27" s="86" t="inlineStr">
         <is>
-          <t>지인 관계 유형(친구/동창/가족 등)</t>
+          <t>검증 시각</t>
         </is>
       </c>
       <c r="D27" s="85" t="inlineStr">
         <is>
-          <t>knows</t>
-        </is>
-      </c>
-      <c r="E27" s="86" t="inlineStr">
-        <is>
-          <t>범주형</t>
+          <t>verified_by</t>
+        </is>
+      </c>
+      <c r="E27" s="92" t="inlineStr">
+        <is>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="54">
       <c r="A28" s="85" t="inlineStr">
         <is>
+          <t>relation_type</t>
+        </is>
+      </c>
+      <c r="B28" s="85" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C28" s="86" t="inlineStr">
+        <is>
+          <t>지인 관계 유형(친구/동창/가족 등)</t>
+        </is>
+      </c>
+      <c r="D28" s="85" t="inlineStr">
+        <is>
+          <t>knows</t>
+        </is>
+      </c>
+      <c r="E28" s="86" t="inlineStr">
+        <is>
+          <t>범주형</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="54">
+      <c r="A29" s="85" t="inlineStr">
+        <is>
           <t>link_basis</t>
         </is>
       </c>
-      <c r="B28" s="85" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C28" s="86" t="inlineStr">
+      <c r="B29" s="85" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C29" s="86" t="inlineStr">
         <is>
           <t>식별자 연결 근거(인증서발급/포털역조회 등)</t>
         </is>
       </c>
-      <c r="D28" s="85" t="inlineStr">
+      <c r="D29" s="85" t="inlineStr">
         <is>
           <t>linked_to(구 linked_id)</t>
         </is>
       </c>
-      <c r="E28" s="86" t="inlineStr">
-        <is>
-          <t>범주형</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1" s="54">
-      <c r="A29" s="98" t="inlineStr">
-        <is>
-          <t>actor_type</t>
-        </is>
-      </c>
-      <c r="B29" s="99" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C29" s="100" t="inlineStr">
-        <is>
-          <t>이벤트 행위 주체의 유형 (person | telno | online_id)</t>
-        </is>
-      </c>
-      <c r="D29" s="99" t="inlineStr">
-        <is>
-          <t>performed_by</t>
-        </is>
-      </c>
-      <c r="E29" s="100" t="inlineStr">
+      <c r="E29" s="86" t="inlineStr">
         <is>
           <t>범주형</t>
         </is>
@@ -13476,7 +13485,7 @@
     <row r="30" ht="18" customHeight="1" s="54">
       <c r="A30" s="98" t="inlineStr">
         <is>
-          <t>resolved_to</t>
+          <t>actor_type</t>
         </is>
       </c>
       <c r="B30" s="99" t="inlineStr">
@@ -13486,7 +13495,7 @@
       </c>
       <c r="C30" s="100" t="inlineStr">
         <is>
-          <t>후속 특정된 vt_psn.psn_id (미특정 시 null)</t>
+          <t>이벤트 행위 주체의 유형 (person | telno | online_id)</t>
         </is>
       </c>
       <c r="D30" s="99" t="inlineStr">
@@ -13496,14 +13505,14 @@
       </c>
       <c r="E30" s="100" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" s="54">
       <c r="A31" s="98" t="inlineStr">
         <is>
-          <t>resolved_at</t>
+          <t>resolved_to</t>
         </is>
       </c>
       <c r="B31" s="99" t="inlineStr">
@@ -13513,7 +13522,7 @@
       </c>
       <c r="C31" s="100" t="inlineStr">
         <is>
-          <t>주체가 인물로 특정된 시각(ISO8601)</t>
+          <t>후속 특정된 vt_psn.psn_id (미특정 시 null)</t>
         </is>
       </c>
       <c r="D31" s="99" t="inlineStr">
@@ -13523,14 +13532,14 @@
       </c>
       <c r="E31" s="100" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="54">
       <c r="A32" s="98" t="inlineStr">
         <is>
-          <t>subject_type</t>
+          <t>resolved_at</t>
         </is>
       </c>
       <c r="B32" s="99" t="inlineStr">
@@ -13540,78 +13549,78 @@
       </c>
       <c r="C32" s="100" t="inlineStr">
         <is>
-          <t>관계 주체의 유형 (person | telno | online_id)</t>
+          <t>주체가 인물로 특정된 시각(ISO8601)</t>
         </is>
       </c>
       <c r="D32" s="99" t="inlineStr">
         <is>
-          <t>used_ip</t>
+          <t>performed_by</t>
         </is>
       </c>
       <c r="E32" s="100" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" s="54">
       <c r="A33" s="98" t="inlineStr">
         <is>
-          <t>duration_days</t>
+          <t>subject_type</t>
         </is>
       </c>
       <c r="B33" s="99" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C33" s="100" t="inlineStr">
         <is>
-          <t>관계 유효 기간(일) = valid_to - valid_from. 파생값</t>
+          <t>관계 주체의 유형 (person | telno | online_id)</t>
         </is>
       </c>
       <c r="D33" s="99" t="inlineStr">
         <is>
-          <t>registered_to, eg_used_* 3종</t>
+          <t>used_ip</t>
         </is>
       </c>
       <c r="E33" s="100" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1" s="54">
       <c r="A34" s="98" t="inlineStr">
         <is>
-          <t>inference_basis_type</t>
+          <t>duration_days</t>
         </is>
       </c>
       <c r="B34" s="99" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C34" s="100" t="inlineStr">
         <is>
-          <t>추론 근거 유형 배열 — 값도메인 시트 참조. 복수 근거 지원</t>
+          <t>관계 유효 기간(일) = valid_to - valid_from. 파생값</t>
         </is>
       </c>
       <c r="D34" s="99" t="inlineStr">
         <is>
-          <t>controls, mentions_account</t>
+          <t>registered_to, eg_used_* 3종</t>
         </is>
       </c>
       <c r="E34" s="100" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1" s="54">
       <c r="A35" s="98" t="inlineStr">
         <is>
-          <t>match_basis_type</t>
+          <t>inference_basis_type</t>
         </is>
       </c>
       <c r="B35" s="99" t="inlineStr">
@@ -13621,12 +13630,12 @@
       </c>
       <c r="C35" s="100" t="inlineStr">
         <is>
-          <t>[V4.9 폐지 → match_basis] 동일성 판단 근거 유형 배열 — 값도메인 시트 참조</t>
+          <t>추론 근거 유형 배열 — 값도메인 시트 참조. 복수 근거 지원</t>
         </is>
       </c>
       <c r="D35" s="99" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>controls, mentions_account</t>
         </is>
       </c>
       <c r="E35" s="100" t="inlineStr">
@@ -13638,7 +13647,7 @@
     <row r="36" ht="30" customHeight="1" s="54">
       <c r="A36" s="98" t="inlineStr">
         <is>
-          <t>evidence_edge_ids</t>
+          <t>match_basis_type</t>
         </is>
       </c>
       <c r="B36" s="99" t="inlineStr">
@@ -13648,34 +13657,34 @@
       </c>
       <c r="C36" s="100" t="inlineStr">
         <is>
-          <t>근거가 된 원천 엣지 ID 배열 (법정 재현용 · 소급 복원 불가)</t>
-        </is>
-      </c>
-      <c r="D36" s="100" t="inlineStr">
-        <is>
-          <t>추론 엣지 6종</t>
+          <t>[V4.9 폐지 → match_basis] 동일성 판단 근거 유형 배열 — 값도메인 시트 참조</t>
+        </is>
+      </c>
+      <c r="D36" s="99" t="inlineStr">
+        <is>
+          <t>sameAs</t>
         </is>
       </c>
       <c r="E36" s="100" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1" s="54">
       <c r="A37" s="98" t="inlineStr">
         <is>
-          <t>evidence_count</t>
+          <t>evidence_edge_ids</t>
         </is>
       </c>
       <c r="B37" s="99" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>list</t>
         </is>
       </c>
       <c r="C37" s="100" t="inlineStr">
         <is>
-          <t>근거 건수 (예: 공유 IP에서의 접속 레코드 수)</t>
+          <t>근거가 된 원천 엣지 ID 배열 (법정 재현용 · 소급 복원 불가)</t>
         </is>
       </c>
       <c r="D37" s="100" t="inlineStr">
@@ -13685,24 +13694,24 @@
       </c>
       <c r="E37" s="100" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1" s="54">
       <c r="A38" s="98" t="inlineStr">
         <is>
-          <t>evidence_summary</t>
+          <t>evidence_count</t>
         </is>
       </c>
       <c r="B38" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C38" s="100" t="inlineStr">
         <is>
-          <t>사람이 읽는 근거 요약 (구 inference_basis / match_basis 역할)</t>
+          <t>근거 건수 (예: 공유 IP에서의 접속 레코드 수)</t>
         </is>
       </c>
       <c r="D38" s="100" t="inlineStr">
@@ -13712,14 +13721,14 @@
       </c>
       <c r="E38" s="100" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1" s="54">
       <c r="A39" s="98" t="inlineStr">
         <is>
-          <t>warrant_no</t>
+          <t>evidence_summary</t>
         </is>
       </c>
       <c r="B39" s="99" t="inlineStr">
@@ -13729,24 +13738,24 @@
       </c>
       <c r="C39" s="100" t="inlineStr">
         <is>
-          <t>근거 영장·허가서 번호</t>
-        </is>
-      </c>
-      <c r="D39" s="99" t="inlineStr">
-        <is>
-          <t>linked_to(구 linked_id), eg_used_* 4종</t>
+          <t>사람이 읽는 근거 요약 (구 inference_basis / match_basis 역할)</t>
+        </is>
+      </c>
+      <c r="D39" s="100" t="inlineStr">
+        <is>
+          <t>추론 엣지 6종</t>
         </is>
       </c>
       <c r="E39" s="100" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1" s="54">
       <c r="A40" s="98" t="inlineStr">
         <is>
-          <t>exchange_nm</t>
+          <t>warrant_no</t>
         </is>
       </c>
       <c r="B40" s="99" t="inlineStr">
@@ -13756,34 +13765,34 @@
       </c>
       <c r="C40" s="100" t="inlineStr">
         <is>
-          <t>가상자산 거래소명</t>
+          <t>근거 영장·허가서 번호</t>
         </is>
       </c>
       <c r="D40" s="99" t="inlineStr">
         <is>
-          <t>exchanged_to</t>
+          <t>linked_to(구 linked_id), eg_used_* 4종</t>
         </is>
       </c>
       <c r="E40" s="100" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1" s="54">
       <c r="A41" s="98" t="inlineStr">
         <is>
-          <t>fiat_amt</t>
+          <t>exchange_nm</t>
         </is>
       </c>
       <c r="B41" s="99" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C41" s="100" t="inlineStr">
         <is>
-          <t>전환 원화 금액(원)</t>
+          <t>가상자산 거래소명</t>
         </is>
       </c>
       <c r="D41" s="99" t="inlineStr">
@@ -13793,24 +13802,24 @@
       </c>
       <c r="E41" s="100" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" s="54">
       <c r="A42" s="98" t="inlineStr">
         <is>
-          <t>asset_amt</t>
+          <t>fiat_amt</t>
         </is>
       </c>
       <c r="B42" s="99" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C42" s="100" t="inlineStr">
         <is>
-          <t>전환 가상자산 수량</t>
+          <t>전환 원화 금액(원)</t>
         </is>
       </c>
       <c r="D42" s="99" t="inlineStr">
@@ -13827,61 +13836,61 @@
     <row r="43" ht="30" customHeight="1" s="54">
       <c r="A43" s="98" t="inlineStr">
         <is>
+          <t>asset_amt</t>
+        </is>
+      </c>
+      <c r="B43" s="99" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C43" s="100" t="inlineStr">
+        <is>
+          <t>전환 가상자산 수량</t>
+        </is>
+      </c>
+      <c r="D43" s="99" t="inlineStr">
+        <is>
+          <t>exchanged_to</t>
+        </is>
+      </c>
+      <c r="E43" s="100" t="inlineStr">
+        <is>
+          <t>수치형</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1" s="54">
+      <c r="A44" s="98" t="inlineStr">
+        <is>
           <t>link_reason</t>
         </is>
       </c>
-      <c r="B43" s="99" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C43" s="100" t="inlineStr">
+      <c r="B44" s="99" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C44" s="100" t="inlineStr">
         <is>
           <t>진정서-사건 연결 사유</t>
         </is>
       </c>
-      <c r="D43" s="99" t="inlineStr">
+      <c r="D44" s="99" t="inlineStr">
         <is>
           <t>linked_petition</t>
         </is>
       </c>
-      <c r="E43" s="100" t="inlineStr">
+      <c r="E44" s="100" t="inlineStr">
         <is>
           <t>텍스트</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1" s="54">
-      <c r="A44" s="106" t="inlineStr">
-        <is>
-          <t>traversal_policy</t>
-        </is>
-      </c>
-      <c r="B44" s="99" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C44" s="107" t="inlineStr">
-        <is>
-          <t>탐색 시 이 엣지를 따라갈지 결정 (follow | candidate_only | block). review_status 와 연동</t>
-        </is>
-      </c>
-      <c r="D44" s="99" t="inlineStr">
-        <is>
-          <t>same_as</t>
-        </is>
-      </c>
-      <c r="E44" s="107" t="inlineStr">
-        <is>
-          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1" s="54">
       <c r="A45" s="106" t="inlineStr">
         <is>
-          <t>edge_id</t>
+          <t>traversal_policy</t>
         </is>
       </c>
       <c r="B45" s="99" t="inlineStr">
@@ -13891,24 +13900,24 @@
       </c>
       <c r="C45" s="107" t="inlineStr">
         <is>
-          <t>엣지의 안정적 고유 식별자 — evidence_edge_ids 가 참조. 재적재 시에도 불변이어야 함</t>
-        </is>
-      </c>
-      <c r="D45" s="107" t="inlineStr">
-        <is>
-          <t>전 엣지 공통</t>
+          <t>탐색 시 이 엣지를 따라갈지 결정 (follow | candidate_only | block). review_status 와 연동</t>
+        </is>
+      </c>
+      <c r="D45" s="99" t="inlineStr">
+        <is>
+          <t>same_as</t>
         </is>
       </c>
       <c r="E45" s="107" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1" s="54">
       <c r="A46" s="106" t="inlineStr">
         <is>
-          <t>target_type</t>
+          <t>edge_id</t>
         </is>
       </c>
       <c r="B46" s="99" t="inlineStr">
@@ -13918,24 +13927,24 @@
       </c>
       <c r="C46" s="107" t="inlineStr">
         <is>
-          <t>접속 목적지 유형 (site | account | online_id)</t>
-        </is>
-      </c>
-      <c r="D46" s="99" t="inlineStr">
-        <is>
-          <t>accessed_to</t>
+          <t>엣지의 안정적 고유 식별자 — evidence_edge_ids 가 참조. 재적재 시에도 불변이어야 함</t>
+        </is>
+      </c>
+      <c r="D46" s="107" t="inlineStr">
+        <is>
+          <t>전 엣지 공통</t>
         </is>
       </c>
       <c r="E46" s="107" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1" s="54">
       <c r="A47" s="106" t="inlineStr">
         <is>
-          <t>direction</t>
+          <t>target_type</t>
         </is>
       </c>
       <c r="B47" s="99" t="inlineStr">
@@ -13945,12 +13954,12 @@
       </c>
       <c r="C47" s="107" t="inlineStr">
         <is>
-          <t>탐색 방향성 (directed | undirected). undirected 선언 시 역방향 인덱스 필수</t>
+          <t>접속 목적지 유형 (site | account | online_id)</t>
         </is>
       </c>
       <c r="D47" s="99" t="inlineStr">
         <is>
-          <t>used_ip, contacted, communicated_with</t>
+          <t>accessed_to</t>
         </is>
       </c>
       <c r="E47" s="107" t="inlineStr">
@@ -13962,7 +13971,7 @@
     <row r="48" ht="30" customHeight="1" s="54">
       <c r="A48" s="106" t="inlineStr">
         <is>
-          <t>valid_from</t>
+          <t>direction</t>
         </is>
       </c>
       <c r="B48" s="99" t="inlineStr">
@@ -13972,24 +13981,24 @@
       </c>
       <c r="C48" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 관계 현실 유효 시작(ISO8601, bitemporal)</t>
+          <t>탐색 방향성 (directed | undirected). undirected 선언 시 역방향 인덱스 필수</t>
         </is>
       </c>
       <c r="D48" s="99" t="inlineStr">
         <is>
-          <t>used_ip, eg_used_account, eg_used_phone, registered_to, has_account 등</t>
+          <t>used_ip, contacted, communicated_with</t>
         </is>
       </c>
       <c r="E48" s="107" t="inlineStr">
         <is>
-          <t>시각</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1" s="54">
       <c r="A49" s="106" t="inlineStr">
         <is>
-          <t>valid_to</t>
+          <t>valid_from</t>
         </is>
       </c>
       <c r="B49" s="99" t="inlineStr">
@@ -13999,12 +14008,12 @@
       </c>
       <c r="C49" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 관계 현실 유효 종료(ISO8601, bitemporal)</t>
+          <t>V4.6. 관계 현실 유효 시작(ISO8601, bitemporal)</t>
         </is>
       </c>
       <c r="D49" s="99" t="inlineStr">
         <is>
-          <t>used_ip, eg_used_account, eg_used_phone 등</t>
+          <t>used_ip, eg_used_account, eg_used_phone, registered_to, has_account 등</t>
         </is>
       </c>
       <c r="E49" s="107" t="inlineStr">
@@ -14016,7 +14025,7 @@
     <row r="50">
       <c r="A50" s="106" t="inlineStr">
         <is>
-          <t>first_dlng_dt</t>
+          <t>valid_to</t>
         </is>
       </c>
       <c r="B50" s="99" t="inlineStr">
@@ -14026,12 +14035,12 @@
       </c>
       <c r="C50" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 출발계좌 첫 거래일시 (추론경로 이체 기간 시작)</t>
+          <t>V4.6. 관계 현실 유효 종료(ISO8601, bitemporal)</t>
         </is>
       </c>
       <c r="D50" s="99" t="inlineStr">
         <is>
-          <t>transferred_to</t>
+          <t>used_ip, eg_used_account, eg_used_phone 등</t>
         </is>
       </c>
       <c r="E50" s="107" t="inlineStr">
@@ -14043,7 +14052,7 @@
     <row r="51">
       <c r="A51" s="106" t="inlineStr">
         <is>
-          <t>last_dlng_dt</t>
+          <t>first_dlng_dt</t>
         </is>
       </c>
       <c r="B51" s="99" t="inlineStr">
@@ -14053,7 +14062,7 @@
       </c>
       <c r="C51" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 출발계좌 마지막 거래일시 (추론경로 이체 기간 종료)</t>
+          <t>V4.6. 출발계좌 첫 거래일시 (추론경로 이체 기간 시작)</t>
         </is>
       </c>
       <c r="D51" s="99" t="inlineStr">
@@ -14070,17 +14079,17 @@
     <row r="52">
       <c r="A52" s="106" t="inlineStr">
         <is>
-          <t>txn_count</t>
+          <t>last_dlng_dt</t>
         </is>
       </c>
       <c r="B52" s="99" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C52" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 출발계좌 거래 건수 (기간 내)</t>
+          <t>V4.6. 출발계좌 마지막 거래일시 (추론경로 이체 기간 종료)</t>
         </is>
       </c>
       <c r="D52" s="99" t="inlineStr">
@@ -14090,14 +14099,14 @@
       </c>
       <c r="E52" s="107" t="inlineStr">
         <is>
-          <t>수치</t>
+          <t>시각</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="106" t="inlineStr">
         <is>
-          <t>total_amount</t>
+          <t>txn_count</t>
         </is>
       </c>
       <c r="B53" s="99" t="inlineStr">
@@ -14107,7 +14116,7 @@
       </c>
       <c r="C53" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 출발계좌 거래 총액(원)</t>
+          <t>V4.6. 출발계좌 거래 건수 (기간 내)</t>
         </is>
       </c>
       <c r="D53" s="99" t="inlineStr">
@@ -14124,52 +14133,52 @@
     <row r="54">
       <c r="A54" s="106" t="inlineStr">
         <is>
+          <t>total_amount</t>
+        </is>
+      </c>
+      <c r="B54" s="99" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C54" s="107" t="inlineStr">
+        <is>
+          <t>V4.6. 출발계좌 거래 총액(원)</t>
+        </is>
+      </c>
+      <c r="D54" s="99" t="inlineStr">
+        <is>
+          <t>transferred_to</t>
+        </is>
+      </c>
+      <c r="E54" s="107" t="inlineStr">
+        <is>
+          <t>수치</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="106" t="inlineStr">
+        <is>
           <t>time_basis</t>
         </is>
       </c>
-      <c r="B54" s="99" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C54" s="107" t="inlineStr">
+      <c r="B55" s="99" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C55" s="107" t="inlineStr">
         <is>
           <t>V4.6. 이체시각 산출 근거 (예: "출발계좌 거래활동 기간(추론경로 근사)")</t>
         </is>
       </c>
-      <c r="D54" s="99" t="inlineStr">
+      <c r="D55" s="99" t="inlineStr">
         <is>
           <t>transferred_to</t>
         </is>
       </c>
-      <c r="E54" s="107" t="inlineStr">
-        <is>
-          <t>텍스트</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="53" t="inlineStr">
-        <is>
-          <t>rprs_se_cd</t>
-        </is>
-      </c>
-      <c r="B55" s="53" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C55" s="53" t="inlineStr">
-        <is>
-          <t>V4.7. 법인 대표 구분코드 (TB_INST_RPRSV_REL_T.RPRS_SE_CD)</t>
-        </is>
-      </c>
-      <c r="D55" s="53" t="inlineStr">
-        <is>
-          <t>represents</t>
-        </is>
-      </c>
-      <c r="E55" s="53" t="inlineStr">
+      <c r="E55" s="107" t="inlineStr">
         <is>
           <t>텍스트</t>
         </is>
@@ -14178,7 +14187,7 @@
     <row r="56">
       <c r="A56" s="53" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>rprs_se_cd</t>
         </is>
       </c>
       <c r="B56" s="53" t="inlineStr">
@@ -14188,24 +14197,24 @@
       </c>
       <c r="C56" s="53" t="inlineStr">
         <is>
-          <t>연락 수단 구분 — 'call'|'kakao'|'sms' (V4.8)</t>
+          <t>V4.7. 법인 대표 구분코드 (TB_INST_RPRSV_REL_T.RPRS_SE_CD)</t>
         </is>
       </c>
       <c r="D56" s="53" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>represents</t>
         </is>
       </c>
       <c r="E56" s="53" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="53" t="inlineStr">
         <is>
-          <t>first_dt / last_dt</t>
+          <t>channel</t>
         </is>
       </c>
       <c r="B57" s="53" t="inlineStr">
@@ -14215,96 +14224,123 @@
       </c>
       <c r="C57" s="53" t="inlineStr">
         <is>
-          <t>쌍 집계 엣지의 최초/최종 관측 시각 (V4.9)</t>
+          <t>연락 수단 구분 — 'call'|'kakao'|'sms' (V4.8)</t>
         </is>
       </c>
       <c r="D57" s="53" t="inlineStr">
         <is>
-          <t>contacted, located_at</t>
+          <t>contacted</t>
         </is>
       </c>
       <c r="E57" s="53" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>enum</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="53" t="inlineStr">
         <is>
-          <t>evt_count</t>
+          <t>first_dt / last_dt</t>
         </is>
       </c>
       <c r="B58" s="53" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C58" s="53" t="inlineStr">
         <is>
-          <t>시각 있는 위치 관측 행 수 (V4.9)</t>
+          <t>쌍 집계 엣지의 최초/최종 관측 시각 (V4.9)</t>
         </is>
       </c>
       <c r="D58" s="53" t="inlineStr">
         <is>
-          <t>located_at</t>
+          <t>contacted, located_at</t>
         </is>
       </c>
       <c r="E58" s="53" t="inlineStr">
         <is>
-          <t>수치</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="53" t="inlineStr">
         <is>
-          <t>access_type</t>
+          <t>evt_count</t>
         </is>
       </c>
       <c r="B59" s="53" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C59" s="53" t="inlineStr">
         <is>
-          <t>접속 유형 web|comm|banking — 여러 값이면 '|' 결합 (V4.9)</t>
+          <t>시각 있는 위치 관측 행 수 (V4.9)</t>
         </is>
       </c>
       <c r="D59" s="53" t="inlineStr">
         <is>
-          <t>used_ip</t>
+          <t>located_at</t>
         </is>
       </c>
       <c r="E59" s="53" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>수치</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="53" t="inlineStr">
         <is>
+          <t>access_type</t>
+        </is>
+      </c>
+      <c r="B60" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C60" s="53" t="inlineStr">
+        <is>
+          <t>접속 유형 web|comm|banking — 여러 값이면 '|' 결합 (V4.9)</t>
+        </is>
+      </c>
+      <c r="D60" s="53" t="inlineStr">
+        <is>
+          <t>used_ip</t>
+        </is>
+      </c>
+      <c r="E60" s="53" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="53" t="inlineStr">
+        <is>
           <t>call_count / msg_count / total_dur_sec</t>
         </is>
       </c>
-      <c r="B60" s="53" t="inlineStr">
+      <c r="B61" s="53" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="C60" s="53" t="inlineStr">
+      <c r="C61" s="53" t="inlineStr">
         <is>
           <t>통화 건수 / 메시지 건수 / 통화 총 초 (V4.9 집계)</t>
         </is>
       </c>
-      <c r="D60" s="53" t="inlineStr">
+      <c r="D61" s="53" t="inlineStr">
         <is>
           <t>contacted</t>
         </is>
       </c>
-      <c r="E60" s="53" t="inlineStr">
+      <c r="E61" s="53" t="inlineStr">
         <is>
           <t>수치</t>
         </is>
@@ -16428,7 +16464,7 @@
       </c>
       <c r="B20" s="110" t="inlineStr">
         <is>
-          <t>53종 (deprecated 0) — V4.9: via_ip·sent_from_ip→accessed_from·occurred_at→located_at·linked_id→linked_to 통합 + vt_email→vt_id 흡수(uses_email·eg_used_email 삭제) + mentions_* 3종→mentions 통합 + 추론 결과 엣지 4종 + 중복·폐기 엣지 7종(owns_device·impersonates·involves·owns·verified_by·linked_petition·works_at) 삭제. 검증자는 엣지 메타 verified_by 속성.</t>
+          <t>52종 (deprecated 0) — V4.9: hosts→resolves_to(basis) 통합 + via_ip·sent_from_ip→accessed_from·occurred_at→located_at·linked_id→linked_to 통합 + vt_email→vt_id 흡수(uses_email·eg_used_email 삭제) + mentions_* 3종→mentions 통합 + 추론 결과 엣지 4종 + 중복·폐기 엣지 7종(owns_device·impersonates·involves·owns·verified_by·linked_petition·works_at) 삭제. 검증자는 엣지 메타 verified_by 속성.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ontology): V4.9 엑셀 잔재 정리 + same_as.review_status 값 확정 + 협력기관 변경 안내 초안
V4.9 엑셀 (handoff/ontology_v4.9/spec, 변경이력 R29)
- sameAs → same_as 표기 통일 (V4.8 개명 잔재 11곳)
- 주 사용 엣지 V4.9 표기: mentions_account→mentions·controls, linked_petition→filed_as,
  verified_by 엣지→엣지 공통 메타, match_basis_type→match_basis
- V4.9 폐지 속성 4행 삭제: transferred_to hop_level·time_basis, same_as match_score·match_basis_type

same_as.review_status = pending | confirmed | rejected (traversal_policy candidate_only|follow|block 1:1)
- V4.5 설계(값 도메인 사전)를 정본으로 — SoT 주석·README 의 confirmed|candidate, refine 스크립트 'candidate' 정정
- 실데이터 review_status 보유 0건이라 이관 불요

OSINT 엔티티 해소(osint_entity_resolution.py): sameAs 라벨(DB 실현 'sameas')→same_as,
match_score→confidence, traversal_policy 설정

handoff/MAIL_NOTICE_V49_20261001.md: 협력기관 공유용 V4.9 변경 안내 메일 초안

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
+++ b/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="53" min="1" max="1"/>
@@ -2761,6 +2761,43 @@
       <c r="G57" s="53" t="inlineStr">
         <is>
           <t>OSINT 13,769건이 모두 DNS 결과의 역방향 복사본(짝 없는 hosts 0건, 속성 없음). 호스팅·DNS 구분은 CDN·가상호스팅 수사에 필요해 속성으로 보존. OSINT 제출 hosts 는 경고 후 변환</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="53" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B58" s="53" t="inlineStr">
+        <is>
+          <t>V4.9</t>
+        </is>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="D58" s="53" t="inlineStr">
+        <is>
+          <t>엑셀 잔재 · same_as.review_status</t>
+        </is>
+      </c>
+      <c r="E58" s="53" t="inlineStr">
+        <is>
+          <t>sameAs 표기·삭제 엣지(mentions_account·linked_petition·verified_by) 참조·transferred_to hop_level/time_basis·match_score/match_basis_type 행 잔존, review_status 값 혼재(pending/candidate)</t>
+        </is>
+      </c>
+      <c r="F58" s="53" t="inlineStr">
+        <is>
+          <t>same_as 로 표기 통일, 주 사용 엣지를 V4.9 표기로, 폐지 속성 4행 삭제(hop_level·time_basis·match_score·match_basis_type). review_status = pending|confirmed|rejected (traversal_policy candidate_only|follow|block 1:1)</t>
+        </is>
+      </c>
+      <c r="G58" s="53" t="inlineStr">
+        <is>
+          <t>V4.5 설계(값 도메인 사전)를 정본으로 확정 — 적재 실데이터 0건이라 이관 불요. OSINT 엔티티 해소 스크립트도 same_as·confidence 로 정정</t>
         </is>
       </c>
     </row>
@@ -12507,7 +12544,7 @@
       </c>
       <c r="D261" s="107" t="inlineStr">
         <is>
-          <t>차수 기반 분류 — linked_entity_cnt 기준. sameAs 해소 전에는 provisional 접미어 부여. 파생</t>
+          <t>차수 기반 분류 — linked_entity_cnt 기준. same_as 해소 전에는 provisional 접미어 부여. 파생</t>
         </is>
       </c>
       <c r="E261" s="107" t="inlineStr">
@@ -12561,7 +12598,7 @@
       </c>
       <c r="D263" s="99" t="inlineStr">
         <is>
-          <t>sameAs(confirmed) 해소 후의 실체 수. ip_role 판정의 정식 입력값. 파생</t>
+          <t>same_as(confirmed) 해소 후의 실체 수. ip_role 판정의 정식 입력값. 파생</t>
         </is>
       </c>
       <c r="E263" s="107" t="inlineStr">
@@ -12691,7 +12728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="53" min="1" max="1"/>
@@ -12744,7 +12781,7 @@
       </c>
       <c r="D2" s="85" t="inlineStr">
         <is>
-          <t>same_as, controls, mentions_account 등</t>
+          <t>same_as, controls, mentions 등</t>
         </is>
       </c>
       <c r="E2" s="92" t="inlineStr">
@@ -12916,36 +12953,36 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" s="54">
-      <c r="A9" s="85" t="inlineStr">
-        <is>
-          <t>match_score</t>
+      <c r="A9" s="95" t="inlineStr">
+        <is>
+          <t>match_basis</t>
         </is>
       </c>
       <c r="B9" s="85" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C9" s="86" t="inlineStr">
         <is>
-          <t>[V4.9 폐지 → confidence] 엔티티 매칭 점수</t>
+          <t>동일인 판단 근거(공유 전화/계좌 등)</t>
         </is>
       </c>
       <c r="D9" s="85" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="E9" s="92" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" s="54">
-      <c r="A10" s="95" t="inlineStr">
-        <is>
-          <t>match_basis</t>
+      <c r="A10" s="85" t="inlineStr">
+        <is>
+          <t>review_status</t>
         </is>
       </c>
       <c r="B10" s="85" t="inlineStr">
@@ -12955,24 +12992,24 @@
       </c>
       <c r="C10" s="86" t="inlineStr">
         <is>
-          <t>동일인 판단 근거(공유 전화/계좌 등)</t>
+          <t>매칭 검토 상태(pending|confirmed|rejected) — traversal_policy 와 1:1</t>
         </is>
       </c>
       <c r="D10" s="85" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="E10" s="92" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="54">
       <c r="A11" s="85" t="inlineStr">
         <is>
-          <t>review_status</t>
+          <t>role / position</t>
         </is>
       </c>
       <c r="B11" s="85" t="inlineStr">
@@ -12982,51 +13019,51 @@
       </c>
       <c r="C11" s="86" t="inlineStr">
         <is>
-          <t>매칭 검토 상태(pending|confirmed)</t>
+          <t>조직 내 역할 / 재직 직위</t>
         </is>
       </c>
       <c r="D11" s="85" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>member_of</t>
         </is>
       </c>
       <c r="E11" s="92" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="54">
       <c r="A12" s="85" t="inlineStr">
         <is>
-          <t>hop_level</t>
+          <t>port / detected_at</t>
         </is>
       </c>
       <c r="B12" s="85" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>int/str</t>
         </is>
       </c>
       <c r="C12" s="86" t="inlineStr">
         <is>
-          <t>자금흐름 세탁 단계(1=직접)</t>
+          <t>호스팅 포트 / 탐지 시각</t>
         </is>
       </c>
       <c r="D12" s="85" t="inlineStr">
         <is>
-          <t>transferred_to</t>
+          <t>contains_file, resolves_to(구 hosts)</t>
         </is>
       </c>
       <c r="E12" s="92" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" s="54">
       <c r="A13" s="85" t="inlineStr">
         <is>
-          <t>role / position</t>
+          <t>resolved_dt</t>
         </is>
       </c>
       <c r="B13" s="85" t="inlineStr">
@@ -13034,80 +13071,80 @@
           <t>str</t>
         </is>
       </c>
-      <c r="C13" s="86" t="inlineStr">
-        <is>
-          <t>조직 내 역할 / 재직 직위</t>
+      <c r="C13" s="85" t="inlineStr">
+        <is>
+          <t>DNS 해석 시각</t>
         </is>
       </c>
       <c r="D13" s="85" t="inlineStr">
         <is>
-          <t>member_of</t>
+          <t>resolves_to</t>
         </is>
       </c>
       <c r="E13" s="92" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" s="54">
       <c r="A14" s="85" t="inlineStr">
         <is>
-          <t>port / detected_at</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="B14" s="85" t="inlineStr">
         <is>
-          <t>int/str</t>
-        </is>
-      </c>
-      <c r="C14" s="86" t="inlineStr">
-        <is>
-          <t>호스팅 포트 / 탐지 시각</t>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C14" s="85" t="inlineStr">
+        <is>
+          <t>연결 근거 — 'dns'(DNS 조회 관측, 미기재 시 기본) · 'origin'(원본 서버 확인: 호스팅사 회신·압수)</t>
         </is>
       </c>
       <c r="D14" s="85" t="inlineStr">
         <is>
-          <t>contains_file, resolves_to(구 hosts)</t>
+          <t>resolves_to</t>
         </is>
       </c>
       <c r="E14" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" s="54">
       <c r="A15" s="85" t="inlineStr">
         <is>
-          <t>resolved_dt</t>
+          <t>src_tier</t>
         </is>
       </c>
       <c r="B15" s="85" t="inlineStr">
         <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C15" s="85" t="inlineStr">
-        <is>
-          <t>DNS 해석 시각</t>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C15" s="86" t="inlineStr">
+        <is>
+          <t>출처 신뢰등급(1~5)</t>
         </is>
       </c>
       <c r="D15" s="85" t="inlineStr">
         <is>
-          <t>resolves_to</t>
+          <t>sourced_from</t>
         </is>
       </c>
       <c r="E15" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="54">
       <c r="A16" s="85" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>link_type / link_reason</t>
         </is>
       </c>
       <c r="B16" s="85" t="inlineStr">
@@ -13115,14 +13152,14 @@
           <t>str</t>
         </is>
       </c>
-      <c r="C16" s="85" t="inlineStr">
-        <is>
-          <t>연결 근거 — 'dns'(DNS 조회 관측, 미기재 시 기본) · 'origin'(원본 서버 확인: 호스팅사 회신·압수)</t>
+      <c r="C16" s="86" t="inlineStr">
+        <is>
+          <t>연결 유형 / 사유</t>
         </is>
       </c>
       <c r="D16" s="85" t="inlineStr">
         <is>
-          <t>resolves_to</t>
+          <t>linked_to</t>
         </is>
       </c>
       <c r="E16" s="92" t="inlineStr">
@@ -13134,34 +13171,34 @@
     <row r="17" ht="18" customHeight="1" s="54">
       <c r="A17" s="85" t="inlineStr">
         <is>
-          <t>src_tier</t>
+          <t>first_seen / last_seen</t>
         </is>
       </c>
       <c r="B17" s="85" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C17" s="86" t="inlineStr">
         <is>
-          <t>출처 신뢰등급(1~5)</t>
+          <t>최초/최종 관측 시각</t>
         </is>
       </c>
       <c r="D17" s="85" t="inlineStr">
         <is>
-          <t>sourced_from</t>
+          <t>used_in_device</t>
         </is>
       </c>
       <c r="E17" s="92" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="54">
       <c r="A18" s="85" t="inlineStr">
         <is>
-          <t>link_type / link_reason</t>
+          <t>converted_dt / converted_by</t>
         </is>
       </c>
       <c r="B18" s="85" t="inlineStr">
@@ -13171,51 +13208,51 @@
       </c>
       <c r="C18" s="86" t="inlineStr">
         <is>
-          <t>연결 유형 / 사유</t>
+          <t>사건 전환 시각 / 주체</t>
         </is>
       </c>
       <c r="D18" s="85" t="inlineStr">
         <is>
-          <t>linked_to</t>
+          <t>filed_as</t>
         </is>
       </c>
       <c r="E18" s="92" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="54">
       <c r="A19" s="85" t="inlineStr">
         <is>
-          <t>first_seen / last_seen</t>
+          <t>damage_amount</t>
         </is>
       </c>
       <c r="B19" s="85" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C19" s="86" t="inlineStr">
         <is>
-          <t>최초/최종 관측 시각</t>
+          <t>피해금액(원)</t>
         </is>
       </c>
       <c r="D19" s="85" t="inlineStr">
         <is>
-          <t>used_in_device</t>
+          <t>victim_in</t>
         </is>
       </c>
       <c r="E19" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="54">
       <c r="A20" s="85" t="inlineStr">
         <is>
-          <t>converted_dt / converted_by</t>
+          <t>statement_date</t>
         </is>
       </c>
       <c r="B20" s="85" t="inlineStr">
@@ -13225,12 +13262,12 @@
       </c>
       <c r="C20" s="86" t="inlineStr">
         <is>
-          <t>사건 전환 시각 / 주체</t>
+          <t>참고인 진술일</t>
         </is>
       </c>
       <c r="D20" s="85" t="inlineStr">
         <is>
-          <t>filed_as</t>
+          <t>witness_in</t>
         </is>
       </c>
       <c r="E20" s="92" t="inlineStr">
@@ -13242,34 +13279,34 @@
     <row r="21" ht="18" customHeight="1" s="54">
       <c r="A21" s="85" t="inlineStr">
         <is>
-          <t>damage_amount</t>
+          <t>recruit_type / payment</t>
         </is>
       </c>
       <c r="B21" s="85" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C21" s="86" t="inlineStr">
         <is>
-          <t>피해금액(원)</t>
+          <t>모집 유형 / 대가</t>
         </is>
       </c>
       <c r="D21" s="85" t="inlineStr">
         <is>
-          <t>victim_in</t>
+          <t>recruits</t>
         </is>
       </c>
       <c r="E21" s="92" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="54">
       <c r="A22" s="85" t="inlineStr">
         <is>
-          <t>statement_date</t>
+          <t>method / date</t>
         </is>
       </c>
       <c r="B22" s="85" t="inlineStr">
@@ -13279,24 +13316,24 @@
       </c>
       <c r="C22" s="86" t="inlineStr">
         <is>
-          <t>참고인 진술일</t>
+          <t>협박 방법 / 일자</t>
         </is>
       </c>
       <c r="D22" s="85" t="inlineStr">
         <is>
-          <t>witness_in</t>
+          <t>blackmails</t>
         </is>
       </c>
       <c r="E22" s="92" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="54">
       <c r="A23" s="85" t="inlineStr">
         <is>
-          <t>recruit_type / payment</t>
+          <t>file_role</t>
         </is>
       </c>
       <c r="B23" s="85" t="inlineStr">
@@ -13306,51 +13343,51 @@
       </c>
       <c r="C23" s="86" t="inlineStr">
         <is>
-          <t>모집 유형 / 대가</t>
+          <t>파일의 역할(첨부/배포/증거)</t>
         </is>
       </c>
       <c r="D23" s="85" t="inlineStr">
         <is>
-          <t>recruits</t>
+          <t>contains_file</t>
         </is>
       </c>
       <c r="E23" s="92" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="54">
       <c r="A24" s="85" t="inlineStr">
         <is>
-          <t>method / date</t>
+          <t>usage_count</t>
         </is>
       </c>
       <c r="B24" s="85" t="inlineStr">
         <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C24" s="86" t="inlineStr">
-        <is>
-          <t>협박 방법 / 일자</t>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C24" s="85" t="inlineStr">
+        <is>
+          <t>IP 사용(접속) 행 수 — (주체,IP)쌍 집계 시 합계 (V4.9)</t>
         </is>
       </c>
       <c r="D24" s="85" t="inlineStr">
         <is>
-          <t>blackmails</t>
+          <t>used_ip</t>
         </is>
       </c>
       <c r="E24" s="92" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="54">
       <c r="A25" s="85" t="inlineStr">
         <is>
-          <t>file_role</t>
+          <t>verified_dt</t>
         </is>
       </c>
       <c r="B25" s="85" t="inlineStr">
@@ -13360,51 +13397,51 @@
       </c>
       <c r="C25" s="86" t="inlineStr">
         <is>
-          <t>파일의 역할(첨부/배포/증거)</t>
+          <t>검증 시각</t>
         </is>
       </c>
       <c r="D25" s="85" t="inlineStr">
         <is>
-          <t>contains_file</t>
+          <t>(엣지 공통 메타 — V4.9 verified_by 엣지 삭제)</t>
         </is>
       </c>
       <c r="E25" s="92" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="54">
       <c r="A26" s="85" t="inlineStr">
         <is>
-          <t>usage_count</t>
+          <t>relation_type</t>
         </is>
       </c>
       <c r="B26" s="85" t="inlineStr">
         <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C26" s="85" t="inlineStr">
-        <is>
-          <t>IP 사용(접속) 행 수 — (주체,IP)쌍 집계 시 합계 (V4.9)</t>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C26" s="86" t="inlineStr">
+        <is>
+          <t>지인 관계 유형(친구/동창/가족 등)</t>
         </is>
       </c>
       <c r="D26" s="85" t="inlineStr">
         <is>
-          <t>used_ip</t>
-        </is>
-      </c>
-      <c r="E26" s="92" t="inlineStr">
-        <is>
-          <t>수치형</t>
+          <t>knows</t>
+        </is>
+      </c>
+      <c r="E26" s="86" t="inlineStr">
+        <is>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="54">
       <c r="A27" s="85" t="inlineStr">
         <is>
-          <t>verified_dt</t>
+          <t>link_basis</t>
         </is>
       </c>
       <c r="B27" s="85" t="inlineStr">
@@ -13414,78 +13451,78 @@
       </c>
       <c r="C27" s="86" t="inlineStr">
         <is>
-          <t>검증 시각</t>
+          <t>식별자 연결 근거(인증서발급/포털역조회 등)</t>
         </is>
       </c>
       <c r="D27" s="85" t="inlineStr">
         <is>
-          <t>verified_by</t>
-        </is>
-      </c>
-      <c r="E27" s="92" t="inlineStr">
-        <is>
-          <t>날짜시간</t>
+          <t>linked_to(구 linked_id)</t>
+        </is>
+      </c>
+      <c r="E27" s="86" t="inlineStr">
+        <is>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="54">
-      <c r="A28" s="85" t="inlineStr">
-        <is>
-          <t>relation_type</t>
-        </is>
-      </c>
-      <c r="B28" s="85" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C28" s="86" t="inlineStr">
-        <is>
-          <t>지인 관계 유형(친구/동창/가족 등)</t>
-        </is>
-      </c>
-      <c r="D28" s="85" t="inlineStr">
-        <is>
-          <t>knows</t>
-        </is>
-      </c>
-      <c r="E28" s="86" t="inlineStr">
+      <c r="A28" s="98" t="inlineStr">
+        <is>
+          <t>actor_type</t>
+        </is>
+      </c>
+      <c r="B28" s="99" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C28" s="100" t="inlineStr">
+        <is>
+          <t>이벤트 행위 주체의 유형 (person | telno | online_id)</t>
+        </is>
+      </c>
+      <c r="D28" s="99" t="inlineStr">
+        <is>
+          <t>performed_by</t>
+        </is>
+      </c>
+      <c r="E28" s="100" t="inlineStr">
         <is>
           <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="54">
-      <c r="A29" s="85" t="inlineStr">
-        <is>
-          <t>link_basis</t>
-        </is>
-      </c>
-      <c r="B29" s="85" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C29" s="86" t="inlineStr">
-        <is>
-          <t>식별자 연결 근거(인증서발급/포털역조회 등)</t>
-        </is>
-      </c>
-      <c r="D29" s="85" t="inlineStr">
-        <is>
-          <t>linked_to(구 linked_id)</t>
-        </is>
-      </c>
-      <c r="E29" s="86" t="inlineStr">
-        <is>
-          <t>범주형</t>
+      <c r="A29" s="98" t="inlineStr">
+        <is>
+          <t>resolved_to</t>
+        </is>
+      </c>
+      <c r="B29" s="99" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C29" s="100" t="inlineStr">
+        <is>
+          <t>후속 특정된 vt_psn.psn_id (미특정 시 null)</t>
+        </is>
+      </c>
+      <c r="D29" s="99" t="inlineStr">
+        <is>
+          <t>performed_by</t>
+        </is>
+      </c>
+      <c r="E29" s="100" t="inlineStr">
+        <is>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="54">
       <c r="A30" s="98" t="inlineStr">
         <is>
-          <t>actor_type</t>
+          <t>resolved_at</t>
         </is>
       </c>
       <c r="B30" s="99" t="inlineStr">
@@ -13495,7 +13532,7 @@
       </c>
       <c r="C30" s="100" t="inlineStr">
         <is>
-          <t>이벤트 행위 주체의 유형 (person | telno | online_id)</t>
+          <t>주체가 인물로 특정된 시각(ISO8601)</t>
         </is>
       </c>
       <c r="D30" s="99" t="inlineStr">
@@ -13505,14 +13542,14 @@
       </c>
       <c r="E30" s="100" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>날짜시간</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" s="54">
       <c r="A31" s="98" t="inlineStr">
         <is>
-          <t>resolved_to</t>
+          <t>subject_type</t>
         </is>
       </c>
       <c r="B31" s="99" t="inlineStr">
@@ -13522,66 +13559,66 @@
       </c>
       <c r="C31" s="100" t="inlineStr">
         <is>
-          <t>후속 특정된 vt_psn.psn_id (미특정 시 null)</t>
+          <t>관계 주체의 유형 (person | telno | online_id)</t>
         </is>
       </c>
       <c r="D31" s="99" t="inlineStr">
         <is>
-          <t>performed_by</t>
+          <t>used_ip</t>
         </is>
       </c>
       <c r="E31" s="100" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="54">
       <c r="A32" s="98" t="inlineStr">
         <is>
-          <t>resolved_at</t>
+          <t>duration_days</t>
         </is>
       </c>
       <c r="B32" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C32" s="100" t="inlineStr">
         <is>
-          <t>주체가 인물로 특정된 시각(ISO8601)</t>
+          <t>관계 유효 기간(일) = valid_to - valid_from. 파생값</t>
         </is>
       </c>
       <c r="D32" s="99" t="inlineStr">
         <is>
-          <t>performed_by</t>
+          <t>registered_to, eg_used_* 3종</t>
         </is>
       </c>
       <c r="E32" s="100" t="inlineStr">
         <is>
-          <t>날짜시간</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" s="54">
       <c r="A33" s="98" t="inlineStr">
         <is>
-          <t>subject_type</t>
+          <t>inference_basis_type</t>
         </is>
       </c>
       <c r="B33" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>list</t>
         </is>
       </c>
       <c r="C33" s="100" t="inlineStr">
         <is>
-          <t>관계 주체의 유형 (person | telno | online_id)</t>
+          <t>추론 근거 유형 배열 — 값도메인 시트 참조. 복수 근거 지원</t>
         </is>
       </c>
       <c r="D33" s="99" t="inlineStr">
         <is>
-          <t>used_ip</t>
+          <t>controls</t>
         </is>
       </c>
       <c r="E33" s="100" t="inlineStr">
@@ -13593,103 +13630,103 @@
     <row r="34" ht="30" customHeight="1" s="54">
       <c r="A34" s="98" t="inlineStr">
         <is>
-          <t>duration_days</t>
+          <t>evidence_edge_ids</t>
         </is>
       </c>
       <c r="B34" s="99" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>list</t>
         </is>
       </c>
       <c r="C34" s="100" t="inlineStr">
         <is>
-          <t>관계 유효 기간(일) = valid_to - valid_from. 파생값</t>
-        </is>
-      </c>
-      <c r="D34" s="99" t="inlineStr">
-        <is>
-          <t>registered_to, eg_used_* 3종</t>
+          <t>근거가 된 원천 엣지 ID 배열 (법정 재현용 · 소급 복원 불가)</t>
+        </is>
+      </c>
+      <c r="D34" s="100" t="inlineStr">
+        <is>
+          <t>추론 엣지 6종</t>
         </is>
       </c>
       <c r="E34" s="100" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1" s="54">
       <c r="A35" s="98" t="inlineStr">
         <is>
-          <t>inference_basis_type</t>
+          <t>evidence_count</t>
         </is>
       </c>
       <c r="B35" s="99" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C35" s="100" t="inlineStr">
         <is>
-          <t>추론 근거 유형 배열 — 값도메인 시트 참조. 복수 근거 지원</t>
-        </is>
-      </c>
-      <c r="D35" s="99" t="inlineStr">
-        <is>
-          <t>controls, mentions_account</t>
+          <t>근거 건수 (예: 공유 IP에서의 접속 레코드 수)</t>
+        </is>
+      </c>
+      <c r="D35" s="100" t="inlineStr">
+        <is>
+          <t>추론 엣지 6종</t>
         </is>
       </c>
       <c r="E35" s="100" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" s="54">
       <c r="A36" s="98" t="inlineStr">
         <is>
-          <t>match_basis_type</t>
+          <t>evidence_summary</t>
         </is>
       </c>
       <c r="B36" s="99" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C36" s="100" t="inlineStr">
         <is>
-          <t>[V4.9 폐지 → match_basis] 동일성 판단 근거 유형 배열 — 값도메인 시트 참조</t>
-        </is>
-      </c>
-      <c r="D36" s="99" t="inlineStr">
-        <is>
-          <t>sameAs</t>
+          <t>사람이 읽는 근거 요약 (구 inference_basis / match_basis 역할)</t>
+        </is>
+      </c>
+      <c r="D36" s="100" t="inlineStr">
+        <is>
+          <t>추론 엣지 6종</t>
         </is>
       </c>
       <c r="E36" s="100" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1" s="54">
       <c r="A37" s="98" t="inlineStr">
         <is>
-          <t>evidence_edge_ids</t>
+          <t>warrant_no</t>
         </is>
       </c>
       <c r="B37" s="99" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C37" s="100" t="inlineStr">
         <is>
-          <t>근거가 된 원천 엣지 ID 배열 (법정 재현용 · 소급 복원 불가)</t>
-        </is>
-      </c>
-      <c r="D37" s="100" t="inlineStr">
-        <is>
-          <t>추론 엣지 6종</t>
+          <t>근거 영장·허가서 번호</t>
+        </is>
+      </c>
+      <c r="D37" s="99" t="inlineStr">
+        <is>
+          <t>linked_to(구 linked_id), eg_used_* 4종</t>
         </is>
       </c>
       <c r="E37" s="100" t="inlineStr">
@@ -13701,88 +13738,88 @@
     <row r="38" ht="30" customHeight="1" s="54">
       <c r="A38" s="98" t="inlineStr">
         <is>
-          <t>evidence_count</t>
+          <t>exchange_nm</t>
         </is>
       </c>
       <c r="B38" s="99" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C38" s="100" t="inlineStr">
         <is>
-          <t>근거 건수 (예: 공유 IP에서의 접속 레코드 수)</t>
-        </is>
-      </c>
-      <c r="D38" s="100" t="inlineStr">
-        <is>
-          <t>추론 엣지 6종</t>
+          <t>가상자산 거래소명</t>
+        </is>
+      </c>
+      <c r="D38" s="99" t="inlineStr">
+        <is>
+          <t>exchanged_to</t>
         </is>
       </c>
       <c r="E38" s="100" t="inlineStr">
         <is>
-          <t>수치형</t>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1" s="54">
       <c r="A39" s="98" t="inlineStr">
         <is>
-          <t>evidence_summary</t>
+          <t>fiat_amt</t>
         </is>
       </c>
       <c r="B39" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C39" s="100" t="inlineStr">
         <is>
-          <t>사람이 읽는 근거 요약 (구 inference_basis / match_basis 역할)</t>
-        </is>
-      </c>
-      <c r="D39" s="100" t="inlineStr">
-        <is>
-          <t>추론 엣지 6종</t>
+          <t>전환 원화 금액(원)</t>
+        </is>
+      </c>
+      <c r="D39" s="99" t="inlineStr">
+        <is>
+          <t>exchanged_to</t>
         </is>
       </c>
       <c r="E39" s="100" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1" s="54">
       <c r="A40" s="98" t="inlineStr">
         <is>
-          <t>warrant_no</t>
+          <t>asset_amt</t>
         </is>
       </c>
       <c r="B40" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float</t>
         </is>
       </c>
       <c r="C40" s="100" t="inlineStr">
         <is>
-          <t>근거 영장·허가서 번호</t>
+          <t>전환 가상자산 수량</t>
         </is>
       </c>
       <c r="D40" s="99" t="inlineStr">
         <is>
-          <t>linked_to(구 linked_id), eg_used_* 4종</t>
+          <t>exchanged_to</t>
         </is>
       </c>
       <c r="E40" s="100" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>수치형</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1" s="54">
       <c r="A41" s="98" t="inlineStr">
         <is>
-          <t>exchange_nm</t>
+          <t>link_reason</t>
         </is>
       </c>
       <c r="B41" s="99" t="inlineStr">
@@ -13792,12 +13829,12 @@
       </c>
       <c r="C41" s="100" t="inlineStr">
         <is>
-          <t>가상자산 거래소명</t>
+          <t>진정서-사건 연결 사유</t>
         </is>
       </c>
       <c r="D41" s="99" t="inlineStr">
         <is>
-          <t>exchanged_to</t>
+          <t>filed_as(구 linked_petition)</t>
         </is>
       </c>
       <c r="E41" s="100" t="inlineStr">
@@ -13807,63 +13844,63 @@
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" s="54">
-      <c r="A42" s="98" t="inlineStr">
-        <is>
-          <t>fiat_amt</t>
+      <c r="A42" s="106" t="inlineStr">
+        <is>
+          <t>traversal_policy</t>
         </is>
       </c>
       <c r="B42" s="99" t="inlineStr">
         <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C42" s="100" t="inlineStr">
-        <is>
-          <t>전환 원화 금액(원)</t>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C42" s="107" t="inlineStr">
+        <is>
+          <t>탐색 시 이 엣지를 따라갈지 결정 (follow | candidate_only | block). review_status 와 연동</t>
         </is>
       </c>
       <c r="D42" s="99" t="inlineStr">
         <is>
-          <t>exchanged_to</t>
-        </is>
-      </c>
-      <c r="E42" s="100" t="inlineStr">
-        <is>
-          <t>수치형</t>
+          <t>same_as</t>
+        </is>
+      </c>
+      <c r="E42" s="107" t="inlineStr">
+        <is>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1" s="54">
-      <c r="A43" s="98" t="inlineStr">
-        <is>
-          <t>asset_amt</t>
+      <c r="A43" s="106" t="inlineStr">
+        <is>
+          <t>edge_id</t>
         </is>
       </c>
       <c r="B43" s="99" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="C43" s="100" t="inlineStr">
-        <is>
-          <t>전환 가상자산 수량</t>
-        </is>
-      </c>
-      <c r="D43" s="99" t="inlineStr">
-        <is>
-          <t>exchanged_to</t>
-        </is>
-      </c>
-      <c r="E43" s="100" t="inlineStr">
-        <is>
-          <t>수치형</t>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C43" s="107" t="inlineStr">
+        <is>
+          <t>엣지의 안정적 고유 식별자 — evidence_edge_ids 가 참조. 재적재 시에도 불변이어야 함</t>
+        </is>
+      </c>
+      <c r="D43" s="107" t="inlineStr">
+        <is>
+          <t>전 엣지 공통</t>
+        </is>
+      </c>
+      <c r="E43" s="107" t="inlineStr">
+        <is>
+          <t>식별자</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" s="54">
-      <c r="A44" s="98" t="inlineStr">
-        <is>
-          <t>link_reason</t>
+      <c r="A44" s="106" t="inlineStr">
+        <is>
+          <t>target_type</t>
         </is>
       </c>
       <c r="B44" s="99" t="inlineStr">
@@ -13871,26 +13908,26 @@
           <t>str</t>
         </is>
       </c>
-      <c r="C44" s="100" t="inlineStr">
-        <is>
-          <t>진정서-사건 연결 사유</t>
+      <c r="C44" s="107" t="inlineStr">
+        <is>
+          <t>접속 목적지 유형 (site | account | online_id)</t>
         </is>
       </c>
       <c r="D44" s="99" t="inlineStr">
         <is>
-          <t>linked_petition</t>
-        </is>
-      </c>
-      <c r="E44" s="100" t="inlineStr">
-        <is>
-          <t>텍스트</t>
+          <t>accessed_to</t>
+        </is>
+      </c>
+      <c r="E44" s="107" t="inlineStr">
+        <is>
+          <t>범주형</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1" s="54">
       <c r="A45" s="106" t="inlineStr">
         <is>
-          <t>traversal_policy</t>
+          <t>direction</t>
         </is>
       </c>
       <c r="B45" s="99" t="inlineStr">
@@ -13900,12 +13937,12 @@
       </c>
       <c r="C45" s="107" t="inlineStr">
         <is>
-          <t>탐색 시 이 엣지를 따라갈지 결정 (follow | candidate_only | block). review_status 와 연동</t>
+          <t>탐색 방향성 (directed | undirected). undirected 선언 시 역방향 인덱스 필수</t>
         </is>
       </c>
       <c r="D45" s="99" t="inlineStr">
         <is>
-          <t>same_as</t>
+          <t>used_ip, contacted, communicated_with</t>
         </is>
       </c>
       <c r="E45" s="107" t="inlineStr">
@@ -13917,7 +13954,7 @@
     <row r="46" ht="30" customHeight="1" s="54">
       <c r="A46" s="106" t="inlineStr">
         <is>
-          <t>edge_id</t>
+          <t>valid_from</t>
         </is>
       </c>
       <c r="B46" s="99" t="inlineStr">
@@ -13927,24 +13964,24 @@
       </c>
       <c r="C46" s="107" t="inlineStr">
         <is>
-          <t>엣지의 안정적 고유 식별자 — evidence_edge_ids 가 참조. 재적재 시에도 불변이어야 함</t>
-        </is>
-      </c>
-      <c r="D46" s="107" t="inlineStr">
-        <is>
-          <t>전 엣지 공통</t>
+          <t>V4.6. 관계 현실 유효 시작(ISO8601, bitemporal)</t>
+        </is>
+      </c>
+      <c r="D46" s="99" t="inlineStr">
+        <is>
+          <t>used_ip, eg_used_account, eg_used_phone, registered_to, has_account 등</t>
         </is>
       </c>
       <c r="E46" s="107" t="inlineStr">
         <is>
-          <t>식별자</t>
+          <t>시각</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1" s="54">
       <c r="A47" s="106" t="inlineStr">
         <is>
-          <t>target_type</t>
+          <t>valid_to</t>
         </is>
       </c>
       <c r="B47" s="99" t="inlineStr">
@@ -13954,24 +13991,24 @@
       </c>
       <c r="C47" s="107" t="inlineStr">
         <is>
-          <t>접속 목적지 유형 (site | account | online_id)</t>
+          <t>V4.6. 관계 현실 유효 종료(ISO8601, bitemporal)</t>
         </is>
       </c>
       <c r="D47" s="99" t="inlineStr">
         <is>
-          <t>accessed_to</t>
+          <t>used_ip, eg_used_account, eg_used_phone 등</t>
         </is>
       </c>
       <c r="E47" s="107" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>시각</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1" s="54">
       <c r="A48" s="106" t="inlineStr">
         <is>
-          <t>direction</t>
+          <t>first_dlng_dt</t>
         </is>
       </c>
       <c r="B48" s="99" t="inlineStr">
@@ -13981,24 +14018,24 @@
       </c>
       <c r="C48" s="107" t="inlineStr">
         <is>
-          <t>탐색 방향성 (directed | undirected). undirected 선언 시 역방향 인덱스 필수</t>
+          <t>V4.6. 출발계좌 첫 거래일시 (추론경로 이체 기간 시작)</t>
         </is>
       </c>
       <c r="D48" s="99" t="inlineStr">
         <is>
-          <t>used_ip, contacted, communicated_with</t>
+          <t>transferred_to</t>
         </is>
       </c>
       <c r="E48" s="107" t="inlineStr">
         <is>
-          <t>범주형</t>
+          <t>시각</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1" s="54">
       <c r="A49" s="106" t="inlineStr">
         <is>
-          <t>valid_from</t>
+          <t>last_dlng_dt</t>
         </is>
       </c>
       <c r="B49" s="99" t="inlineStr">
@@ -14008,12 +14045,12 @@
       </c>
       <c r="C49" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 관계 현실 유효 시작(ISO8601, bitemporal)</t>
+          <t>V4.6. 출발계좌 마지막 거래일시 (추론경로 이체 기간 종료)</t>
         </is>
       </c>
       <c r="D49" s="99" t="inlineStr">
         <is>
-          <t>used_ip, eg_used_account, eg_used_phone, registered_to, has_account 등</t>
+          <t>transferred_to</t>
         </is>
       </c>
       <c r="E49" s="107" t="inlineStr">
@@ -14025,44 +14062,44 @@
     <row r="50">
       <c r="A50" s="106" t="inlineStr">
         <is>
-          <t>valid_to</t>
+          <t>txn_count</t>
         </is>
       </c>
       <c r="B50" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C50" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 관계 현실 유효 종료(ISO8601, bitemporal)</t>
+          <t>V4.6. 출발계좌 거래 건수 (기간 내)</t>
         </is>
       </c>
       <c r="D50" s="99" t="inlineStr">
         <is>
-          <t>used_ip, eg_used_account, eg_used_phone 등</t>
+          <t>transferred_to</t>
         </is>
       </c>
       <c r="E50" s="107" t="inlineStr">
         <is>
-          <t>시각</t>
+          <t>수치</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="106" t="inlineStr">
         <is>
-          <t>first_dlng_dt</t>
+          <t>total_amount</t>
         </is>
       </c>
       <c r="B51" s="99" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C51" s="107" t="inlineStr">
         <is>
-          <t>V4.6. 출발계좌 첫 거래일시 (추론경로 이체 기간 시작)</t>
+          <t>V4.6. 출발계좌 거래 총액(원)</t>
         </is>
       </c>
       <c r="D51" s="99" t="inlineStr">
@@ -14072,122 +14109,122 @@
       </c>
       <c r="E51" s="107" t="inlineStr">
         <is>
-          <t>시각</t>
+          <t>수치</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="106" t="inlineStr">
-        <is>
-          <t>last_dlng_dt</t>
-        </is>
-      </c>
-      <c r="B52" s="99" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C52" s="107" t="inlineStr">
-        <is>
-          <t>V4.6. 출발계좌 마지막 거래일시 (추론경로 이체 기간 종료)</t>
-        </is>
-      </c>
-      <c r="D52" s="99" t="inlineStr">
-        <is>
-          <t>transferred_to</t>
-        </is>
-      </c>
-      <c r="E52" s="107" t="inlineStr">
-        <is>
-          <t>시각</t>
+      <c r="A52" s="53" t="inlineStr">
+        <is>
+          <t>rprs_se_cd</t>
+        </is>
+      </c>
+      <c r="B52" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C52" s="53" t="inlineStr">
+        <is>
+          <t>V4.7. 법인 대표 구분코드 (TB_INST_RPRSV_REL_T.RPRS_SE_CD)</t>
+        </is>
+      </c>
+      <c r="D52" s="53" t="inlineStr">
+        <is>
+          <t>represents</t>
+        </is>
+      </c>
+      <c r="E52" s="53" t="inlineStr">
+        <is>
+          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="106" t="inlineStr">
-        <is>
-          <t>txn_count</t>
-        </is>
-      </c>
-      <c r="B53" s="99" t="inlineStr">
+      <c r="A53" s="53" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="B53" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C53" s="53" t="inlineStr">
+        <is>
+          <t>연락 수단 구분 — 'call'|'kakao'|'sms' (V4.8)</t>
+        </is>
+      </c>
+      <c r="D53" s="53" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="E53" s="53" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="53" t="inlineStr">
+        <is>
+          <t>first_dt / last_dt</t>
+        </is>
+      </c>
+      <c r="B54" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C54" s="53" t="inlineStr">
+        <is>
+          <t>쌍 집계 엣지의 최초/최종 관측 시각 (V4.9)</t>
+        </is>
+      </c>
+      <c r="D54" s="53" t="inlineStr">
+        <is>
+          <t>contacted, located_at</t>
+        </is>
+      </c>
+      <c r="E54" s="53" t="inlineStr">
+        <is>
+          <t>날짜시간</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="53" t="inlineStr">
+        <is>
+          <t>evt_count</t>
+        </is>
+      </c>
+      <c r="B55" s="53" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="C53" s="107" t="inlineStr">
-        <is>
-          <t>V4.6. 출발계좌 거래 건수 (기간 내)</t>
-        </is>
-      </c>
-      <c r="D53" s="99" t="inlineStr">
-        <is>
-          <t>transferred_to</t>
-        </is>
-      </c>
-      <c r="E53" s="107" t="inlineStr">
+      <c r="C55" s="53" t="inlineStr">
+        <is>
+          <t>시각 있는 위치 관측 행 수 (V4.9)</t>
+        </is>
+      </c>
+      <c r="D55" s="53" t="inlineStr">
+        <is>
+          <t>located_at</t>
+        </is>
+      </c>
+      <c r="E55" s="53" t="inlineStr">
         <is>
           <t>수치</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="106" t="inlineStr">
-        <is>
-          <t>total_amount</t>
-        </is>
-      </c>
-      <c r="B54" s="99" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C54" s="107" t="inlineStr">
-        <is>
-          <t>V4.6. 출발계좌 거래 총액(원)</t>
-        </is>
-      </c>
-      <c r="D54" s="99" t="inlineStr">
-        <is>
-          <t>transferred_to</t>
-        </is>
-      </c>
-      <c r="E54" s="107" t="inlineStr">
-        <is>
-          <t>수치</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="106" t="inlineStr">
-        <is>
-          <t>time_basis</t>
-        </is>
-      </c>
-      <c r="B55" s="99" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C55" s="107" t="inlineStr">
-        <is>
-          <t>V4.6. 이체시각 산출 근거 (예: "출발계좌 거래활동 기간(추론경로 근사)")</t>
-        </is>
-      </c>
-      <c r="D55" s="99" t="inlineStr">
-        <is>
-          <t>transferred_to</t>
-        </is>
-      </c>
-      <c r="E55" s="107" t="inlineStr">
-        <is>
-          <t>텍스트</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="53" t="inlineStr">
         <is>
-          <t>rprs_se_cd</t>
+          <t>access_type</t>
         </is>
       </c>
       <c r="B56" s="53" t="inlineStr">
@@ -14197,34 +14234,34 @@
       </c>
       <c r="C56" s="53" t="inlineStr">
         <is>
-          <t>V4.7. 법인 대표 구분코드 (TB_INST_RPRSV_REL_T.RPRS_SE_CD)</t>
+          <t>접속 유형 web|comm|banking — 여러 값이면 '|' 결합 (V4.9)</t>
         </is>
       </c>
       <c r="D56" s="53" t="inlineStr">
         <is>
-          <t>represents</t>
+          <t>used_ip</t>
         </is>
       </c>
       <c r="E56" s="53" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>enum</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="53" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>call_count / msg_count / total_dur_sec</t>
         </is>
       </c>
       <c r="B57" s="53" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="C57" s="53" t="inlineStr">
         <is>
-          <t>연락 수단 구분 — 'call'|'kakao'|'sms' (V4.8)</t>
+          <t>통화 건수 / 메시지 건수 / 통화 총 초 (V4.9 집계)</t>
         </is>
       </c>
       <c r="D57" s="53" t="inlineStr">
@@ -14233,114 +14270,6 @@
         </is>
       </c>
       <c r="E57" s="53" t="inlineStr">
-        <is>
-          <t>enum</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="53" t="inlineStr">
-        <is>
-          <t>first_dt / last_dt</t>
-        </is>
-      </c>
-      <c r="B58" s="53" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C58" s="53" t="inlineStr">
-        <is>
-          <t>쌍 집계 엣지의 최초/최종 관측 시각 (V4.9)</t>
-        </is>
-      </c>
-      <c r="D58" s="53" t="inlineStr">
-        <is>
-          <t>contacted, located_at</t>
-        </is>
-      </c>
-      <c r="E58" s="53" t="inlineStr">
-        <is>
-          <t>날짜시간</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="53" t="inlineStr">
-        <is>
-          <t>evt_count</t>
-        </is>
-      </c>
-      <c r="B59" s="53" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C59" s="53" t="inlineStr">
-        <is>
-          <t>시각 있는 위치 관측 행 수 (V4.9)</t>
-        </is>
-      </c>
-      <c r="D59" s="53" t="inlineStr">
-        <is>
-          <t>located_at</t>
-        </is>
-      </c>
-      <c r="E59" s="53" t="inlineStr">
-        <is>
-          <t>수치</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="53" t="inlineStr">
-        <is>
-          <t>access_type</t>
-        </is>
-      </c>
-      <c r="B60" s="53" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C60" s="53" t="inlineStr">
-        <is>
-          <t>접속 유형 web|comm|banking — 여러 값이면 '|' 결합 (V4.9)</t>
-        </is>
-      </c>
-      <c r="D60" s="53" t="inlineStr">
-        <is>
-          <t>used_ip</t>
-        </is>
-      </c>
-      <c r="E60" s="53" t="inlineStr">
-        <is>
-          <t>enum</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="53" t="inlineStr">
-        <is>
-          <t>call_count / msg_count / total_dur_sec</t>
-        </is>
-      </c>
-      <c r="B61" s="53" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C61" s="53" t="inlineStr">
-        <is>
-          <t>통화 건수 / 메시지 건수 / 통화 총 초 (V4.9 집계)</t>
-        </is>
-      </c>
-      <c r="D61" s="53" t="inlineStr">
-        <is>
-          <t>contacted</t>
-        </is>
-      </c>
-      <c r="E61" s="53" t="inlineStr">
         <is>
           <t>수치</t>
         </is>
@@ -14474,7 +14403,7 @@
       </c>
       <c r="B6" s="99" t="inlineStr">
         <is>
-          <t>controls / mentions_account</t>
+          <t>controls</t>
         </is>
       </c>
       <c r="C6" s="105" t="inlineStr">
@@ -14581,12 +14510,12 @@
     <row r="12" ht="18" customHeight="1" s="54">
       <c r="A12" s="98" t="inlineStr">
         <is>
-          <t>match_basis_type</t>
+          <t>match_basis</t>
         </is>
       </c>
       <c r="B12" s="99" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="C12" s="105" t="inlineStr">
@@ -14604,7 +14533,7 @@
       <c r="A13" s="105" t="n"/>
       <c r="B13" s="99" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="C13" s="105" t="inlineStr">
@@ -14622,7 +14551,7 @@
       <c r="A14" s="105" t="n"/>
       <c r="B14" s="99" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="C14" s="105" t="inlineStr">
@@ -14640,7 +14569,7 @@
       <c r="A15" s="105" t="n"/>
       <c r="B15" s="99" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="C15" s="105" t="inlineStr">
@@ -15274,7 +15203,7 @@
       </c>
       <c r="B48" s="99" t="inlineStr">
         <is>
-          <t>sameAs</t>
+          <t>same_as</t>
         </is>
       </c>
       <c r="C48" s="105" t="inlineStr">
@@ -15350,7 +15279,7 @@
       </c>
       <c r="D51" s="99" t="inlineStr">
         <is>
-          <t>sameAs 해소 전 산출 — 참고용</t>
+          <t>same_as 해소 전 산출 — 참고용</t>
         </is>
       </c>
     </row>
@@ -15372,7 +15301,7 @@
       </c>
       <c r="D52" s="99" t="inlineStr">
         <is>
-          <t>sameAs(confirmed) 해소 후 산출 — 정식</t>
+          <t>same_as(confirmed) 해소 후 산출 — 정식</t>
         </is>
       </c>
     </row>
@@ -15704,7 +15633,7 @@
       </c>
       <c r="B7" s="64" t="inlineStr">
         <is>
-          <t>sameAs 탐색</t>
+          <t>same_as 탐색</t>
         </is>
       </c>
       <c r="C7" s="61" t="inlineStr">
@@ -15790,7 +15719,7 @@
       </c>
       <c r="C10" s="61" t="inlineStr">
         <is>
-          <t>ip_role 은 sameAs 해소 이후에 산출한다</t>
+          <t>ip_role 은 same_as 해소 이후에 산출한다</t>
         </is>
       </c>
       <c r="D10" s="61" t="inlineStr">
@@ -15827,7 +15756,7 @@
       </c>
       <c r="E11" s="61" t="inlineStr">
         <is>
-          <t>O(n²) clusters_with 회피. 설계: docs/ONTOLOGY_V46_LAZY_EXPANSION_DESIGN.md</t>
+          <t>O(n²) clusters_with(V4.9 삭제) 회피. 설계: docs/ONTOLOGY_V46_LAZY_EXPANSION_DESIGN.md</t>
         </is>
       </c>
     </row>
@@ -16125,17 +16054,17 @@
       </c>
       <c r="C9" s="61" t="inlineStr">
         <is>
-          <t>linked_subject_cnt · sameAs(confirmed)</t>
+          <t>linked_subject_cnt · same_as(confirmed)</t>
         </is>
       </c>
       <c r="D9" s="61" t="inlineStr">
         <is>
-          <t>sameAs(confirmed) 로 병합한 실체 기준 distinct count</t>
+          <t>same_as(confirmed) 로 병합한 실체 기준 distinct count</t>
         </is>
       </c>
       <c r="E9" s="61" t="inlineStr">
         <is>
-          <t>sameAs 확정 시마다</t>
+          <t>same_as 확정 시마다</t>
         </is>
       </c>
       <c r="F9" s="66" t="inlineStr">
@@ -16194,7 +16123,7 @@
       </c>
       <c r="D11" s="61" t="inlineStr">
         <is>
-          <t>used_ip 시간구간별 role 판정 list (sameAs 해소 후 entity_cnt, 인접 동일구간 coalesce)</t>
+          <t>used_ip 시간구간별 role 판정 list (same_as 해소 후 entity_cnt, 인접 동일구간 coalesce)</t>
         </is>
       </c>
       <c r="E11" s="61" t="inlineStr">
@@ -16428,7 +16357,7 @@
       </c>
       <c r="B17" s="99" t="inlineStr">
         <is>
-          <t>sameAs 의 review_status 가 pending 인 엣지는 기본 탐색에서 제외하고, 후보 탐색 모드에서만 따라간다. 결과는 확정분과 분리해 표시한다.</t>
+          <t>same_as 의 review_status 가 pending 인 엣지는 기본 탐색에서 제외하고, 후보 탐색 모드에서만 따라간다. 결과는 확정분과 분리해 표시한다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(etl,graph): 정합 2단계 2d — CSV ETL·수동 생성 API·모델러 적재를 GraphWriter 로
- GraphWriter: 구조/속성 정책 분리(prop_mode), key_override(자유 설계 키), check_edge(id 연결 검사), node_props
- CSV ETL: 구조 strict + 속성 warn. 키 열 → SoT 정경 키(정규화), 인물 psn:csv:<파일명>:<이름>,
  엣지 양끝을 라벨+키로 MATCH(종전 라벨 무관 ag_vertex LIMIT 1 → 다른 노드 연결 가능), 위반 행은 거부·보고
- 수동 노드/엣지: SoT strict + 속성 warn, MERGE(같은 키 재입력 → 같은 노드), 인물·사건형 키 자동 생성,
  delete_element id 검증
- 모델러: warn 모드(SoT 강제 없음), 사용자 키 유지, SET += 로 재적재 갱신, warnings 응답
- SoT: 노드 공통 그룹 annotation·etl, EDGE_COMMON_GROUPS 신설 (엑셀 재생성)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
+++ b/handoff/ontology_v4.9/spec/CCOP_Ontology_V4.9_node_edge_attrs.xlsx
@@ -17415,7 +17415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="54" min="1" max="1"/>
@@ -17884,6 +17884,182 @@
       <c r="D21" s="85" t="inlineStr">
         <is>
           <t>적재 출처 메타 — V4.0 적재기(make_node_props_v40)·화면 수동 입력이 기록</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="85" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
+      <c r="B22" s="85" t="inlineStr">
+        <is>
+          <t>ontology_type</t>
+        </is>
+      </c>
+      <c r="C22" s="86" t="inlineStr">
+        <is>
+          <t>POLE 레이어 개념</t>
+        </is>
+      </c>
+      <c r="D22" s="85" t="inlineStr">
+        <is>
+          <t>온톨로지 주석 — OntologyEnricher 가 라벨에서 파생해 붙임(라벨로 결정되는 값, 키워드 검색이 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="85" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
+      <c r="B23" s="85" t="inlineStr">
+        <is>
+          <t>domain_concept</t>
+        </is>
+      </c>
+      <c r="C23" s="86" t="inlineStr">
+        <is>
+          <t>도메인 개념(한글)</t>
+        </is>
+      </c>
+      <c r="D23" s="85" t="inlineStr">
+        <is>
+          <t>온톨로지 주석 — OntologyEnricher 가 라벨에서 파생해 붙임(라벨로 결정되는 값, 키워드 검색이 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="85" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
+      <c r="B24" s="85" t="inlineStr">
+        <is>
+          <t>entity_subtype</t>
+        </is>
+      </c>
+      <c r="C24" s="86" t="inlineStr">
+        <is>
+          <t>개념 세부 유형</t>
+        </is>
+      </c>
+      <c r="D24" s="85" t="inlineStr">
+        <is>
+          <t>온톨로지 주석 — OntologyEnricher 가 라벨에서 파생해 붙임(라벨로 결정되는 값, 키워드 검색이 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="85" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
+      <c r="B25" s="85" t="inlineStr">
+        <is>
+          <t>kics_compliant</t>
+        </is>
+      </c>
+      <c r="C25" s="86" t="inlineStr">
+        <is>
+          <t>KICS 표준 준수 표시</t>
+        </is>
+      </c>
+      <c r="D25" s="85" t="inlineStr">
+        <is>
+          <t>온톨로지 주석 — OntologyEnricher 가 라벨에서 파생해 붙임(라벨로 결정되는 값, 키워드 검색이 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="85" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
+      <c r="B26" s="85" t="inlineStr">
+        <is>
+          <t>layer</t>
+        </is>
+      </c>
+      <c r="C26" s="86" t="inlineStr">
+        <is>
+          <t>레이어명</t>
+        </is>
+      </c>
+      <c r="D26" s="85" t="inlineStr">
+        <is>
+          <t>온톨로지 주석 — OntologyEnricher 가 라벨에서 파생해 붙임(라벨로 결정되는 값, 키워드 검색이 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="85" t="inlineStr">
+        <is>
+          <t>annotation</t>
+        </is>
+      </c>
+      <c r="B27" s="85" t="inlineStr">
+        <is>
+          <t>legal_category</t>
+        </is>
+      </c>
+      <c r="C27" s="86" t="inlineStr">
+        <is>
+          <t>법적 분류</t>
+        </is>
+      </c>
+      <c r="D27" s="85" t="inlineStr">
+        <is>
+          <t>온톨로지 주석 — OntologyEnricher 가 라벨에서 파생해 붙임(라벨로 결정되는 값, 키워드 검색이 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="85" t="inlineStr">
+        <is>
+          <t>etl</t>
+        </is>
+      </c>
+      <c r="B28" s="85" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C28" s="86" t="inlineStr">
+        <is>
+          <t>ETL 최초 적재 시각</t>
+        </is>
+      </c>
+      <c r="D28" s="85" t="inlineStr">
+        <is>
+          <t>CSV ETL 적재 메타</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="85" t="inlineStr">
+        <is>
+          <t>etl</t>
+        </is>
+      </c>
+      <c r="B29" s="85" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="C29" s="86" t="inlineStr">
+        <is>
+          <t>ETL 갱신 표시</t>
+        </is>
+      </c>
+      <c r="D29" s="85" t="inlineStr">
+        <is>
+          <t>CSV ETL 적재 메타</t>
         </is>
       </c>
     </row>

</xml_diff>